<commit_message>
auto: data update 2026-05-04 15:51 EDT
Score: 62/100
USD/CNY: 6.83
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.827300071716309</v>
       </c>
       <c r="F522" t="n">
-        <v>6.8314</v>
+        <v>6.8301</v>
       </c>
       <c r="G522" t="n">
         <v>6.8225</v>
       </c>
       <c r="H522" t="n">
-        <v>0.004099928283691767</v>
+        <v>0.002799928283691244</v>
       </c>
       <c r="I522" t="n">
         <v>98.20999908447266</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-05 11:41 EDT
Score: 61/100
USD/CNY: 6.83
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA522"/>
+  <dimension ref="A1:BA523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85472,7 +85472,7 @@
         </is>
       </c>
       <c r="B522" t="n">
-        <v>3.88</v>
+        <v>3.95</v>
       </c>
       <c r="C522" t="n">
         <v>1.2552</v>
@@ -85481,22 +85481,22 @@
         <v>2.6248</v>
       </c>
       <c r="E522" t="n">
-        <v>6.827300071716309</v>
+        <v>6.827499866485596</v>
       </c>
       <c r="F522" t="n">
-        <v>6.8315</v>
+        <v>6.8311</v>
       </c>
       <c r="G522" t="n">
         <v>6.8225</v>
       </c>
       <c r="H522" t="n">
-        <v>0.004199928283691534</v>
+        <v>0.003600133514404469</v>
       </c>
       <c r="I522" t="n">
-        <v>98.20999908447266</v>
+        <v>98.47000122070312</v>
       </c>
       <c r="J522" t="n">
-        <v>0</v>
+        <v>0.002647410026008101</v>
       </c>
       <c r="K522" t="n">
         <v>2.6248</v>
@@ -85529,19 +85529,19 @@
         <v>2.258</v>
       </c>
       <c r="U522" t="n">
-        <v>-5.291221289575493</v>
+        <v>-5.146385663190559</v>
       </c>
       <c r="V522" t="n">
         <v>6.6687</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.323027698362734</v>
+        <v>-2.32588604307562</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.1516766315116547</v>
+        <v>-0.1546415924823297</v>
       </c>
       <c r="Y522" t="n">
-        <v>1.004016064257028</v>
+        <v>0.8032128514056225</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85549,40 +85549,40 @@
         </is>
       </c>
       <c r="AA522" t="n">
-        <v>1.68606</v>
+        <v>1.68697</v>
       </c>
       <c r="AB522" t="n">
-        <v>1.52758</v>
+        <v>1.52879</v>
       </c>
       <c r="AC522" t="n">
-        <v>1.17879</v>
+        <v>1.04409</v>
       </c>
       <c r="AD522" t="n">
-        <v>0.2140599999999999</v>
+        <v>0.2149700000000001</v>
       </c>
       <c r="AE522" t="n">
-        <v>9.126984126984127</v>
+        <v>9.523809523809524</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.3657366315116484</v>
+        <v>-0.3696115924823218</v>
       </c>
       <c r="AG522" t="n">
-        <v>7.188547626614165</v>
+        <v>7.178869340768765</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.3612475548978562</v>
+        <v>-0.3513694742831692</v>
       </c>
       <c r="AI522" t="n">
-        <v>7.06121823198884</v>
+        <v>7.061175551975938</v>
       </c>
       <c r="AJ522" t="n">
-        <v>-0.2339181602725313</v>
+        <v>-0.2336756854903426</v>
       </c>
       <c r="AK522" t="n">
         <v>7.061105294515807</v>
       </c>
       <c r="AL522" t="n">
-        <v>-0.2338052227994982</v>
+        <v>-0.2336054280302111</v>
       </c>
       <c r="AM522" t="n">
         <v>0.01023096587809675</v>
@@ -85594,40 +85594,205 @@
         <v>0.000253092979595082</v>
       </c>
       <c r="AP522" t="n">
-        <v>-1.380145243579625</v>
+        <v>-1.377677384899655</v>
       </c>
       <c r="AQ522" t="n">
-        <v>25.6</v>
+        <v>27.2</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.02841602611953694</v>
+        <v>-0.02818071124961601</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.8309</v>
+        <v>6.830390374574751</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.008399999999999963</v>
+        <v>-0.007890374574751391</v>
       </c>
       <c r="AU522" t="n">
         <v>-0.008399999999999963</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.0134771761608925</v>
+        <v>-0.01345169488963007</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.01164336970322905</v>
+        <v>-0.01163487594614157</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01421946032823592</v>
+        <v>0.0142181862646728</v>
       </c>
       <c r="AY522" t="n">
-        <v>69.04761904761905</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="AZ522" t="n">
-        <v>66.42666666666666</v>
+        <v>67.73999999999999</v>
       </c>
       <c r="BA522" t="n">
-        <v>61.92444444444444</v>
+        <v>62.18711111111111</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B523" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="C523" t="n">
+        <v>1.2552</v>
+      </c>
+      <c r="D523" t="n">
+        <v>2.6248</v>
+      </c>
+      <c r="E523" t="n">
+        <v>6.827499866485596</v>
+      </c>
+      <c r="F523" t="n">
+        <v>6.8275</v>
+      </c>
+      <c r="G523" t="n">
+        <v>6.8225</v>
+      </c>
+      <c r="H523" t="n">
+        <v>1.335144039771308e-07</v>
+      </c>
+      <c r="I523" t="n">
+        <v>98.47000122070312</v>
+      </c>
+      <c r="J523" t="n">
+        <v>0</v>
+      </c>
+      <c r="K523" t="n">
+        <v>2.6248</v>
+      </c>
+      <c r="L523" t="n">
+        <v>2.523225</v>
+      </c>
+      <c r="M523" t="n">
+        <v/>
+      </c>
+      <c r="N523" t="n">
+        <v/>
+      </c>
+      <c r="O523" t="n">
+        <v>98.60000000000001</v>
+      </c>
+      <c r="P523" t="n">
+        <v>73.15369261477046</v>
+      </c>
+      <c r="Q523" t="n">
+        <v>1.472</v>
+      </c>
+      <c r="R523" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="S523" t="n">
+        <v>2.258</v>
+      </c>
+      <c r="T523" t="n">
+        <v>2.258</v>
+      </c>
+      <c r="U523" t="n">
+        <v>-5.155196762221919</v>
+      </c>
+      <c r="V523" t="n">
+        <v>6.6687</v>
+      </c>
+      <c r="W523" t="n">
+        <v>-2.32588604307562</v>
+      </c>
+      <c r="X523" t="n">
+        <v>-0.1546415924823297</v>
+      </c>
+      <c r="Y523" t="n">
+        <v>1.004016064257028</v>
+      </c>
+      <c r="Z523" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA523" t="n">
+        <v>1.68697</v>
+      </c>
+      <c r="AB523" t="n">
+        <v>1.52879</v>
+      </c>
+      <c r="AC523" t="n">
+        <v>1.04409</v>
+      </c>
+      <c r="AD523" t="n">
+        <v>0.2149700000000001</v>
+      </c>
+      <c r="AE523" t="n">
+        <v>9.722222222222221</v>
+      </c>
+      <c r="AF523" t="n">
+        <v>-0.3696115924823218</v>
+      </c>
+      <c r="AG523" t="n">
+        <v>7.179470918543367</v>
+      </c>
+      <c r="AH523" t="n">
+        <v>-0.3519710520577712</v>
+      </c>
+      <c r="AI523" t="n">
+        <v>7.05559572069098</v>
+      </c>
+      <c r="AJ523" t="n">
+        <v>-0.2280958542053844</v>
+      </c>
+      <c r="AK523" t="n">
+        <v>7.055107231813516</v>
+      </c>
+      <c r="AL523" t="n">
+        <v>-0.2276073653279198</v>
+      </c>
+      <c r="AM523" t="n">
+        <v>-0.001349940557735129</v>
+      </c>
+      <c r="AN523" t="n">
+        <v>-0.001242569541730205</v>
+      </c>
+      <c r="AO523" t="n">
+        <v>9.828375502884956e-05</v>
+      </c>
+      <c r="AP523" t="n">
+        <v>-1.309209105676507</v>
+      </c>
+      <c r="AQ523" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="AR523" t="n">
+        <v>-0.02840561701476885</v>
+      </c>
+      <c r="AS523" t="n">
+        <v>6.8311</v>
+      </c>
+      <c r="AT523" t="n">
+        <v>-0.008600000000000385</v>
+      </c>
+      <c r="AU523" t="n">
+        <v>-0.008600000000000385</v>
+      </c>
+      <c r="AV523" t="n">
+        <v>-0.01264331410734045</v>
+      </c>
+      <c r="AW523" t="n">
+        <v>-0.01152325874948465</v>
+      </c>
+      <c r="AX523" t="n">
+        <v>0.01416402028237764</v>
+      </c>
+      <c r="AY523" t="n">
+        <v>68.25396825396825</v>
+      </c>
+      <c r="AZ523" t="n">
+        <v>66.67888888888888</v>
+      </c>
+      <c r="BA523" t="n">
+        <v>61.03799999999999</v>
       </c>
     </row>
   </sheetData>
@@ -85834,7 +85999,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -85854,7 +86019,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>3.95</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -85864,7 +86029,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>98.21</t>
+          <t>98.47</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -85929,7 +86094,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -85939,7 +86104,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -85949,7 +86114,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.36</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -85964,12 +86129,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>0.010</t>
+          <t>-0.001</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>-0.0002</t>
+          <t>-0.0012</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -85979,7 +86144,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-1.38</t>
+          <t>-1.31</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -85989,7 +86154,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.8309</t>
+          <t>6.8311</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -86014,7 +86179,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>61</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-05-05 12:20 EDT
Score: 61/100
USD/CNY: 6.83
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.827499866485596</v>
       </c>
       <c r="F523" t="n">
-        <v>6.8275</v>
+        <v>6.8278</v>
       </c>
       <c r="G523" t="n">
         <v>6.8225</v>
       </c>
       <c r="H523" t="n">
-        <v>1.335144039771308e-07</v>
+        <v>0.0003001335144041661</v>
       </c>
       <c r="I523" t="n">
         <v>98.47000122070312</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-05 15:46 EDT
Score: 61/100
USD/CNY: 6.83
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.827499866485596</v>
       </c>
       <c r="F523" t="n">
-        <v>6.8278</v>
+        <v>6.8288</v>
       </c>
       <c r="G523" t="n">
         <v>6.8225</v>
       </c>
       <c r="H523" t="n">
-        <v>0.0003001335144041661</v>
+        <v>0.0013001335144045</v>
       </c>
       <c r="I523" t="n">
         <v>98.47000122070312</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-06 11:59 EDT
Score: 58/100
USD/CNY: 6.83
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85520,13 +85520,13 @@
         <v>1.472</v>
       </c>
       <c r="R522" t="n">
-        <v>3.73</v>
+        <v>3.78</v>
       </c>
       <c r="S522" t="n">
-        <v>2.258</v>
+        <v>2.308</v>
       </c>
       <c r="T522" t="n">
-        <v>2.258</v>
+        <v>2.308</v>
       </c>
       <c r="U522" t="n">
         <v>-5.146385663190559</v>
@@ -85538,10 +85538,10 @@
         <v>-2.32588604307562</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.1546415924823297</v>
+        <v>-0.1058045355038839</v>
       </c>
       <c r="Y522" t="n">
-        <v>0.8032128514056225</v>
+        <v>1.204819277108434</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,7 +85564,7 @@
         <v>9.523809523809524</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.3696115924823218</v>
+        <v>-0.320774535503876</v>
       </c>
       <c r="AG522" t="n">
         <v>7.178869340768765</v>
@@ -85637,7 +85637,7 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>3.95</v>
+        <v>3.93</v>
       </c>
       <c r="C523" t="n">
         <v>1.2552</v>
@@ -85646,22 +85646,22 @@
         <v>2.6248</v>
       </c>
       <c r="E523" t="n">
-        <v>6.827499866485596</v>
+        <v>6.829999923706055</v>
       </c>
       <c r="F523" t="n">
-        <v>6.8288</v>
+        <v>6.8278</v>
       </c>
       <c r="G523" t="n">
         <v>6.8225</v>
       </c>
       <c r="H523" t="n">
-        <v>0.0013001335144045</v>
+        <v>-0.002199923706054818</v>
       </c>
       <c r="I523" t="n">
-        <v>98.47000122070312</v>
+        <v>98.48000335693359</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>0.0001015754656898959</v>
       </c>
       <c r="K523" t="n">
         <v>2.6248</v>
@@ -85685,28 +85685,28 @@
         <v>1.472</v>
       </c>
       <c r="R523" t="n">
-        <v>3.73</v>
+        <v>3.78</v>
       </c>
       <c r="S523" t="n">
-        <v>2.258</v>
+        <v>2.308</v>
       </c>
       <c r="T523" t="n">
-        <v>2.258</v>
+        <v>2.308</v>
       </c>
       <c r="U523" t="n">
-        <v>-5.155196762221919</v>
+        <v>-5.157166317042675</v>
       </c>
       <c r="V523" t="n">
         <v>6.6687</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.32588604307562</v>
+        <v>-2.361638733643368</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.1546415924823297</v>
+        <v>-0.1429086777750888</v>
       </c>
       <c r="Y523" t="n">
-        <v>1.004016064257028</v>
+        <v>1.204819277108434</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85714,40 +85714,40 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.68697</v>
+        <v>1.68333</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.52879</v>
+        <v>1.52515</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.04409</v>
+        <v>1.03061</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.2149700000000001</v>
+        <v>0.21133</v>
       </c>
       <c r="AE523" t="n">
-        <v>9.722222222222221</v>
+        <v>7.142857142857142</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.3696115924823218</v>
+        <v>-0.3542386777750872</v>
       </c>
       <c r="AG523" t="n">
-        <v>7.179470918543367</v>
+        <v>7.182234379225464</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3519710520577712</v>
+        <v>-0.352234455519409</v>
       </c>
       <c r="AI523" t="n">
-        <v>7.05559572069098</v>
+        <v>7.055583292341148</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.2280958542053844</v>
+        <v>-0.2255833686350934</v>
       </c>
       <c r="AK523" t="n">
         <v>7.055107231813516</v>
       </c>
       <c r="AL523" t="n">
-        <v>-0.2276073653279198</v>
+        <v>-0.2251073081074608</v>
       </c>
       <c r="AM523" t="n">
         <v>-0.001349940557735129</v>
@@ -85759,31 +85759,31 @@
         <v>9.828375502884956e-05</v>
       </c>
       <c r="AP523" t="n">
-        <v>-1.309209105676507</v>
+        <v>-1.283638191630508</v>
       </c>
       <c r="AQ523" t="n">
         <v>27.6</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.02840561701476885</v>
+        <v>-0.02837946088320876</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.8311</v>
+        <v>6.831080308282073</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.008600000000000385</v>
+        <v>-0.008580308282073013</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.008600000000000385</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01264331410734045</v>
+        <v>-0.01264232952144408</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01152325874948465</v>
+        <v>-0.01152293055418586</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01416402028237764</v>
+        <v>0.01416397105308282</v>
       </c>
       <c r="AY523" t="n">
         <v>68.25396825396825</v>
@@ -85793,6 +85793,171 @@
       </c>
       <c r="BA523" t="n">
         <v>61.03799999999999</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2802</v>
+      </c>
+      <c r="D524" t="n">
+        <v>2.6248</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.829999923706055</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.8125</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.8001</v>
+      </c>
+      <c r="H524" t="n">
+        <v>-0.01749992370605469</v>
+      </c>
+      <c r="I524" t="n">
+        <v>98.48000335693359</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>2.6248</v>
+      </c>
+      <c r="L524" t="n">
+        <v>2.53104</v>
+      </c>
+      <c r="M524" t="n">
+        <v/>
+      </c>
+      <c r="N524" t="n">
+        <v/>
+      </c>
+      <c r="O524" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="P524" t="n">
+        <v>73.25349301397206</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.471</v>
+      </c>
+      <c r="R524" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.309</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.309</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-5.246927963312807</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.6511</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-2.619325412949369</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.4093359135588504</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>0.4016064257028112</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.68333</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.52515</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.03061</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.2123299999999999</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>7.936507936507936</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.6216659135588554</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>7.188365099597231</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.3583651758911763</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>7.050171901864974</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>-0.2201719781589198</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>7.049240044502209</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>-0.2192401207961545</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.01245927794565181</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>-0.002690846636687002</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.0009149443224349962</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>-1.218013920592748</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>-0.02769955905545405</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.8278</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>-0.02770000000000028</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>-0.02770000000000028</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.01217274711458152</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.01177119541575803</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.01404900908920962</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>9.126984126984127</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>45.79444444444444</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>57.7771111111111</v>
       </c>
     </row>
   </sheetData>
@@ -85999,7 +86164,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86009,27 +86174,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.83</t>
+          <t>6.81</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.82</t>
+          <t>6.80</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3.95</t>
+          <t>3.93</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>98.47</t>
+          <t>98.48</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86039,7 +86204,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>98</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -86054,27 +86219,27 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.73</t>
+          <t>3.78</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.26</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.67</t>
+          <t>6.65</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.41</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86084,7 +86249,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>1.68</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -86094,7 +86259,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86104,47 +86269,47 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.37</t>
+          <t>-0.62</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.35</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.001</t>
+          <t>-0.012</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>-0.0012</t>
+          <t>-0.0027</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-1.31</t>
+          <t>-1.22</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86154,24 +86319,24 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.8311</t>
+          <t>6.8278</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
           <t>-0.01</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
-      </c>
       <c r="AJ2" t="inlineStr">
         <is>
           <t>0.01</t>
@@ -86179,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-05-07 16:18 EDT
Score: 58/100
USD/CNY: 6.81
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.471</v>
       </c>
       <c r="R523" t="n">
-        <v>3.77</v>
+        <v>3.73</v>
       </c>
       <c r="S523" t="n">
-        <v>2.299</v>
+        <v>2.259</v>
       </c>
       <c r="T523" t="n">
-        <v>2.299</v>
+        <v>2.259</v>
       </c>
       <c r="U523" t="n">
         <v>-5.367009029103583</v>
@@ -85703,7 +85703,7 @@
         <v>-2.363070205458651</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.1531579522044302</v>
+        <v>-0.1922127241222427</v>
       </c>
       <c r="Y523" t="n">
         <v>0.8032128514056225</v>
@@ -85729,7 +85729,7 @@
         <v>14.68253968253968</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.3839779522044395</v>
+        <v>-0.423032724122252</v>
       </c>
       <c r="AG523" t="n">
         <v>7.196672146399949</v>
@@ -85811,16 +85811,16 @@
         <v>2.5898</v>
       </c>
       <c r="E524" t="n">
-        <v>6.830100059509277</v>
+        <v>6.810999870300293</v>
       </c>
       <c r="F524" t="n">
-        <v>6.8069</v>
+        <v>6.8073</v>
       </c>
       <c r="G524" t="n">
         <v>6.7911</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.02320005950927762</v>
+        <v>-0.003699870300293284</v>
       </c>
       <c r="I524" t="n">
         <v>98.01999664306641</v>
@@ -85850,25 +85850,25 @@
         <v>1.47</v>
       </c>
       <c r="R524" t="n">
-        <v>3.77</v>
+        <v>3.73</v>
       </c>
       <c r="S524" t="n">
-        <v>2.3</v>
+        <v>2.26</v>
       </c>
       <c r="T524" t="n">
-        <v>2.3</v>
+        <v>2.26</v>
       </c>
       <c r="U524" t="n">
-        <v>-5.310919393762621</v>
+        <v>-5.606244386347636</v>
       </c>
       <c r="V524" t="n">
         <v>6.641</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.768627953641778</v>
+        <v>-2.495960557004062</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.5730052274940611</v>
+        <v>-0.3290598857802918</v>
       </c>
       <c r="Y524" t="n">
         <v>0.4016064257028112</v>
@@ -85894,25 +85894,25 @@
         <v>15.87301587301587</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.804825227494077</v>
+        <v>-0.5608798857803077</v>
       </c>
       <c r="AG524" t="n">
         <v>7.192841168183148</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3627411086738705</v>
+        <v>-0.3818412978828549</v>
       </c>
       <c r="AI524" t="n">
         <v>7.047055026501724</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.2169549669924464</v>
+        <v>-0.2360551562014308</v>
       </c>
       <c r="AK524" t="n">
         <v>7.044607485549974</v>
       </c>
       <c r="AL524" t="n">
-        <v>-0.2145074260406963</v>
+        <v>-0.2336076152496807</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.02351974718911115</v>
@@ -85924,13 +85924,13 @@
         <v>0.002235402288773614</v>
       </c>
       <c r="AP524" t="n">
-        <v>-1.175295076012844</v>
+        <v>-1.369531872337947</v>
       </c>
       <c r="AQ524" t="n">
-        <v>26.8</v>
+        <v>23.6</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.02771913005585205</v>
+        <v>-0.02777884854528146</v>
       </c>
       <c r="AS524" t="n">
         <v>6.8135</v>
@@ -85954,10 +85954,10 @@
         <v>17.46031746031746</v>
       </c>
       <c r="AZ524" t="n">
-        <v>48.1011111111111</v>
+        <v>47.1411111111111</v>
       </c>
       <c r="BA524" t="n">
-        <v>58.35666666666666</v>
+        <v>58.16466666666665</v>
       </c>
     </row>
   </sheetData>
@@ -86169,7 +86169,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.83</t>
+          <t>6.81</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.77</t>
+          <t>3.73</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.30</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,7 +86234,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.57</t>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86274,22 +86274,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.80</t>
+          <t>-0.56</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.36</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.24</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.21</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-1.18</t>
+          <t>-1.37</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-05-11 15:59 EDT
Score: 53/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.801400184631348</v>
       </c>
       <c r="F522" t="n">
-        <v>6.792759895324707</v>
+        <v>6.792240142822266</v>
       </c>
       <c r="G522" t="n">
         <v>6.782999999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.008640289306640625</v>
+        <v>-0.009160041809082031</v>
       </c>
       <c r="I522" t="n">
         <v>97.83999633789062</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-11 16:49 EDT
Score: 53/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85355,13 +85355,13 @@
         <v>1.469</v>
       </c>
       <c r="R521" t="n">
-        <v>3.76</v>
+        <v>3.75</v>
       </c>
       <c r="S521" t="n">
-        <v>2.290999999999999</v>
+        <v>2.281</v>
       </c>
       <c r="T521" t="n">
-        <v>2.290999999999999</v>
+        <v>2.281</v>
       </c>
       <c r="U521" t="n">
         <v>-5.938320338731486</v>
@@ -85373,7 +85373,7 @@
         <v>-1.951071559223949</v>
       </c>
       <c r="X521" t="n">
-        <v>0.2665681501492267</v>
+        <v>0.2567632573051482</v>
       </c>
       <c r="Y521" t="n">
         <v>2.811244979919679</v>
@@ -85399,7 +85399,7 @@
         <v>17.85714285714286</v>
       </c>
       <c r="AF521" t="n">
-        <v>0.03192815014922967</v>
+        <v>0.02212325730515108</v>
       </c>
       <c r="AG521" t="n">
         <v>7.205289115113832</v>
@@ -85481,16 +85481,16 @@
         <v>2.6192</v>
       </c>
       <c r="E522" t="n">
-        <v>6.801400184631348</v>
+        <v>6.80049991607666</v>
       </c>
       <c r="F522" t="n">
-        <v>6.792240142822266</v>
+        <v>6.79203987121582</v>
       </c>
       <c r="G522" t="n">
         <v>6.782999999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.009160041809082031</v>
+        <v>-0.008460044860839844</v>
       </c>
       <c r="I522" t="n">
         <v>97.83999633789062</v>
@@ -85520,25 +85520,25 @@
         <v>1.469</v>
       </c>
       <c r="R522" t="n">
-        <v>3.76</v>
+        <v>3.75</v>
       </c>
       <c r="S522" t="n">
-        <v>2.290999999999999</v>
+        <v>2.281</v>
       </c>
       <c r="T522" t="n">
-        <v>2.290999999999999</v>
+        <v>2.281</v>
       </c>
       <c r="U522" t="n">
-        <v>-5.670057572394559</v>
+        <v>-5.684046460149642</v>
       </c>
       <c r="V522" t="n">
         <v>6.6314</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.499488046821374</v>
+        <v>-2.486580665590499</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.3024687973818496</v>
+        <v>-0.2988274405501423</v>
       </c>
       <c r="Y522" t="n">
         <v>0.8032128514056225</v>
@@ -85564,25 +85564,25 @@
         <v>18.05555555555555</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.5371087973818467</v>
+        <v>-0.5334674405501394</v>
       </c>
       <c r="AG522" t="n">
         <v>7.187043490828895</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.3856433061975473</v>
+        <v>-0.3865435747522348</v>
       </c>
       <c r="AI522" t="n">
         <v>7.034769539496025</v>
       </c>
       <c r="AJ522" t="n">
-        <v>-0.2333693548646769</v>
+        <v>-0.2342696234193644</v>
       </c>
       <c r="AK522" t="n">
         <v>7.031531243279008</v>
       </c>
       <c r="AL522" t="n">
-        <v>-0.2301310586476601</v>
+        <v>-0.2310313272023476</v>
       </c>
       <c r="AM522" t="n">
         <v>-0.04964211158845274</v>
@@ -85594,13 +85594,13 @@
         <v>0.007358432861331865</v>
       </c>
       <c r="AP522" t="n">
-        <v>-1.319074284750444</v>
+        <v>-1.328198129730001</v>
       </c>
       <c r="AQ522" t="n">
-        <v>23.6</v>
+        <v>23.2</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.0232092035776862</v>
+        <v>-0.02321208643354045</v>
       </c>
       <c r="AS522" t="n">
         <v>6.801400184631348</v>
@@ -85624,10 +85624,10 @@
         <v>38.09523809523809</v>
       </c>
       <c r="AZ522" t="n">
-        <v>54.36333333333333</v>
+        <v>54.24333333333333</v>
       </c>
       <c r="BA522" t="n">
-        <v>52.89666666666667</v>
+        <v>52.87266666666667</v>
       </c>
     </row>
   </sheetData>
@@ -85889,12 +85889,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.76</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.29</t>
+          <t>2.28</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -85944,7 +85944,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.54</t>
+          <t>-0.53</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -85979,7 +85979,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-1.32</t>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-05-12 13:04 EDT
Score: 51/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -80945,13 +80945,13 @@
         <v>6.80049991607666</v>
       </c>
       <c r="F523" t="n">
-        <v>6.793879985809326</v>
+        <v>6.793479919433594</v>
       </c>
       <c r="G523" t="n">
         <v>6.7849</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.006619930267333984</v>
+        <v>-0.007019996643066406</v>
       </c>
       <c r="I523" t="n">
         <v>97.94000244140625</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-13 16:06 EDT
Score: 57/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.7947998046875</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7865</v>
+        <v>6.7877</v>
       </c>
       <c r="G524" t="n">
         <v>6.7784</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.008299804687499801</v>
+        <v>-0.007099804687499933</v>
       </c>
       <c r="I524" t="n">
         <v>98.29000091552734</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-14 12:58 EDT
Score: 56/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.791999816894531</v>
       </c>
       <c r="F524" t="n">
-        <v>6.785470008850098</v>
+        <v>6.785950183868408</v>
       </c>
       <c r="G524" t="n">
         <v>6.7759</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.006529808044433594</v>
+        <v>-0.006049633026123047</v>
       </c>
       <c r="I524" t="n">
         <v>98.48000335693359</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-14 15:57 EDT
Score: 56/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.791999816894531</v>
       </c>
       <c r="F524" t="n">
-        <v>6.785950183868408</v>
+        <v>6.786439895629883</v>
       </c>
       <c r="G524" t="n">
         <v>6.7759</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.006049633026123047</v>
+        <v>-0.005559921264648438</v>
       </c>
       <c r="I524" t="n">
         <v>98.48000335693359</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-14 16:39 EDT
Score: 56/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.468</v>
       </c>
       <c r="R523" t="n">
-        <v>3.8</v>
+        <v>3.79</v>
       </c>
       <c r="S523" t="n">
-        <v>2.332</v>
+        <v>2.322</v>
       </c>
       <c r="T523" t="n">
-        <v>2.332</v>
+        <v>2.322</v>
       </c>
       <c r="U523" t="n">
         <v>-5.693050673107019</v>
@@ -85703,7 +85703,7 @@
         <v>-1.81536837777635</v>
       </c>
       <c r="X523" t="n">
-        <v>0.4476476238681526</v>
+        <v>0.4378291607059381</v>
       </c>
       <c r="Y523" t="n">
         <v>4.016064257028113</v>
@@ -85729,7 +85729,7 @@
         <v>16.26984126984127</v>
       </c>
       <c r="AF523" t="n">
-        <v>0.2165576238681632</v>
+        <v>0.2067391607059488</v>
       </c>
       <c r="AG523" t="n">
         <v>7.178671808187673</v>
@@ -85811,16 +85811,16 @@
         <v>2.7083</v>
       </c>
       <c r="E524" t="n">
-        <v>6.791999816894531</v>
+        <v>6.790800094604492</v>
       </c>
       <c r="F524" t="n">
-        <v>6.786439895629883</v>
+        <v>6.787330150604248</v>
       </c>
       <c r="G524" t="n">
         <v>6.7759</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.005559921264648438</v>
+        <v>-0.003469944000244141</v>
       </c>
       <c r="I524" t="n">
         <v>98.48000335693359</v>
@@ -85850,25 +85850,25 @@
         <v>1.468</v>
       </c>
       <c r="R524" t="n">
-        <v>3.8</v>
+        <v>3.79</v>
       </c>
       <c r="S524" t="n">
-        <v>2.332</v>
+        <v>2.322</v>
       </c>
       <c r="T524" t="n">
-        <v>2.332</v>
+        <v>2.322</v>
       </c>
       <c r="U524" t="n">
-        <v>-5.526151054470739</v>
+        <v>-5.544794229625117</v>
       </c>
       <c r="V524" t="n">
         <v>6.6201</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.530916100247016</v>
+        <v>-2.513696357224815</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2950909120563949</v>
+        <v>-0.2869654491636231</v>
       </c>
       <c r="Y524" t="n">
         <v>0.8032128514056225</v>
@@ -85894,25 +85894,25 @@
         <v>16.46825396825397</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.5261809120563843</v>
+        <v>-0.5180554491636125</v>
       </c>
       <c r="AG524" t="n">
         <v>7.167335986395499</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3753361695009678</v>
+        <v>-0.3765358917910069</v>
       </c>
       <c r="AI524" t="n">
         <v>7.004613652506715</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.2126138356121841</v>
+        <v>-0.2138135579022231</v>
       </c>
       <c r="AK524" t="n">
         <v>7.003692382618654</v>
       </c>
       <c r="AL524" t="n">
-        <v>-0.2116925657241229</v>
+        <v>-0.2128922880141619</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.09225745624393311</v>
@@ -85924,13 +85924,13 @@
         <v>0.02283737241168693</v>
       </c>
       <c r="AP524" t="n">
-        <v>-1.078440409053589</v>
+        <v>-1.090614339877033</v>
       </c>
       <c r="AQ524" t="n">
-        <v>27.8</v>
+        <v>27.4</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.02365317153516138</v>
+        <v>-0.02365493255620223</v>
       </c>
       <c r="AS524" t="n">
         <v>6.791999816894531</v>
@@ -85954,10 +85954,10 @@
         <v>43.65079365079365</v>
       </c>
       <c r="AZ524" t="n">
-        <v>58.40777777777777</v>
+        <v>58.28777777777778</v>
       </c>
       <c r="BA524" t="n">
-        <v>56.16133333333332</v>
+        <v>56.13733333333332</v>
       </c>
     </row>
   </sheetData>
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>3.79</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.33</t>
+          <t>2.32</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,7 +86234,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.53</t>
+          <t>-0.52</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-1.08</t>
+          <t>-1.09</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-05-15 15:49 EDT
Score: 62/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.790800094604492</v>
       </c>
       <c r="F524" t="n">
-        <v>6.813169956207275</v>
+        <v>6.815010070800781</v>
       </c>
       <c r="G524" t="n">
         <v>6.800800000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>0.0223698616027832</v>
+        <v>0.02420997619628906</v>
       </c>
       <c r="I524" t="n">
         <v>98.87999725341797</v>
@@ -86174,7 +86174,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.81</t>
+          <t>6.82</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-05-18 16:27 EDT
Score: 67/100
USD/CNY: 6.81
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85355,13 +85355,13 @@
         <v>1.468</v>
       </c>
       <c r="R521" t="n">
-        <v>3.79</v>
+        <v>3.82</v>
       </c>
       <c r="S521" t="n">
-        <v>2.322</v>
+        <v>2.352</v>
       </c>
       <c r="T521" t="n">
-        <v>2.322</v>
+        <v>2.352</v>
       </c>
       <c r="U521" t="n">
         <v>-5.482743970135634</v>
@@ -85373,7 +85373,7 @@
         <v>-1.715523477963132</v>
       </c>
       <c r="X521" t="n">
-        <v>0.5414581822220654</v>
+        <v>0.5709435251786799</v>
       </c>
       <c r="Y521" t="n">
         <v>4.819277108433734</v>
@@ -85399,7 +85399,7 @@
         <v>18.45238095238095</v>
       </c>
       <c r="AF521" t="n">
-        <v>0.3076381822220586</v>
+        <v>0.3371235251786731</v>
       </c>
       <c r="AG521" t="n">
         <v>7.157109643412745</v>
@@ -85481,16 +85481,16 @@
         <v>2.8167</v>
       </c>
       <c r="E522" t="n">
-        <v>6.785099983215332</v>
+        <v>6.809199810028076</v>
       </c>
       <c r="F522" t="n">
-        <v>6.797860145568848</v>
+        <v>6.798220157623291</v>
       </c>
       <c r="G522" t="n">
         <v>6.7888</v>
       </c>
       <c r="H522" t="n">
-        <v>0.01276016235351562</v>
+        <v>-0.01097965240478516</v>
       </c>
       <c r="I522" t="n">
         <v>99.26999664306641</v>
@@ -85520,28 +85520,28 @@
         <v>1.467</v>
       </c>
       <c r="R522" t="n">
-        <v>3.79</v>
+        <v>3.82</v>
       </c>
       <c r="S522" t="n">
-        <v>2.323</v>
+        <v>2.353</v>
       </c>
       <c r="T522" t="n">
-        <v>2.323</v>
+        <v>2.353</v>
       </c>
       <c r="U522" t="n">
-        <v>-5.36646682791881</v>
+        <v>-4.993542890706116</v>
       </c>
       <c r="V522" t="n">
         <v>6.6286</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.306524348977534</v>
+        <v>-2.652291239303961</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.07094162180376617</v>
+        <v>-0.4006087646453604</v>
       </c>
       <c r="Y522" t="n">
-        <v>2.409638554216867</v>
+        <v>0.4016064257028112</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,25 +85564,25 @@
         <v>20.23809523809524</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.3057616218037795</v>
+        <v>-0.6354287646453738</v>
       </c>
       <c r="AG522" t="n">
         <v>7.149220123055708</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.3641201398403755</v>
+        <v>-0.3400203130276314</v>
       </c>
       <c r="AI522" t="n">
         <v>6.972797972602756</v>
       </c>
       <c r="AJ522" t="n">
-        <v>-0.1876979893874235</v>
+        <v>-0.1635981625746794</v>
       </c>
       <c r="AK522" t="n">
         <v>6.976048621620001</v>
       </c>
       <c r="AL522" t="n">
-        <v>-0.1909486384046692</v>
+        <v>-0.1668488115919251</v>
       </c>
       <c r="AM522" t="n">
         <v>-0.1171809788132889</v>
@@ -85594,13 +85594,13 @@
         <v>0.03914952746580458</v>
       </c>
       <c r="AP522" t="n">
-        <v>-0.8092415685953788</v>
+        <v>-0.563311520375112</v>
       </c>
       <c r="AQ522" t="n">
-        <v>30.4</v>
+        <v>35.6</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.02423167728780784</v>
+        <v>-0.02423831890392438</v>
       </c>
       <c r="AS522" t="n">
         <v>6.785099983215332</v>
@@ -85624,10 +85624,10 @@
         <v>92.46031746031747</v>
       </c>
       <c r="AZ522" t="n">
-        <v>76.41111111111111</v>
+        <v>77.97111111111111</v>
       </c>
       <c r="BA522" t="n">
-        <v>66.19066666666666</v>
+        <v>66.50266666666667</v>
       </c>
     </row>
   </sheetData>
@@ -85839,19 +85839,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>6.81</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>6.80</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>6.79</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>6.80</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6.79</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>4.09</t>
@@ -85889,12 +85889,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.79</t>
+          <t>3.82</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.32</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -85904,12 +85904,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.40</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85944,22 +85944,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.64</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.36</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.19</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.19</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -85979,7 +85979,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-0.81</t>
+          <t>-0.56</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86014,7 +86014,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-05-19 12:45 EDT
Score: 69/100
USD/CNY: 6.81
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA522"/>
+  <dimension ref="A1:BA523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85472,49 +85472,49 @@
         </is>
       </c>
       <c r="B522" t="n">
-        <v>4.09</v>
+        <v>4.07</v>
       </c>
       <c r="C522" t="n">
         <v>1.2684</v>
       </c>
       <c r="D522" t="n">
-        <v>2.8167</v>
+        <v>2.801600000000001</v>
       </c>
       <c r="E522" t="n">
         <v>6.809199810028076</v>
       </c>
       <c r="F522" t="n">
-        <v>6.798220157623291</v>
+        <v>6.829599857330322</v>
       </c>
       <c r="G522" t="n">
         <v>6.7888</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.01097965240478516</v>
+        <v>0.02040004730224609</v>
       </c>
       <c r="I522" t="n">
-        <v>99.26999664306641</v>
+        <v>98.97000122070312</v>
       </c>
       <c r="J522" t="n">
-        <v>0</v>
+        <v>-0.003022015034834125</v>
       </c>
       <c r="K522" t="n">
-        <v>2.8167</v>
+        <v>2.801600000000001</v>
       </c>
       <c r="L522" t="n">
-        <v>2.636145</v>
+        <v>2.63539</v>
       </c>
       <c r="M522" t="n">
-        <v>2.468116666666667</v>
+        <v>2.467865</v>
       </c>
       <c r="N522" t="n">
         <v/>
       </c>
       <c r="O522" t="n">
-        <v>99.80000000000001</v>
+        <v>99.60000000000001</v>
       </c>
       <c r="P522" t="n">
-        <v>79.74051896207585</v>
+        <v>78.64271457085829</v>
       </c>
       <c r="Q522" t="n">
         <v>1.467</v>
@@ -85529,19 +85529,19 @@
         <v>2.353</v>
       </c>
       <c r="U522" t="n">
-        <v>-4.993542890706116</v>
+        <v>-5.033901738263791</v>
       </c>
       <c r="V522" t="n">
-        <v>6.6286</v>
+        <v>6.6687</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.652291239303961</v>
+        <v>-2.063382099922495</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.4006087646453604</v>
+        <v>0.2107967038604608</v>
       </c>
       <c r="Y522" t="n">
-        <v>0.4016064257028112</v>
+        <v>2.811244979919679</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85549,34 +85549,34 @@
         </is>
       </c>
       <c r="AA522" t="n">
-        <v>1.70182</v>
+        <v>1.69636</v>
       </c>
       <c r="AB522" t="n">
-        <v>1.56939</v>
+        <v>1.57212</v>
       </c>
       <c r="AC522" t="n">
-        <v>1.23485</v>
+        <v>1.3</v>
       </c>
       <c r="AD522" t="n">
-        <v>0.23482</v>
+        <v>0.22936</v>
       </c>
       <c r="AE522" t="n">
-        <v>20.23809523809524</v>
+        <v>14.48412698412698</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.6354287646453738</v>
+        <v>-0.01856329613953989</v>
       </c>
       <c r="AG522" t="n">
-        <v>7.149220123055708</v>
+        <v>7.151968237626934</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.3400203130276314</v>
+        <v>-0.3427684275988581</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.972797972602756</v>
+        <v>6.976537964100194</v>
       </c>
       <c r="AJ522" t="n">
-        <v>-0.1635981625746794</v>
+        <v>-0.1673381540721177</v>
       </c>
       <c r="AK522" t="n">
         <v>6.976048621620001</v>
@@ -85594,40 +85594,205 @@
         <v>0.03914952746580458</v>
       </c>
       <c r="AP522" t="n">
-        <v>-0.563311520375112</v>
+        <v>-0.6015084152656183</v>
       </c>
       <c r="AQ522" t="n">
-        <v>35.6</v>
+        <v>35.2</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.02423831890392438</v>
+        <v>-0.02745253965785189</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.785099983215332</v>
+        <v>6.785662888595939</v>
       </c>
       <c r="AT522" t="n">
-        <v>0.003700016784668136</v>
+        <v>0.003137111404060811</v>
       </c>
       <c r="AU522" t="n">
         <v>0.003700016784668136</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.01074931834752251</v>
+        <v>-0.01077746361655287</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.01348373076595875</v>
+        <v>-0.01349311252230221</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01435928802699876</v>
+        <v>0.01436069529045027</v>
       </c>
       <c r="AY522" t="n">
         <v>92.46031746031747</v>
       </c>
       <c r="AZ522" t="n">
-        <v>77.97111111111111</v>
+        <v>77.78111111111112</v>
       </c>
       <c r="BA522" t="n">
-        <v>66.50266666666667</v>
+        <v>66.46466666666666</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B523" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="C523" t="n">
+        <v>1.2617</v>
+      </c>
+      <c r="D523" t="n">
+        <v>2.801600000000001</v>
+      </c>
+      <c r="E523" t="n">
+        <v>6.809199810028076</v>
+      </c>
+      <c r="F523" t="n">
+        <v>6.815730094909668</v>
+      </c>
+      <c r="G523" t="n">
+        <v>6.803</v>
+      </c>
+      <c r="H523" t="n">
+        <v>0.006530284881591797</v>
+      </c>
+      <c r="I523" t="n">
+        <v>98.97000122070312</v>
+      </c>
+      <c r="J523" t="n">
+        <v>0</v>
+      </c>
+      <c r="K523" t="n">
+        <v>2.801600000000001</v>
+      </c>
+      <c r="L523" t="n">
+        <v>2.65053</v>
+      </c>
+      <c r="M523" t="n">
+        <v>2.480006666666667</v>
+      </c>
+      <c r="N523" t="n">
+        <v/>
+      </c>
+      <c r="O523" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="P523" t="n">
+        <v>78.74251497005989</v>
+      </c>
+      <c r="Q523" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="R523" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="S523" t="n">
+        <v>2.354</v>
+      </c>
+      <c r="T523" t="n">
+        <v>2.354</v>
+      </c>
+      <c r="U523" t="n">
+        <v>-5.012763174232644</v>
+      </c>
+      <c r="V523" t="n">
+        <v>6.6344</v>
+      </c>
+      <c r="W523" t="n">
+        <v>-2.567112361288681</v>
+      </c>
+      <c r="X523" t="n">
+        <v>-0.3111760534898922</v>
+      </c>
+      <c r="Y523" t="n">
+        <v>0.8032128514056225</v>
+      </c>
+      <c r="Z523" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA523" t="n">
+        <v>1.69636</v>
+      </c>
+      <c r="AB523" t="n">
+        <v>1.57212</v>
+      </c>
+      <c r="AC523" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AD523" t="n">
+        <v>0.2303600000000001</v>
+      </c>
+      <c r="AE523" t="n">
+        <v>15.07936507936508</v>
+      </c>
+      <c r="AF523" t="n">
+        <v>-0.5415360534898994</v>
+      </c>
+      <c r="AG523" t="n">
+        <v>7.150528870565083</v>
+      </c>
+      <c r="AH523" t="n">
+        <v>-0.3413290605370065</v>
+      </c>
+      <c r="AI523" t="n">
+        <v>6.96919812791216</v>
+      </c>
+      <c r="AJ523" t="n">
+        <v>-0.1599983178840843</v>
+      </c>
+      <c r="AK523" t="n">
+        <v>6.970728111892008</v>
+      </c>
+      <c r="AL523" t="n">
+        <v>-0.1615283018639317</v>
+      </c>
+      <c r="AM523" t="n">
+        <v>-0.127636816539944</v>
+      </c>
+      <c r="AN523" t="n">
+        <v>-0.00745101973257789</v>
+      </c>
+      <c r="AO523" t="n">
+        <v>0.04750067483060672</v>
+      </c>
+      <c r="AP523" t="n">
+        <v>-0.5204714121791216</v>
+      </c>
+      <c r="AQ523" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="AR523" t="n">
+        <v>-0.02748672558764965</v>
+      </c>
+      <c r="AS523" t="n">
+        <v>6.809199810028076</v>
+      </c>
+      <c r="AT523" t="n">
+        <v>-0.006199810028076236</v>
+      </c>
+      <c r="AU523" t="n">
+        <v>-0.006199810028076236</v>
+      </c>
+      <c r="AV523" t="n">
+        <v>-0.01081597547059343</v>
+      </c>
+      <c r="AW523" t="n">
+        <v>-0.01295318526773368</v>
+      </c>
+      <c r="AX523" t="n">
+        <v>0.0140753149311943</v>
+      </c>
+      <c r="AY523" t="n">
+        <v>75</v>
+      </c>
+      <c r="AZ523" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="BA523" t="n">
+        <v>68.95955555555557</v>
       </c>
     </row>
   </sheetData>
@@ -85834,7 +85999,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -85844,42 +86009,42 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>6.82</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>6.80</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6.79</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>4.07</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.27</t>
+          <t>98.97</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.82</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>99</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>79</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -85904,12 +86069,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.40</t>
+          <t>-0.31</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85929,7 +86094,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -85939,12 +86104,12 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.64</t>
+          <t>-0.54</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -85959,47 +86124,47 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.117</t>
+          <t>-0.128</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>-0.0066</t>
+          <t>-0.0075</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.039</t>
+          <t>0.048</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-0.56</t>
+          <t>-0.52</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>-0.024</t>
+          <t>-0.027</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.7851</t>
+          <t>6.8092</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
@@ -86014,7 +86179,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>69</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-05-19 13:34 EDT
Score: 69/100
USD/CNY: 6.81
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.809199810028076</v>
       </c>
       <c r="F523" t="n">
-        <v>6.815730094909668</v>
+        <v>6.815559864044189</v>
       </c>
       <c r="G523" t="n">
         <v>6.803</v>
       </c>
       <c r="H523" t="n">
-        <v>0.006530284881591797</v>
+        <v>0.006360054016113281</v>
       </c>
       <c r="I523" t="n">
         <v>98.97000122070312</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-19 16:01 EDT
Score: 69/100
USD/CNY: 6.81
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.809199810028076</v>
       </c>
       <c r="F523" t="n">
-        <v>6.815559864044189</v>
+        <v>6.816050052642822</v>
       </c>
       <c r="G523" t="n">
         <v>6.803</v>
       </c>
       <c r="H523" t="n">
-        <v>0.006360054016113281</v>
+        <v>0.006850242614746094</v>
       </c>
       <c r="I523" t="n">
         <v>98.97000122070312</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-19 16:48 EDT
Score: 69/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85520,13 +85520,13 @@
         <v>1.467</v>
       </c>
       <c r="R522" t="n">
-        <v>3.82</v>
+        <v>3.81</v>
       </c>
       <c r="S522" t="n">
-        <v>2.353</v>
+        <v>2.343</v>
       </c>
       <c r="T522" t="n">
-        <v>2.353</v>
+        <v>2.343</v>
       </c>
       <c r="U522" t="n">
         <v>-5.033901738263791</v>
@@ -85538,7 +85538,7 @@
         <v>-2.063382099922495</v>
       </c>
       <c r="X522" t="n">
-        <v>0.2107967038604608</v>
+        <v>0.2010030420704689</v>
       </c>
       <c r="Y522" t="n">
         <v>2.811244979919679</v>
@@ -85564,7 +85564,7 @@
         <v>14.48412698412698</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.01856329613953989</v>
+        <v>-0.02835695792953175</v>
       </c>
       <c r="AG522" t="n">
         <v>7.151968237626934</v>
@@ -85646,16 +85646,16 @@
         <v>2.801600000000001</v>
       </c>
       <c r="E523" t="n">
-        <v>6.809199810028076</v>
+        <v>6.800000190734863</v>
       </c>
       <c r="F523" t="n">
-        <v>6.816050052642822</v>
+        <v>6.816780090332031</v>
       </c>
       <c r="G523" t="n">
         <v>6.803</v>
       </c>
       <c r="H523" t="n">
-        <v>0.006850242614746094</v>
+        <v>0.01677989959716797</v>
       </c>
       <c r="I523" t="n">
         <v>98.97000122070312</v>
@@ -85685,28 +85685,28 @@
         <v>1.466</v>
       </c>
       <c r="R523" t="n">
-        <v>3.82</v>
+        <v>3.81</v>
       </c>
       <c r="S523" t="n">
-        <v>2.354</v>
+        <v>2.344</v>
       </c>
       <c r="T523" t="n">
-        <v>2.354</v>
+        <v>2.344</v>
       </c>
       <c r="U523" t="n">
-        <v>-5.012763174232644</v>
+        <v>-5.154833382325809</v>
       </c>
       <c r="V523" t="n">
         <v>6.6344</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.567112361288681</v>
+        <v>-2.43529685426328</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.3111760534898922</v>
+        <v>-0.1840816644107068</v>
       </c>
       <c r="Y523" t="n">
-        <v>0.8032128514056225</v>
+        <v>1.204819277108434</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,25 +85729,25 @@
         <v>15.07936507936508</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.5415360534898994</v>
+        <v>-0.4144416644107141</v>
       </c>
       <c r="AG523" t="n">
         <v>7.150528870565083</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3413290605370065</v>
+        <v>-0.3505286798302194</v>
       </c>
       <c r="AI523" t="n">
         <v>6.96919812791216</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.1599983178840843</v>
+        <v>-0.1691979371772971</v>
       </c>
       <c r="AK523" t="n">
         <v>6.970728111892008</v>
       </c>
       <c r="AL523" t="n">
-        <v>-0.1615283018639317</v>
+        <v>-0.1707279211571446</v>
       </c>
       <c r="AM523" t="n">
         <v>-0.127636816539944</v>
@@ -85759,13 +85759,13 @@
         <v>0.04750067483060672</v>
       </c>
       <c r="AP523" t="n">
-        <v>-0.5204714121791216</v>
+        <v>-0.6146422262444703</v>
       </c>
       <c r="AQ523" t="n">
-        <v>36.2</v>
+        <v>34.8</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.02748672558764965</v>
+        <v>-0.0274896389508797</v>
       </c>
       <c r="AS523" t="n">
         <v>6.809199810028076</v>
@@ -85789,10 +85789,10 @@
         <v>75</v>
       </c>
       <c r="AZ523" t="n">
-        <v>71.90000000000001</v>
+        <v>71.48</v>
       </c>
       <c r="BA523" t="n">
-        <v>68.95955555555557</v>
+        <v>68.87555555555556</v>
       </c>
     </row>
   </sheetData>
@@ -86004,7 +86004,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.81</t>
+          <t>6.80</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -86054,12 +86054,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.82</t>
+          <t>3.81</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>2.34</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86069,7 +86069,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.18</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86109,22 +86109,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.54</t>
+          <t>-0.41</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.34</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.16</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.16</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86144,7 +86144,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-0.52</t>
+          <t>-0.61</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-05-20 12:45 EDT
Score: 71/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85637,49 +85637,49 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>4.07</v>
+        <v>4.13</v>
       </c>
       <c r="C523" t="n">
         <v>1.2617</v>
       </c>
       <c r="D523" t="n">
-        <v>2.801600000000001</v>
+        <v>2.8683</v>
       </c>
       <c r="E523" t="n">
         <v>6.800000190734863</v>
       </c>
       <c r="F523" t="n">
-        <v>6.816780090332031</v>
+        <v>6.829599857330322</v>
       </c>
       <c r="G523" t="n">
         <v>6.803</v>
       </c>
       <c r="H523" t="n">
-        <v>0.01677989959716797</v>
+        <v>0.02959966659545898</v>
       </c>
       <c r="I523" t="n">
-        <v>98.97000122070312</v>
+        <v>99.30000305175781</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>0.003334362200509533</v>
       </c>
       <c r="K523" t="n">
-        <v>2.801600000000001</v>
+        <v>2.8683</v>
       </c>
       <c r="L523" t="n">
-        <v>2.65053</v>
+        <v>2.653865</v>
       </c>
       <c r="M523" t="n">
-        <v>2.480006666666667</v>
+        <v>2.481118333333333</v>
       </c>
       <c r="N523" t="n">
         <v/>
       </c>
       <c r="O523" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="P523" t="n">
-        <v>78.74251497005989</v>
+        <v>83.63273453093812</v>
       </c>
       <c r="Q523" t="n">
         <v>1.466</v>
@@ -85694,19 +85694,19 @@
         <v>2.344</v>
       </c>
       <c r="U523" t="n">
-        <v>-5.154833382325809</v>
+        <v>-5.033687270973033</v>
       </c>
       <c r="V523" t="n">
-        <v>6.6344</v>
+        <v>6.6687</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.43529685426328</v>
+        <v>-1.930885103705759</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.1840816644107068</v>
+        <v>0.3395481738430739</v>
       </c>
       <c r="Y523" t="n">
-        <v>1.204819277108434</v>
+        <v>4.016064257028113</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85714,34 +85714,34 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.69636</v>
+        <v>1.69061</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.57212</v>
+        <v>1.57788</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.2303600000000001</v>
+        <v>0.22461</v>
       </c>
       <c r="AE523" t="n">
-        <v>15.07936507936508</v>
+        <v>11.9047619047619</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4144416644107141</v>
+        <v>0.114938173843071</v>
       </c>
       <c r="AG523" t="n">
-        <v>7.150528870565083</v>
+        <v>7.142290934762026</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3505286798302194</v>
+        <v>-0.3422907440271628</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.96919812791216</v>
+        <v>6.958225902093972</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.1691979371772971</v>
+        <v>-0.1582257113591083</v>
       </c>
       <c r="AK523" t="n">
         <v>6.970728111892008</v>
@@ -85759,40 +85759,205 @@
         <v>0.04750067483060672</v>
       </c>
       <c r="AP523" t="n">
-        <v>-0.6146422262444703</v>
+        <v>-0.5023195973522656</v>
       </c>
       <c r="AQ523" t="n">
-        <v>34.8</v>
+        <v>36.2</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.0274896389508797</v>
+        <v>-0.02847560855589688</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.809199810028076</v>
+        <v>6.808553290173504</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.006199810028076236</v>
+        <v>-0.005553290173503811</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.006199810028076236</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01081597547059343</v>
+        <v>-0.01078364947786481</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01295318526773368</v>
+        <v>-0.01294240993682414</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.0140753149311943</v>
+        <v>0.01407369863155787</v>
       </c>
       <c r="AY523" t="n">
-        <v>75</v>
+        <v>75.79365079365078</v>
       </c>
       <c r="AZ523" t="n">
-        <v>71.48</v>
+        <v>72.38777777777777</v>
       </c>
       <c r="BA523" t="n">
-        <v>68.87555555555556</v>
+        <v>69.05711111111111</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2552</v>
+      </c>
+      <c r="D524" t="n">
+        <v>2.8683</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.800000190734863</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.800429821014404</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.7869</v>
+      </c>
+      <c r="H524" t="n">
+        <v>0.0004296302795410156</v>
+      </c>
+      <c r="I524" t="n">
+        <v>99.30000305175781</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>2.8683</v>
+      </c>
+      <c r="L524" t="n">
+        <v>2.670785</v>
+      </c>
+      <c r="M524" t="n">
+        <v>2.494103333333333</v>
+      </c>
+      <c r="N524" t="n">
+        <v/>
+      </c>
+      <c r="O524" t="n">
+        <v>99.80000000000001</v>
+      </c>
+      <c r="P524" t="n">
+        <v>83.73253493013972</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.4655</v>
+      </c>
+      <c r="R524" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.3445</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.3445</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-5.12131566561011</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.6336</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-2.447061559815633</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.1957946052446147</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>0.8032128514056225</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.69061</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.57788</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.2251099999999999</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>13.09523809523809</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.4209046052445986</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>7.148249665764485</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.3482494750296219</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.949729636722528</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>-0.1497294459876644</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.953963455493896</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>-0.1539632647590325</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.1380359583680638</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>-0.008628156625159727</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.05751510742764021</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>-0.4094938780597987</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>-0.02839164707068662</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.800000190734863</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>-0.01310019073486313</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>-0.01310019073486313</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.0113775958908537</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.0122026671815605</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.01378854940036814</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>53.96825396825397</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>65.09888888888889</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>70.52155555555557</v>
       </c>
     </row>
   </sheetData>
@@ -85999,7 +86164,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86009,17 +86174,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.82</t>
+          <t>6.80</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.80</t>
+          <t>6.79</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.07</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86029,22 +86194,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>98.97</t>
+          <t>99.30</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>84</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86069,7 +86234,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.18</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86084,17 +86249,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86104,57 +86269,57 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
+          <t>-0.42</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>-0.35</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>-0.15</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>-0.15</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>-0.138</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>-0.0086</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>0.058</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
           <t>-0.41</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>-0.35</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>-0.17</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>-0.17</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>-0.128</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>-0.0075</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>0.048</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>-0.61</t>
-        </is>
-      </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>-0.027</t>
+          <t>-0.028</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.8092</t>
+          <t>6.8000</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -86179,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>71</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-05-20 13:51 EDT
Score: 71/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.800000190734863</v>
       </c>
       <c r="F524" t="n">
-        <v>6.800429821014404</v>
+        <v>6.800300121307373</v>
       </c>
       <c r="G524" t="n">
         <v>6.7869</v>
       </c>
       <c r="H524" t="n">
-        <v>0.0004296302795410156</v>
+        <v>0.0002999305725097656</v>
       </c>
       <c r="I524" t="n">
         <v>99.30000305175781</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-21 13:27 EDT
Score: 70/100
USD/CNY: 6.81
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.814499855041504</v>
       </c>
       <c r="F524" t="n">
-        <v>6.803679943084717</v>
+        <v>6.798550128936768</v>
       </c>
       <c r="G524" t="n">
         <v>6.7935</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01081991195678711</v>
+        <v>-0.01594972610473633</v>
       </c>
       <c r="I524" t="n">
         <v>99.11000061035156</v>

</xml_diff>

<commit_message>
auto: data update 2026-05-21 16:54 EDT
Score: 69/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.4655</v>
       </c>
       <c r="R523" t="n">
-        <v>3.83</v>
+        <v>3.79</v>
       </c>
       <c r="S523" t="n">
-        <v>2.3645</v>
+        <v>2.3245</v>
       </c>
       <c r="T523" t="n">
-        <v>2.3645</v>
+        <v>2.3245</v>
       </c>
       <c r="U523" t="n">
         <v>-5.079204361014216</v>
@@ -85703,10 +85703,10 @@
         <v>-2.139553278200423</v>
       </c>
       <c r="X523" t="n">
-        <v>0.1430018312444936</v>
+        <v>0.1038576525557833</v>
       </c>
       <c r="Y523" t="n">
-        <v>2.811244979919679</v>
+        <v>2.409638554216867</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>21.03174603174603</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.09240816875550895</v>
+        <v>-0.1315523474442193</v>
       </c>
       <c r="AG523" t="n">
         <v>7.160622228860079</v>
@@ -85811,16 +85811,16 @@
         <v>2.7848</v>
       </c>
       <c r="E524" t="n">
-        <v>6.814499855041504</v>
+        <v>6.80049991607666</v>
       </c>
       <c r="F524" t="n">
-        <v>6.79902982711792</v>
+        <v>6.799650192260742</v>
       </c>
       <c r="G524" t="n">
         <v>6.7935</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01547002792358398</v>
+        <v>-0.0008497238159179688</v>
       </c>
       <c r="I524" t="n">
         <v>99.11000061035156</v>
@@ -85850,25 +85850,25 @@
         <v>1.4655</v>
       </c>
       <c r="R524" t="n">
-        <v>3.83</v>
+        <v>3.79</v>
       </c>
       <c r="S524" t="n">
-        <v>2.3645</v>
+        <v>2.3245</v>
       </c>
       <c r="T524" t="n">
-        <v>2.3645</v>
+        <v>2.3245</v>
       </c>
       <c r="U524" t="n">
-        <v>-5.081751648398355</v>
+        <v>-5.298079584219457</v>
       </c>
       <c r="V524" t="n">
         <v>6.6263</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.761755947536926</v>
+        <v>-2.561575152215567</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.5030312003275972</v>
+        <v>-0.3341588504845339</v>
       </c>
       <c r="Y524" t="n">
         <v>0.4016064257028112</v>
@@ -85894,25 +85894,25 @@
         <v>21.23015873015873</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.7384412003275997</v>
+        <v>-0.5695688504845364</v>
       </c>
       <c r="AG524" t="n">
         <v>7.160795813755179</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3462959587136751</v>
+        <v>-0.3602958976785189</v>
       </c>
       <c r="AI524" t="n">
         <v>6.956789555379176</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.1422897003376722</v>
+        <v>-0.1562896393025159</v>
       </c>
       <c r="AK524" t="n">
         <v>6.959853578800648</v>
       </c>
       <c r="AL524" t="n">
-        <v>-0.1453537237591442</v>
+        <v>-0.159353662723988</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.1469566450661554</v>
@@ -85924,13 +85924,13 @@
         <v>0.06603756167960406</v>
       </c>
       <c r="AP524" t="n">
-        <v>-0.3277228511052615</v>
+        <v>-0.4718309230162251</v>
       </c>
       <c r="AQ524" t="n">
-        <v>39.59999999999999</v>
+        <v>34.2</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.03030691992100944</v>
+        <v>-0.03030620409286429</v>
       </c>
       <c r="AS524" t="n">
         <v>6.814499855041504</v>
@@ -85954,10 +85954,10 @@
         <v>28.57142857142857</v>
       </c>
       <c r="AZ524" t="n">
-        <v>56.38999999999999</v>
+        <v>54.77</v>
       </c>
       <c r="BA524" t="n">
-        <v>69.71622222222221</v>
+        <v>69.39222222222222</v>
       </c>
     </row>
   </sheetData>
@@ -86169,7 +86169,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.81</t>
+          <t>6.80</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.83</t>
+          <t>3.79</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.36</t>
+          <t>2.32</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,7 +86234,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.50</t>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86274,22 +86274,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.74</t>
+          <t>-0.57</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.35</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.14</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-0.33</t>
+          <t>-0.47</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86344,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>69</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-01 18:13 EDT
Score: 62/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.766200065612793</v>
       </c>
       <c r="F522" t="n">
-        <v>6.762810230255127</v>
+        <v>6.763050079345703</v>
       </c>
       <c r="G522" t="n">
         <v>6.7551</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.003389835357666016</v>
+        <v>-0.003149986267089844</v>
       </c>
       <c r="I522" t="n">
         <v>98.91000366210938</v>

</xml_diff>

<commit_message>
auto: data update 2026-06-03 17:26 EDT
Score: 63/100
USD/CNY: 6.76
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -39045,7 +39045,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X254" t="n">
@@ -39201,7 +39201,7 @@
       </c>
       <c r="W255" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X255" t="n">
@@ -39357,7 +39357,7 @@
       </c>
       <c r="W256" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X256" t="n">
@@ -39513,7 +39513,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X257" t="n">
@@ -39669,7 +39669,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X258" t="n">
@@ -39825,7 +39825,7 @@
       </c>
       <c r="W259" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X259" t="n">
@@ -39981,7 +39981,7 @@
       </c>
       <c r="W260" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X260" t="n">
@@ -40137,7 +40137,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X261" t="n">
@@ -40293,7 +40293,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X262" t="n">
@@ -40449,7 +40449,7 @@
       </c>
       <c r="W263" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X263" t="n">
@@ -40605,7 +40605,7 @@
       </c>
       <c r="W264" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X264" t="n">
@@ -40761,7 +40761,7 @@
       </c>
       <c r="W265" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X265" t="n">
@@ -40917,7 +40917,7 @@
       </c>
       <c r="W266" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X266" t="n">
@@ -41073,7 +41073,7 @@
       </c>
       <c r="W267" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X267" t="n">
@@ -41229,7 +41229,7 @@
       </c>
       <c r="W268" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X268" t="n">
@@ -41385,7 +41385,7 @@
       </c>
       <c r="W269" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X269" t="n">
@@ -41541,7 +41541,7 @@
       </c>
       <c r="W270" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X270" t="n">
@@ -41697,7 +41697,7 @@
       </c>
       <c r="W271" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X271" t="n">
@@ -41853,7 +41853,7 @@
       </c>
       <c r="W272" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X272" t="n">
@@ -42009,7 +42009,7 @@
       </c>
       <c r="W273" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X273" t="n">
@@ -42165,7 +42165,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X274" t="n">
@@ -42321,7 +42321,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X275" t="n">
@@ -42477,7 +42477,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X276" t="n">
@@ -42633,7 +42633,7 @@
       </c>
       <c r="W277" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X277" t="n">
@@ -42789,7 +42789,7 @@
       </c>
       <c r="W278" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X278" t="n">
@@ -42945,7 +42945,7 @@
       </c>
       <c r="W279" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X279" t="n">
@@ -43101,7 +43101,7 @@
       </c>
       <c r="W280" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X280" t="n">
@@ -43257,7 +43257,7 @@
       </c>
       <c r="W281" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X281" t="n">
@@ -43413,7 +43413,7 @@
       </c>
       <c r="W282" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X282" t="n">
@@ -43569,7 +43569,7 @@
       </c>
       <c r="W283" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X283" t="n">
@@ -43725,7 +43725,7 @@
       </c>
       <c r="W284" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X284" t="n">
@@ -43881,7 +43881,7 @@
       </c>
       <c r="W285" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X285" t="n">
@@ -44037,7 +44037,7 @@
       </c>
       <c r="W286" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X286" t="n">
@@ -44193,7 +44193,7 @@
       </c>
       <c r="W287" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X287" t="n">
@@ -44349,7 +44349,7 @@
       </c>
       <c r="W288" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X288" t="n">
@@ -44505,7 +44505,7 @@
       </c>
       <c r="W289" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X289" t="n">
@@ -44661,7 +44661,7 @@
       </c>
       <c r="W290" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X290" t="n">
@@ -44817,7 +44817,7 @@
       </c>
       <c r="W291" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X291" t="n">
@@ -44973,7 +44973,7 @@
       </c>
       <c r="W292" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X292" t="n">
@@ -45129,7 +45129,7 @@
       </c>
       <c r="W293" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X293" t="n">
@@ -45285,7 +45285,7 @@
       </c>
       <c r="W294" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X294" t="n">
@@ -45441,7 +45441,7 @@
       </c>
       <c r="W295" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X295" t="n">
@@ -45597,7 +45597,7 @@
       </c>
       <c r="W296" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X296" t="n">
@@ -45753,7 +45753,7 @@
       </c>
       <c r="W297" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X297" t="n">
@@ -45909,7 +45909,7 @@
       </c>
       <c r="W298" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X298" t="n">
@@ -46065,7 +46065,7 @@
       </c>
       <c r="W299" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X299" t="n">
@@ -46221,7 +46221,7 @@
       </c>
       <c r="W300" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X300" t="n">
@@ -46377,7 +46377,7 @@
       </c>
       <c r="W301" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X301" t="n">
@@ -46533,7 +46533,7 @@
       </c>
       <c r="W302" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X302" t="n">
@@ -46689,7 +46689,7 @@
       </c>
       <c r="W303" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X303" t="n">
@@ -46845,7 +46845,7 @@
       </c>
       <c r="W304" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X304" t="n">
@@ -47001,7 +47001,7 @@
       </c>
       <c r="W305" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X305" t="n">
@@ -47157,7 +47157,7 @@
       </c>
       <c r="W306" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X306" t="n">
@@ -47313,7 +47313,7 @@
       </c>
       <c r="W307" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X307" t="n">
@@ -47469,7 +47469,7 @@
       </c>
       <c r="W308" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X308" t="n">
@@ -47625,7 +47625,7 @@
       </c>
       <c r="W309" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X309" t="n">
@@ -47781,7 +47781,7 @@
       </c>
       <c r="W310" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X310" t="n">
@@ -47937,7 +47937,7 @@
       </c>
       <c r="W311" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X311" t="n">
@@ -48093,7 +48093,7 @@
       </c>
       <c r="W312" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X312" t="n">
@@ -48249,7 +48249,7 @@
       </c>
       <c r="W313" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X313" t="n">
@@ -48405,7 +48405,7 @@
       </c>
       <c r="W314" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X314" t="n">
@@ -48561,7 +48561,7 @@
       </c>
       <c r="W315" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X315" t="n">
@@ -48717,7 +48717,7 @@
       </c>
       <c r="W316" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X316" t="n">
@@ -48873,7 +48873,7 @@
       </c>
       <c r="W317" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X317" t="n">
@@ -49029,7 +49029,7 @@
       </c>
       <c r="W318" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X318" t="n">
@@ -49185,7 +49185,7 @@
       </c>
       <c r="W319" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X319" t="n">
@@ -49341,7 +49341,7 @@
       </c>
       <c r="W320" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X320" t="n">
@@ -49497,7 +49497,7 @@
       </c>
       <c r="W321" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X321" t="n">
@@ -49653,7 +49653,7 @@
       </c>
       <c r="W322" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X322" t="n">
@@ -49809,7 +49809,7 @@
       </c>
       <c r="W323" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X323" t="n">
@@ -49965,7 +49965,7 @@
       </c>
       <c r="W324" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X324" t="n">
@@ -50121,7 +50121,7 @@
       </c>
       <c r="W325" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X325" t="n">
@@ -50277,7 +50277,7 @@
       </c>
       <c r="W326" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X326" t="n">
@@ -50433,7 +50433,7 @@
       </c>
       <c r="W327" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X327" t="n">
@@ -50589,7 +50589,7 @@
       </c>
       <c r="W328" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X328" t="n">
@@ -50745,7 +50745,7 @@
       </c>
       <c r="W329" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X329" t="n">
@@ -50901,7 +50901,7 @@
       </c>
       <c r="W330" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X330" t="n">
@@ -51057,7 +51057,7 @@
       </c>
       <c r="W331" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X331" t="n">
@@ -51213,7 +51213,7 @@
       </c>
       <c r="W332" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X332" t="n">
@@ -51369,7 +51369,7 @@
       </c>
       <c r="W333" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X333" t="n">
@@ -51525,7 +51525,7 @@
       </c>
       <c r="W334" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X334" t="n">
@@ -51681,7 +51681,7 @@
       </c>
       <c r="W335" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X335" t="n">
@@ -51837,7 +51837,7 @@
       </c>
       <c r="W336" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X336" t="n">
@@ -51993,7 +51993,7 @@
       </c>
       <c r="W337" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X337" t="n">
@@ -52149,7 +52149,7 @@
       </c>
       <c r="W338" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X338" t="n">
@@ -52305,7 +52305,7 @@
       </c>
       <c r="W339" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X339" t="n">
@@ -52461,7 +52461,7 @@
       </c>
       <c r="W340" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X340" t="n">
@@ -52617,7 +52617,7 @@
       </c>
       <c r="W341" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X341" t="n">
@@ -52773,7 +52773,7 @@
       </c>
       <c r="W342" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X342" t="n">
@@ -52929,7 +52929,7 @@
       </c>
       <c r="W343" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X343" t="n">
@@ -53085,7 +53085,7 @@
       </c>
       <c r="W344" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X344" t="n">
@@ -53241,7 +53241,7 @@
       </c>
       <c r="W345" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X345" t="n">
@@ -53397,7 +53397,7 @@
       </c>
       <c r="W346" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X346" t="n">
@@ -53553,7 +53553,7 @@
       </c>
       <c r="W347" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X347" t="n">
@@ -53709,7 +53709,7 @@
       </c>
       <c r="W348" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X348" t="n">
@@ -53865,7 +53865,7 @@
       </c>
       <c r="W349" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X349" t="n">
@@ -54021,7 +54021,7 @@
       </c>
       <c r="W350" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X350" t="n">
@@ -54177,7 +54177,7 @@
       </c>
       <c r="W351" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X351" t="n">
@@ -54333,7 +54333,7 @@
       </c>
       <c r="W352" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X352" t="n">
@@ -54489,7 +54489,7 @@
       </c>
       <c r="W353" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X353" t="n">
@@ -54797,7 +54797,7 @@
       </c>
       <c r="W355" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X355" t="n">
@@ -54953,7 +54953,7 @@
       </c>
       <c r="W356" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X356" t="n">
@@ -55109,7 +55109,7 @@
       </c>
       <c r="W357" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X357" t="n">
@@ -55265,7 +55265,7 @@
       </c>
       <c r="W358" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X358" t="n">
@@ -55421,7 +55421,7 @@
       </c>
       <c r="W359" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X359" t="n">
@@ -55577,7 +55577,7 @@
       </c>
       <c r="W360" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X360" t="n">
@@ -55733,7 +55733,7 @@
       </c>
       <c r="W361" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X361" t="n">
@@ -55889,7 +55889,7 @@
       </c>
       <c r="W362" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X362" t="n">
@@ -56045,7 +56045,7 @@
       </c>
       <c r="W363" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X363" t="n">
@@ -56201,7 +56201,7 @@
       </c>
       <c r="W364" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X364" t="n">
@@ -56357,7 +56357,7 @@
       </c>
       <c r="W365" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X365" t="n">
@@ -56513,7 +56513,7 @@
       </c>
       <c r="W366" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X366" t="n">
@@ -56669,7 +56669,7 @@
       </c>
       <c r="W367" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X367" t="n">
@@ -56825,7 +56825,7 @@
       </c>
       <c r="W368" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X368" t="n">
@@ -56981,7 +56981,7 @@
       </c>
       <c r="W369" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X369" t="n">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="W370" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X370" t="n">
@@ -57293,7 +57293,7 @@
       </c>
       <c r="W371" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X371" t="n">
@@ -57449,7 +57449,7 @@
       </c>
       <c r="W372" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X372" t="n">
@@ -57605,7 +57605,7 @@
       </c>
       <c r="W373" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X373" t="n">
@@ -57761,7 +57761,7 @@
       </c>
       <c r="W374" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X374" t="n">
@@ -57917,7 +57917,7 @@
       </c>
       <c r="W375" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X375" t="n">
@@ -58073,7 +58073,7 @@
       </c>
       <c r="W376" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X376" t="n">
@@ -58229,7 +58229,7 @@
       </c>
       <c r="W377" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X377" t="n">
@@ -58385,7 +58385,7 @@
       </c>
       <c r="W378" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X378" t="n">
@@ -58541,7 +58541,7 @@
       </c>
       <c r="W379" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X379" t="n">
@@ -58697,7 +58697,7 @@
       </c>
       <c r="W380" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X380" t="n">
@@ -58853,7 +58853,7 @@
       </c>
       <c r="W381" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X381" t="n">
@@ -59009,7 +59009,7 @@
       </c>
       <c r="W382" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X382" t="n">
@@ -59165,7 +59165,7 @@
       </c>
       <c r="W383" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X383" t="n">
@@ -59321,7 +59321,7 @@
       </c>
       <c r="W384" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X384" t="n">
@@ -59477,7 +59477,7 @@
       </c>
       <c r="W385" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X385" t="n">
@@ -59633,7 +59633,7 @@
       </c>
       <c r="W386" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X386" t="n">
@@ -59789,7 +59789,7 @@
       </c>
       <c r="W387" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X387" t="n">
@@ -59945,7 +59945,7 @@
       </c>
       <c r="W388" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X388" t="n">
@@ -60101,7 +60101,7 @@
       </c>
       <c r="W389" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X389" t="n">
@@ -60257,7 +60257,7 @@
       </c>
       <c r="W390" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X390" t="n">
@@ -60413,7 +60413,7 @@
       </c>
       <c r="W391" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X391" t="n">
@@ -60569,7 +60569,7 @@
       </c>
       <c r="W392" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X392" t="n">
@@ -60725,7 +60725,7 @@
       </c>
       <c r="W393" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X393" t="n">
@@ -60881,7 +60881,7 @@
       </c>
       <c r="W394" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X394" t="n">
@@ -61037,7 +61037,7 @@
       </c>
       <c r="W395" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X395" t="n">
@@ -61193,7 +61193,7 @@
       </c>
       <c r="W396" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X396" t="n">
@@ -61349,7 +61349,7 @@
       </c>
       <c r="W397" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X397" t="n">
@@ -61505,7 +61505,7 @@
       </c>
       <c r="W398" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X398" t="n">
@@ -61661,7 +61661,7 @@
       </c>
       <c r="W399" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X399" t="n">
@@ -61817,7 +61817,7 @@
       </c>
       <c r="W400" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X400" t="n">
@@ -61973,7 +61973,7 @@
       </c>
       <c r="W401" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X401" t="n">
@@ -62129,7 +62129,7 @@
       </c>
       <c r="W402" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X402" t="n">
@@ -62285,7 +62285,7 @@
       </c>
       <c r="W403" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X403" t="n">
@@ -62441,7 +62441,7 @@
       </c>
       <c r="W404" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X404" t="n">
@@ -62597,7 +62597,7 @@
       </c>
       <c r="W405" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X405" t="n">
@@ -62753,7 +62753,7 @@
       </c>
       <c r="W406" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X406" t="n">
@@ -62909,7 +62909,7 @@
       </c>
       <c r="W407" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X407" t="n">
@@ -63065,7 +63065,7 @@
       </c>
       <c r="W408" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X408" t="n">
@@ -63221,7 +63221,7 @@
       </c>
       <c r="W409" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X409" t="n">
@@ -63377,7 +63377,7 @@
       </c>
       <c r="W410" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X410" t="n">
@@ -63533,7 +63533,7 @@
       </c>
       <c r="W411" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X411" t="n">
@@ -63689,7 +63689,7 @@
       </c>
       <c r="W412" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X412" t="n">
@@ -63845,7 +63845,7 @@
       </c>
       <c r="W413" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X413" t="n">
@@ -64001,7 +64001,7 @@
       </c>
       <c r="W414" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X414" t="n">
@@ -64157,7 +64157,7 @@
       </c>
       <c r="W415" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X415" t="n">
@@ -64313,7 +64313,7 @@
       </c>
       <c r="W416" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X416" t="n">
@@ -64469,7 +64469,7 @@
       </c>
       <c r="W417" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X417" t="n">
@@ -64625,7 +64625,7 @@
       </c>
       <c r="W418" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X418" t="n">
@@ -64781,7 +64781,7 @@
       </c>
       <c r="W419" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X419" t="n">
@@ -64937,7 +64937,7 @@
       </c>
       <c r="W420" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X420" t="n">
@@ -65093,7 +65093,7 @@
       </c>
       <c r="W421" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X421" t="n">
@@ -65249,7 +65249,7 @@
       </c>
       <c r="W422" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X422" t="n">
@@ -65405,7 +65405,7 @@
       </c>
       <c r="W423" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X423" t="n">
@@ -65561,7 +65561,7 @@
       </c>
       <c r="W424" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X424" t="n">
@@ -65717,7 +65717,7 @@
       </c>
       <c r="W425" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X425" t="n">
@@ -65873,7 +65873,7 @@
       </c>
       <c r="W426" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X426" t="n">
@@ -66029,7 +66029,7 @@
       </c>
       <c r="W427" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X427" t="n">
@@ -66185,7 +66185,7 @@
       </c>
       <c r="W428" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X428" t="n">
@@ -66341,7 +66341,7 @@
       </c>
       <c r="W429" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X429" t="n">
@@ -66649,7 +66649,7 @@
       </c>
       <c r="W431" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X431" t="n">
@@ -66805,7 +66805,7 @@
       </c>
       <c r="W432" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X432" t="n">
@@ -66961,7 +66961,7 @@
       </c>
       <c r="W433" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X433" t="n">
@@ -67117,7 +67117,7 @@
       </c>
       <c r="W434" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X434" t="n">
@@ -67273,7 +67273,7 @@
       </c>
       <c r="W435" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X435" t="n">
@@ -67429,7 +67429,7 @@
       </c>
       <c r="W436" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X436" t="n">
@@ -67585,7 +67585,7 @@
       </c>
       <c r="W437" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X437" t="n">
@@ -67741,7 +67741,7 @@
       </c>
       <c r="W438" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X438" t="n">
@@ -67897,7 +67897,7 @@
       </c>
       <c r="W439" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X439" t="n">
@@ -68053,7 +68053,7 @@
       </c>
       <c r="W440" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X440" t="n">
@@ -68209,7 +68209,7 @@
       </c>
       <c r="W441" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X441" t="n">
@@ -68365,7 +68365,7 @@
       </c>
       <c r="W442" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X442" t="n">
@@ -68521,7 +68521,7 @@
       </c>
       <c r="W443" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X443" t="n">
@@ -68677,7 +68677,7 @@
       </c>
       <c r="W444" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X444" t="n">
@@ -68833,7 +68833,7 @@
       </c>
       <c r="W445" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X445" t="n">
@@ -68989,7 +68989,7 @@
       </c>
       <c r="W446" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X446" t="n">
@@ -69145,7 +69145,7 @@
       </c>
       <c r="W447" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X447" t="n">
@@ -69301,7 +69301,7 @@
       </c>
       <c r="W448" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X448" t="n">
@@ -69457,7 +69457,7 @@
       </c>
       <c r="W449" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X449" t="n">
@@ -69613,7 +69613,7 @@
       </c>
       <c r="W450" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X450" t="n">
@@ -69769,7 +69769,7 @@
       </c>
       <c r="W451" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X451" t="n">
@@ -70077,7 +70077,7 @@
       </c>
       <c r="W453" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X453" t="n">
@@ -70233,7 +70233,7 @@
       </c>
       <c r="W454" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X454" t="n">
@@ -70389,7 +70389,7 @@
       </c>
       <c r="W455" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X455" t="n">
@@ -70545,7 +70545,7 @@
       </c>
       <c r="W456" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X456" t="n">
@@ -70701,7 +70701,7 @@
       </c>
       <c r="W457" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X457" t="n">
@@ -70857,7 +70857,7 @@
       </c>
       <c r="W458" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X458" t="n">
@@ -71013,7 +71013,7 @@
       </c>
       <c r="W459" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X459" t="n">
@@ -71169,7 +71169,7 @@
       </c>
       <c r="W460" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X460" t="n">
@@ -71325,7 +71325,7 @@
       </c>
       <c r="W461" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X461" t="n">
@@ -71481,7 +71481,7 @@
       </c>
       <c r="W462" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X462" t="n">
@@ -71637,7 +71637,7 @@
       </c>
       <c r="W463" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X463" t="n">
@@ -71793,7 +71793,7 @@
       </c>
       <c r="W464" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X464" t="n">
@@ -71949,7 +71949,7 @@
       </c>
       <c r="W465" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X465" t="n">
@@ -72105,7 +72105,7 @@
       </c>
       <c r="W466" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X466" t="n">
@@ -72261,7 +72261,7 @@
       </c>
       <c r="W467" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X467" t="n">
@@ -72417,7 +72417,7 @@
       </c>
       <c r="W468" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X468" t="n">
@@ -72573,7 +72573,7 @@
       </c>
       <c r="W469" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X469" t="n">
@@ -72729,7 +72729,7 @@
       </c>
       <c r="W470" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X470" t="n">
@@ -72885,7 +72885,7 @@
       </c>
       <c r="W471" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X471" t="n">
@@ -73041,7 +73041,7 @@
       </c>
       <c r="W472" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X472" t="n">
@@ -73197,7 +73197,7 @@
       </c>
       <c r="W473" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X473" t="n">
@@ -73353,7 +73353,7 @@
       </c>
       <c r="W474" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X474" t="n">
@@ -73509,7 +73509,7 @@
       </c>
       <c r="W475" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X475" t="n">
@@ -73665,7 +73665,7 @@
       </c>
       <c r="W476" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X476" t="n">
@@ -73821,7 +73821,7 @@
       </c>
       <c r="W477" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X477" t="n">
@@ -73977,7 +73977,7 @@
       </c>
       <c r="W478" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X478" t="n">
@@ -74133,7 +74133,7 @@
       </c>
       <c r="W479" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X479" t="n">
@@ -74289,7 +74289,7 @@
       </c>
       <c r="W480" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X480" t="n">
@@ -74445,7 +74445,7 @@
       </c>
       <c r="W481" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X481" t="n">
@@ -74601,7 +74601,7 @@
       </c>
       <c r="W482" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X482" t="n">
@@ -74757,7 +74757,7 @@
       </c>
       <c r="W483" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X483" t="n">
@@ -74913,7 +74913,7 @@
       </c>
       <c r="W484" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X484" t="n">
@@ -75069,7 +75069,7 @@
       </c>
       <c r="W485" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X485" t="n">
@@ -75225,7 +75225,7 @@
       </c>
       <c r="W486" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X486" t="n">
@@ -75381,7 +75381,7 @@
       </c>
       <c r="W487" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X487" t="n">
@@ -75537,7 +75537,7 @@
       </c>
       <c r="W488" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X488" t="n">
@@ -75693,7 +75693,7 @@
       </c>
       <c r="W489" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X489" t="n">
@@ -75849,7 +75849,7 @@
       </c>
       <c r="W490" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X490" t="n">
@@ -76005,7 +76005,7 @@
       </c>
       <c r="W491" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X491" t="n">
@@ -76161,7 +76161,7 @@
       </c>
       <c r="W492" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X492" t="n">
@@ -76317,7 +76317,7 @@
       </c>
       <c r="W493" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X493" t="n">
@@ -76473,7 +76473,7 @@
       </c>
       <c r="W494" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X494" t="n">
@@ -76629,7 +76629,7 @@
       </c>
       <c r="W495" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X495" t="n">
@@ -76785,7 +76785,7 @@
       </c>
       <c r="W496" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X496" t="n">
@@ -76941,7 +76941,7 @@
       </c>
       <c r="W497" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X497" t="n">
@@ -77097,7 +77097,7 @@
       </c>
       <c r="W498" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X498" t="n">
@@ -77253,7 +77253,7 @@
       </c>
       <c r="W499" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>cip_proxy_2y_theoretical</t>
         </is>
       </c>
       <c r="X499" t="n">
@@ -77399,17 +77399,17 @@
         <v>6.6687</v>
       </c>
       <c r="T500" t="n">
-        <v/>
+        <v>-2.46873993437744</v>
       </c>
       <c r="U500" t="n">
-        <v>7.900767654244428</v>
+        <v>-0.1565270438312893</v>
       </c>
       <c r="V500" t="n">
-        <v>72.54098360655738</v>
+        <v>0.4098360655737705</v>
       </c>
       <c r="W500" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X500" t="n">
@@ -77428,7 +77428,7 @@
         <v>8.730158730158729</v>
       </c>
       <c r="AC500" t="n">
-        <v/>
+        <v>-0.370587043831283</v>
       </c>
       <c r="AD500" t="n">
         <v>7.198244388757949</v>
@@ -77555,17 +77555,17 @@
         <v>6.6687</v>
       </c>
       <c r="T501" t="n">
-        <v/>
+        <v>-2.323027698362734</v>
       </c>
       <c r="U501" t="n">
-        <v>8.136673550765465</v>
+        <v>-0.005161173059220481</v>
       </c>
       <c r="V501" t="n">
-        <v>77.14285714285714</v>
+        <v>0.8163265306122449</v>
       </c>
       <c r="W501" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X501" t="n">
@@ -77584,7 +77584,7 @@
         <v>8.928571428571429</v>
       </c>
       <c r="AC501" t="n">
-        <v/>
+        <v>-0.2192211730592142</v>
       </c>
       <c r="AD501" t="n">
         <v>7.203612218600632</v>
@@ -77711,17 +77711,17 @@
         <v>6.6687</v>
       </c>
       <c r="T502" t="n">
-        <v/>
+        <v>-2.32588604307562</v>
       </c>
       <c r="U502" t="n">
-        <v>7.771185663190558</v>
+        <v>0.06024145822289828</v>
       </c>
       <c r="V502" t="n">
-        <v>69.51219512195122</v>
+        <v>1.219512195121951</v>
       </c>
       <c r="W502" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X502" t="n">
@@ -77740,7 +77740,7 @@
         <v>9.523809523809524</v>
       </c>
       <c r="AC502" t="n">
-        <v/>
+        <v>-0.1547285417770938</v>
       </c>
       <c r="AD502" t="n">
         <v>7.178869340768765</v>
@@ -77867,17 +77867,17 @@
         <v>6.6687</v>
       </c>
       <c r="T503" t="n">
-        <v/>
+        <v>-2.361638733643368</v>
       </c>
       <c r="U503" t="n">
-        <v>7.781966317042674</v>
+        <v>0.003548864124436335</v>
       </c>
       <c r="V503" t="n">
-        <v>69.63562753036437</v>
+        <v>1.214574898785425</v>
       </c>
       <c r="W503" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X503" t="n">
@@ -77896,7 +77896,7 @@
         <v>7.142857142857142</v>
       </c>
       <c r="AC503" t="n">
-        <v/>
+        <v>-0.2077811358755621</v>
       </c>
       <c r="AD503" t="n">
         <v>7.182234379225464</v>
@@ -78023,17 +78023,17 @@
         <v>6.6687</v>
       </c>
       <c r="T504" t="n">
-        <v/>
+        <v>-2.363070205458651</v>
       </c>
       <c r="U504" t="n">
-        <v>7.956809029103583</v>
+        <v>-0.05552102240991008</v>
       </c>
       <c r="V504" t="n">
-        <v>73.38709677419354</v>
+        <v>0.8064516129032258</v>
       </c>
       <c r="W504" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X504" t="n">
@@ -78052,7 +78052,7 @@
         <v>14.68253968253968</v>
       </c>
       <c r="AC504" t="n">
-        <v/>
+        <v>-0.2863410224099194</v>
       </c>
       <c r="AD504" t="n">
         <v>7.196672146399949</v>
@@ -78179,17 +78179,17 @@
         <v>6.6687</v>
       </c>
       <c r="T505" t="n">
-        <v/>
+        <v>-2.089265497137927</v>
       </c>
       <c r="U505" t="n">
-        <v>8.152546196656434</v>
+        <v>0.278835295374269</v>
       </c>
       <c r="V505" t="n">
-        <v>78.31325301204819</v>
+        <v>2.409638554216867</v>
       </c>
       <c r="W505" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X505" t="n">
@@ -78208,7 +78208,7 @@
         <v>15.47619047619047</v>
       </c>
       <c r="AC505" t="n">
-        <v/>
+        <v>0.0479252953742515</v>
       </c>
       <c r="AD505" t="n">
         <v>7.185921315615053</v>
@@ -78335,17 +78335,17 @@
         <v>6.6687</v>
       </c>
       <c r="T506" t="n">
-        <v/>
+        <v>-1.951071559223949</v>
       </c>
       <c r="U506" t="n">
-        <v>8.557520338731486</v>
+        <v>0.4038366499663049</v>
       </c>
       <c r="V506" t="n">
-        <v>87.14859437751004</v>
+        <v>2.811244979919679</v>
       </c>
       <c r="W506" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X506" t="n">
@@ -78364,7 +78364,7 @@
         <v>17.85714285714286</v>
       </c>
       <c r="AC506" t="n">
-        <v/>
+        <v>0.1691966499663078</v>
       </c>
       <c r="AD506" t="n">
         <v>7.205289115113832</v>
@@ -78491,17 +78491,17 @@
         <v>6.6687</v>
       </c>
       <c r="T507" t="n">
-        <v/>
+        <v>-1.938091577136547</v>
       </c>
       <c r="U507" t="n">
-        <v>8.254502757002351</v>
+        <v>0.4663538055665661</v>
       </c>
       <c r="V507" t="n">
-        <v>80.72289156626506</v>
+        <v>3.21285140562249</v>
       </c>
       <c r="W507" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X507" t="n">
@@ -78520,7 +78520,7 @@
         <v>16.26984126984127</v>
       </c>
       <c r="AC507" t="n">
-        <v/>
+        <v>0.2335338055665659</v>
       </c>
       <c r="AD507" t="n">
         <v>7.180131210881666</v>
@@ -78647,17 +78647,17 @@
         <v>6.6687</v>
       </c>
       <c r="T508" t="n">
-        <v/>
+        <v>-1.855828108438273</v>
       </c>
       <c r="U508" t="n">
-        <v>8.328792365406855</v>
+        <v>0.6009387672241795</v>
       </c>
       <c r="V508" t="n">
-        <v>81.92771084337349</v>
+        <v>4.016064257028113</v>
       </c>
       <c r="W508" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X508" t="n">
@@ -78676,7 +78676,7 @@
         <v>11.50793650793651</v>
       </c>
       <c r="AC508" t="n">
-        <v/>
+        <v>0.3766087672241847</v>
       </c>
       <c r="AD508" t="n">
         <v>7.17574294218218</v>
@@ -78803,17 +78803,17 @@
         <v>6.6687</v>
       </c>
       <c r="T509" t="n">
-        <v/>
+        <v>-1.81536837777635</v>
       </c>
       <c r="U509" t="n">
-        <v>8.401350673107018</v>
+        <v>0.6243799607881462</v>
       </c>
       <c r="V509" t="n">
-        <v>83.13253012048193</v>
+        <v>4.417670682730924</v>
       </c>
       <c r="W509" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X509" t="n">
@@ -78832,7 +78832,7 @@
         <v>16.26984126984127</v>
       </c>
       <c r="AC509" t="n">
-        <v/>
+        <v>0.3932899607881568</v>
       </c>
       <c r="AD509" t="n">
         <v>7.178671808187673</v>
@@ -78959,17 +78959,17 @@
         <v>6.6687</v>
       </c>
       <c r="T510" t="n">
-        <v/>
+        <v>-1.798022219819195</v>
       </c>
       <c r="U510" t="n">
-        <v>8.229903981282138</v>
+        <v>0.6620568913880298</v>
       </c>
       <c r="V510" t="n">
-        <v>78.714859437751</v>
+        <v>4.819277108433734</v>
       </c>
       <c r="W510" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X510" t="n">
@@ -78988,7 +78988,7 @@
         <v>19.44444444444444</v>
       </c>
       <c r="AC510" t="n">
-        <v/>
+        <v>0.4273268913880246</v>
       </c>
       <c r="AD510" t="n">
         <v>7.164579583772624</v>
@@ -79115,17 +79115,17 @@
         <v>6.6687</v>
       </c>
       <c r="T511" t="n">
-        <v/>
+        <v>-1.715523477963132</v>
       </c>
       <c r="U511" t="n">
-        <v>8.299443970135634</v>
+        <v>0.8363116117881653</v>
       </c>
       <c r="V511" t="n">
-        <v>80.72289156626506</v>
+        <v>5.220883534136546</v>
       </c>
       <c r="W511" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X511" t="n">
@@ -79144,7 +79144,7 @@
         <v>18.45238095238095</v>
       </c>
       <c r="AC511" t="n">
-        <v/>
+        <v>0.6024916117881585</v>
       </c>
       <c r="AD511" t="n">
         <v>7.157109643412745</v>
@@ -79271,17 +79271,17 @@
         <v>6.6687</v>
       </c>
       <c r="T512" t="n">
-        <v/>
+        <v>-2.063382099922495</v>
       </c>
       <c r="U512" t="n">
-        <v>7.835501738263791</v>
+        <v>0.4556382486106569</v>
       </c>
       <c r="V512" t="n">
-        <v>67.8714859437751</v>
+        <v>3.21285140562249</v>
       </c>
       <c r="W512" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X512" t="n">
@@ -79300,7 +79300,7 @@
         <v>14.48412698412698</v>
       </c>
       <c r="AC512" t="n">
-        <v/>
+        <v>0.2262782486106563</v>
       </c>
       <c r="AD512" t="n">
         <v>7.151968237626934</v>
@@ -79427,17 +79427,17 @@
         <v>6.6687</v>
       </c>
       <c r="T513" t="n">
-        <v/>
+        <v>-1.930885103705759</v>
       </c>
       <c r="U513" t="n">
-        <v>7.901987270973033</v>
+        <v>0.6533693415111896</v>
       </c>
       <c r="V513" t="n">
-        <v>69.47791164658635</v>
+        <v>5.220883534136546</v>
       </c>
       <c r="W513" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X513" t="n">
@@ -79456,7 +79456,7 @@
         <v>11.9047619047619</v>
       </c>
       <c r="AC513" t="n">
-        <v/>
+        <v>0.4287593415111868</v>
       </c>
       <c r="AD513" t="n">
         <v>7.142290934762026</v>
@@ -79583,17 +79583,17 @@
         <v>6.6687</v>
       </c>
       <c r="T514" t="n">
-        <v/>
+        <v>-2.139553278200423</v>
       </c>
       <c r="U514" t="n">
-        <v>7.864004361014215</v>
+        <v>0.3485087693602784</v>
       </c>
       <c r="V514" t="n">
-        <v>68.67469879518072</v>
+        <v>2.811244979919679</v>
       </c>
       <c r="W514" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X514" t="n">
@@ -79612,7 +79612,7 @@
         <v>21.03174603174603</v>
       </c>
       <c r="AC514" t="n">
-        <v/>
+        <v>0.1130987693602759</v>
       </c>
       <c r="AD514" t="n">
         <v>7.160622228860079</v>
@@ -79739,17 +79739,17 @@
         <v>6.6687</v>
       </c>
       <c r="T515" t="n">
-        <v/>
+        <v>-1.938091577136547</v>
       </c>
       <c r="U515" t="n">
-        <v>8.038858872829618</v>
+        <v>0.5973342865162712</v>
       </c>
       <c r="V515" t="n">
-        <v>71.88755020080322</v>
+        <v>4.819277108433734</v>
       </c>
       <c r="W515" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X515" t="n">
@@ -79768,7 +79768,7 @@
         <v>21.42857142857143</v>
       </c>
       <c r="AC515" t="n">
-        <v/>
+        <v>0.3610142865162702</v>
       </c>
       <c r="AD515" t="n">
         <v>7.155292800845024</v>
@@ -79895,17 +79895,17 @@
         <v>6.6687</v>
       </c>
       <c r="T516" t="n">
-        <v/>
+        <v>-1.966920626535651</v>
       </c>
       <c r="U516" t="n">
-        <v>7.822994126337567</v>
+        <v>0.6133455515884068</v>
       </c>
       <c r="V516" t="n">
-        <v>65.86345381526104</v>
+        <v>5.622489959839357</v>
       </c>
       <c r="W516" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X516" t="n">
@@ -79924,7 +79924,7 @@
         <v>21.03174603174603</v>
       </c>
       <c r="AC516" t="n">
-        <v/>
+        <v>0.3782055515884064</v>
       </c>
       <c r="AD516" t="n">
         <v>7.139583642720509</v>
@@ -80051,17 +80051,17 @@
         <v>6.6687</v>
       </c>
       <c r="T517" t="n">
-        <v/>
+        <v>-1.851495716325635</v>
       </c>
       <c r="U517" t="n">
-        <v>8.082366728057</v>
+        <v>0.7345375105901164</v>
       </c>
       <c r="V517" t="n">
-        <v>72.28915662650603</v>
+        <v>7.228915662650603</v>
       </c>
       <c r="W517" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X517" t="n">
@@ -80080,7 +80080,7 @@
         <v>21.82539682539682</v>
       </c>
       <c r="AC517" t="n">
-        <v/>
+        <v>0.4983975105901095</v>
       </c>
       <c r="AD517" t="n">
         <v>7.148810398388339</v>
@@ -80207,17 +80207,17 @@
         <v>6.6687</v>
       </c>
       <c r="T518" t="n">
-        <v/>
+        <v>-1.851495716325635</v>
       </c>
       <c r="U518" t="n">
-        <v>8.056695742819171</v>
+        <v>0.6177593054497166</v>
       </c>
       <c r="V518" t="n">
-        <v>71.4859437751004</v>
+        <v>6.024096385542169</v>
       </c>
       <c r="W518" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X518" t="n">
@@ -80236,7 +80236,7 @@
         <v>25.3968253968254</v>
       </c>
       <c r="AC518" t="n">
-        <v/>
+        <v>0.3774393054497116</v>
       </c>
       <c r="AD518" t="n">
         <v>7.154472188191456</v>
@@ -80363,17 +80363,17 @@
         <v>6.6687</v>
       </c>
       <c r="T519" t="n">
-        <v/>
+        <v>-1.728555538215026</v>
       </c>
       <c r="U519" t="n">
-        <v>8.317132266711024</v>
+        <v>0.7368022402563623</v>
       </c>
       <c r="V519" t="n">
-        <v>81.12449799196787</v>
+        <v>8.032128514056225</v>
       </c>
       <c r="W519" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X519" t="n">
@@ -80392,7 +80392,7 @@
         <v>22.42063492063492</v>
       </c>
       <c r="AC519" t="n">
-        <v/>
+        <v>0.5004822402563613</v>
       </c>
       <c r="AD519" t="n">
         <v>7.162957466049544</v>
@@ -80519,17 +80519,17 @@
         <v>6.6687</v>
       </c>
       <c r="T520" t="n">
-        <v/>
+        <v>-1.624181426029248</v>
       </c>
       <c r="U520" t="n">
-        <v>8.294331618574041</v>
+        <v>0.8355137350721797</v>
       </c>
       <c r="V520" t="n">
-        <v>79.91967871485944</v>
+        <v>8.433734939759036</v>
       </c>
       <c r="W520" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X520" t="n">
@@ -80548,7 +80548,7 @@
         <v>5.952380952380952</v>
       </c>
       <c r="AC520" t="n">
-        <v/>
+        <v>0.6334337350721864</v>
       </c>
       <c r="AD520" t="n">
         <v>7.153717246231795</v>
@@ -80675,17 +80675,17 @@
         <v>6.6687</v>
       </c>
       <c r="T521" t="n">
-        <v/>
+        <v>-1.634338926243883</v>
       </c>
       <c r="U521" t="n">
-        <v>8.180994386823921</v>
+        <v>0.8151143844915998</v>
       </c>
       <c r="V521" t="n">
-        <v>76.70682730923694</v>
+        <v>8.433734939759036</v>
       </c>
       <c r="W521" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X521" t="n">
@@ -80704,7 +80704,7 @@
         <v>3.174603174603174</v>
       </c>
       <c r="AC521" t="n">
-        <v/>
+        <v>0.6269743844916187</v>
       </c>
       <c r="AD521" t="n">
         <v>7.147395974498139</v>
@@ -80831,17 +80831,17 @@
         <v>6.6687</v>
       </c>
       <c r="T522" t="n">
-        <v/>
+        <v>-1.440987033598196</v>
       </c>
       <c r="U522" t="n">
-        <v>8.406079637798825</v>
+        <v>1.086152991541067</v>
       </c>
       <c r="V522" t="n">
-        <v>83.13253012048193</v>
+        <v>11.64658634538153</v>
       </c>
       <c r="W522" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X522" t="n">
@@ -80860,7 +80860,7 @@
         <v>3.571428571428571</v>
       </c>
       <c r="AC522" t="n">
-        <v/>
+        <v>0.8970129915410796</v>
       </c>
       <c r="AD522" t="n">
         <v>7.144003000929145</v>
@@ -80987,17 +80987,17 @@
         <v>6.5909</v>
       </c>
       <c r="T523" t="n">
-        <v/>
+        <v>-2.573538358043459</v>
       </c>
       <c r="U523" t="n">
-        <v>8.575109003254395</v>
+        <v>-0.09026666154423602</v>
       </c>
       <c r="V523" t="n">
-        <v>87.95180722891567</v>
+        <v>0.8032128514056225</v>
       </c>
       <c r="W523" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X523" t="n">
@@ -81016,7 +81016,7 @@
         <v>3.174603174603174</v>
       </c>
       <c r="AC523" t="n">
-        <v/>
+        <v>-0.2777666615442209</v>
       </c>
       <c r="AD523" t="n">
         <v>7.154231507873859</v>
@@ -81089,25 +81089,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.05</v>
+        <v>4.08</v>
       </c>
       <c r="C524" t="n">
         <v>1.2352</v>
       </c>
       <c r="D524" t="n">
-        <v>2.8215</v>
+        <v>2.8448</v>
       </c>
       <c r="E524" t="n">
-        <v>6.764999866485596</v>
+        <v>6.762199878692627</v>
       </c>
       <c r="F524" t="n">
-        <v>6.780620098114014</v>
+        <v>6.777989864349365</v>
       </c>
       <c r="G524" t="n">
         <v>6.763999999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>0.01562023162841797</v>
+        <v>0.01578998565673828</v>
       </c>
       <c r="I524" t="n">
         <v>99.22000122070312</v>
@@ -81116,44 +81116,44 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>2.8215</v>
+        <v>2.8448</v>
       </c>
       <c r="L524" t="n">
-        <v>2.77142</v>
+        <v>2.772585</v>
       </c>
       <c r="M524" t="n">
-        <v>2.59926</v>
+        <v>2.599648333333334</v>
       </c>
       <c r="N524" t="n">
         <v/>
       </c>
       <c r="O524" t="n">
-        <v>97.80000000000001</v>
+        <v>98.80000000000001</v>
       </c>
       <c r="P524" t="n">
-        <v>81.33732534930139</v>
+        <v>84.03193612774452</v>
       </c>
       <c r="Q524" t="n">
         <v>1.4605</v>
       </c>
       <c r="R524" t="n">
-        <v>-5.635243321940901</v>
+        <v>-5.618070138747425</v>
       </c>
       <c r="S524" t="n">
         <v>6.5986</v>
       </c>
       <c r="T524" t="n">
-        <v/>
+        <v>-2.419329236453394</v>
       </c>
       <c r="U524" t="n">
-        <v>8.456743321940902</v>
+        <v>0.1014621306993035</v>
       </c>
       <c r="V524" t="n">
-        <v>85.14056224899598</v>
+        <v>2.811244979919679</v>
       </c>
       <c r="W524" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="X524" t="n">
@@ -81172,25 +81172,25 @@
         <v>4.365079365079365</v>
       </c>
       <c r="AC524" t="n">
-        <v/>
+        <v>-0.08803786930069446</v>
       </c>
       <c r="AD524" t="n">
-        <v>7.146224069691036</v>
+        <v>7.142105010799872</v>
       </c>
       <c r="AE524" t="n">
-        <v>-0.3812242032054405</v>
+        <v>-0.3799051321072451</v>
       </c>
       <c r="AF524" t="n">
-        <v>6.888817548231072</v>
+        <v>6.883372506719561</v>
       </c>
       <c r="AG524" t="n">
-        <v>-0.1238176817454759</v>
+        <v>-0.1211726280269341</v>
       </c>
       <c r="AH524" t="n">
         <v>6.893260360395011</v>
       </c>
       <c r="AI524" t="n">
-        <v>-0.1282604939094156</v>
+        <v>-0.1310604817023844</v>
       </c>
       <c r="AJ524" t="n">
         <v>-0.233692768734331</v>
@@ -81202,13 +81202,13 @@
         <v>0.1791295233320873</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.09513356192173777</v>
+        <v>-0.06748586878697399</v>
       </c>
       <c r="AN524" t="n">
-        <v>39.2</v>
+        <v>39.4</v>
       </c>
       <c r="AO524" t="n">
-        <v>-0.0218385226497959</v>
+        <v>-0.02183156141261109</v>
       </c>
       <c r="AP524" t="n">
         <v>6.765779972076416</v>
@@ -81232,10 +81232,10 @@
         <v>50</v>
       </c>
       <c r="AW524" t="n">
-        <v>63.49</v>
+        <v>63.9</v>
       </c>
       <c r="AX524" t="n">
-        <v>62.77</v>
+        <v>62.852</v>
       </c>
     </row>
   </sheetData>
@@ -81462,7 +81462,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.05</t>
+          <t>4.08</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -81477,17 +81477,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.82</t>
+          <t>2.84</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>84</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -81512,17 +81512,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>8.46</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>cip_proxy_2y</t>
+          <t>market_1y_us2y_subst</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -81552,7 +81552,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -81587,7 +81587,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-03 17:53 EDT
Score: 63/100
USD/CNY: 6.76
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81101,13 +81101,13 @@
         <v>6.762199878692627</v>
       </c>
       <c r="F524" t="n">
-        <v>6.777989864349365</v>
+        <v>6.778619766235352</v>
       </c>
       <c r="G524" t="n">
         <v>6.763999999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>0.01578998565673828</v>
+        <v>0.01641988754272461</v>
       </c>
       <c r="I524" t="n">
         <v>99.22000122070312</v>

</xml_diff>

<commit_message>
auto: data update 2026-06-04 13:41 EDT
Score: 63/100
USD/CNY: 6.76
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81101,13 +81101,13 @@
         <v>6.762199878692627</v>
       </c>
       <c r="F524" t="n">
-        <v>6.774020195007324</v>
+        <v>6.775619983673096</v>
       </c>
       <c r="G524" t="n">
         <v>6.7662</v>
       </c>
       <c r="H524" t="n">
-        <v>0.01182031631469727</v>
+        <v>0.01342010498046875</v>
       </c>
       <c r="I524" t="n">
         <v>99.52999877929688</v>
@@ -81452,7 +81452,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.77</t>
+          <t>6.78</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-09 12:26 EDT
Score: 66/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX522"/>
+  <dimension ref="A1:AX523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80794,10 +80794,10 @@
         <v>0.01929993133544894</v>
       </c>
       <c r="I522" t="n">
-        <v>100.0699996948242</v>
+        <v>100.0500030517578</v>
       </c>
       <c r="J522" t="n">
-        <v>0</v>
+        <v>-0.0001998265526870213</v>
       </c>
       <c r="K522" t="n">
         <v>2.8913</v>
@@ -80824,13 +80824,13 @@
         <v>-5.59620521284861</v>
       </c>
       <c r="S522" t="n">
-        <v>6.6062</v>
+        <v>6.5986</v>
       </c>
       <c r="T522" t="n">
-        <v>-2.354594147480293</v>
+        <v>-2.466928785317346</v>
       </c>
       <c r="U522" t="n">
-        <v>0.2376901953992983</v>
+        <v>0.1206936700919981</v>
       </c>
       <c r="V522" t="n">
         <v>4.016064257028113</v>
@@ -80844,10 +80844,10 @@
         <v>1.65</v>
       </c>
       <c r="Y522" t="n">
-        <v>1.57303</v>
+        <v>1.57212</v>
       </c>
       <c r="Z522" t="n">
-        <v>1.27606</v>
+        <v>1.37061</v>
       </c>
       <c r="AA522" t="n">
         <v>0.1899999999999999</v>
@@ -80856,7 +80856,7 @@
         <v>4.365079365079365</v>
       </c>
       <c r="AC522" t="n">
-        <v>0.04769019539929698</v>
+        <v>-0.06930632990800323</v>
       </c>
       <c r="AD522" t="n">
         <v>7.144111336182433</v>
@@ -80865,10 +80865,10 @@
         <v>-0.3786112675178819</v>
       </c>
       <c r="AF522" t="n">
-        <v>6.841702928065738</v>
+        <v>6.841963898035329</v>
       </c>
       <c r="AG522" t="n">
-        <v>-0.07620285940118698</v>
+        <v>-0.07646382937077778</v>
       </c>
       <c r="AH522" t="n">
         <v>6.844785316397215</v>
@@ -80886,31 +80886,31 @@
         <v>0.2277185089957525</v>
       </c>
       <c r="AM522" t="n">
-        <v>0.4128813181252697</v>
+        <v>0.4101443851821273</v>
       </c>
       <c r="AN522" t="n">
         <v>46</v>
       </c>
       <c r="AO522" t="n">
-        <v>-0.02097176910605342</v>
+        <v>-0.02091425746642509</v>
       </c>
       <c r="AP522" t="n">
-        <v>6.791</v>
+        <v>6.791028381109991</v>
       </c>
       <c r="AQ522" t="n">
-        <v>-0.01970000000000027</v>
+        <v>-0.01972838110999131</v>
       </c>
       <c r="AR522" t="n">
         <v>-0.01970000000000027</v>
       </c>
       <c r="AS522" t="n">
-        <v>-0.01201086308907922</v>
+        <v>-0.01201228214457877</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.01334723655786362</v>
+        <v>-0.01334770957636347</v>
       </c>
       <c r="AU522" t="n">
-        <v>0.01326688921921189</v>
+        <v>0.01326696017198687</v>
       </c>
       <c r="AV522" t="n">
         <v>23.01587301587302</v>
@@ -80920,6 +80920,162 @@
       </c>
       <c r="AX522" t="n">
         <v>66.87977777777778</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B523" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="C523" t="n">
+        <v>1.2706</v>
+      </c>
+      <c r="D523" t="n">
+        <v>2.8913</v>
+      </c>
+      <c r="E523" t="n">
+        <v>6.765500068664551</v>
+      </c>
+      <c r="F523" t="n">
+        <v>6.7771</v>
+      </c>
+      <c r="G523" t="n">
+        <v>6.7603</v>
+      </c>
+      <c r="H523" t="n">
+        <v>0.01159993133544912</v>
+      </c>
+      <c r="I523" t="n">
+        <v>100.0500030517578</v>
+      </c>
+      <c r="J523" t="n">
+        <v>0</v>
+      </c>
+      <c r="K523" t="n">
+        <v>2.8913</v>
+      </c>
+      <c r="L523" t="n">
+        <v>2.81591</v>
+      </c>
+      <c r="M523" t="n">
+        <v>2.634503333333333</v>
+      </c>
+      <c r="N523" t="n">
+        <v/>
+      </c>
+      <c r="O523" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="P523" t="n">
+        <v>87.32534930139721</v>
+      </c>
+      <c r="Q523" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="R523" t="n">
+        <v>-5.53612850894153</v>
+      </c>
+      <c r="S523" t="n">
+        <v>6.5945</v>
+      </c>
+      <c r="T523" t="n">
+        <v>-2.527530366255759</v>
+      </c>
+      <c r="U523" t="n">
+        <v>0.05757712354463873</v>
+      </c>
+      <c r="V523" t="n">
+        <v>3.21285140562249</v>
+      </c>
+      <c r="W523" t="inlineStr">
+        <is>
+          <t>market_1y_us2y_subst</t>
+        </is>
+      </c>
+      <c r="X523" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="Y523" t="n">
+        <v>1.57212</v>
+      </c>
+      <c r="Z523" t="n">
+        <v>1.37061</v>
+      </c>
+      <c r="AA523" t="n">
+        <v>0.1899999999999999</v>
+      </c>
+      <c r="AB523" t="n">
+        <v>4.563492063492063</v>
+      </c>
+      <c r="AC523" t="n">
+        <v>-0.1324228764553625</v>
+      </c>
+      <c r="AD523" t="n">
+        <v>7.140046846738348</v>
+      </c>
+      <c r="AE523" t="n">
+        <v>-0.374546778073797</v>
+      </c>
+      <c r="AF523" t="n">
+        <v>6.835218810322361</v>
+      </c>
+      <c r="AG523" t="n">
+        <v>-0.06971874165781067</v>
+      </c>
+      <c r="AH523" t="n">
+        <v>6.849407886968131</v>
+      </c>
+      <c r="AI523" t="n">
+        <v>-0.08390781830358041</v>
+      </c>
+      <c r="AJ523" t="n">
+        <v>-0.2668003223256258</v>
+      </c>
+      <c r="AK523" t="n">
+        <v>-0.01367989020054922</v>
+      </c>
+      <c r="AL523" t="n">
+        <v>0.2456601220977567</v>
+      </c>
+      <c r="AM523" t="n">
+        <v>0.4841164455449952</v>
+      </c>
+      <c r="AN523" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="AO523" t="n">
+        <v>-0.02086501094564525</v>
+      </c>
+      <c r="AP523" t="n">
+        <v>6.7848</v>
+      </c>
+      <c r="AQ523" t="n">
+        <v>-0.02449999999999974</v>
+      </c>
+      <c r="AR523" t="n">
+        <v>-0.02449999999999974</v>
+      </c>
+      <c r="AS523" t="n">
+        <v>-0.01291524452689878</v>
+      </c>
+      <c r="AT523" t="n">
+        <v>-0.01350141723837999</v>
+      </c>
+      <c r="AU523" t="n">
+        <v>0.01325434297922609</v>
+      </c>
+      <c r="AV523" t="n">
+        <v>13.88888888888889</v>
+      </c>
+      <c r="AW523" t="n">
+        <v>54.17111111111112</v>
+      </c>
+      <c r="AX523" t="n">
+        <v>65.57466666666667</v>
       </c>
     </row>
   </sheetData>
@@ -81126,7 +81282,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -81141,7 +81297,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.77</t>
+          <t>6.76</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -81151,12 +81307,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>100.07</t>
+          <t>100.05</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -81166,7 +81322,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>99</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -81191,17 +81347,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.61</t>
+          <t>6.59</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -81221,7 +81377,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.37</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -81231,47 +81387,47 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>-0.13</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.38</t>
+          <t>-0.37</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>-0.07</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>-0.08</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>-0.08</t>
-        </is>
-      </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.259</t>
+          <t>-0.267</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>-0.0131</t>
+          <t>-0.0137</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.228</t>
+          <t>0.246</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.41</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -81281,7 +81437,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.7910</t>
+          <t>6.7848</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -81306,7 +81462,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>66</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-09 16:17 EDT
Score: 66/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -80941,13 +80941,13 @@
         <v>6.765500068664551</v>
       </c>
       <c r="F523" t="n">
-        <v>6.777170181274414</v>
+        <v>6.777470111846924</v>
       </c>
       <c r="G523" t="n">
         <v>6.7603</v>
       </c>
       <c r="H523" t="n">
-        <v>0.01167011260986328</v>
+        <v>0.01197004318237305</v>
       </c>
       <c r="I523" t="n">
         <v>100.0500030517578</v>

</xml_diff>

<commit_message>
auto: data update 2026-06-09 17:02 EDT
Score: 65/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -80929,25 +80929,25 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>4.15</v>
+        <v>4.13</v>
       </c>
       <c r="C523" t="n">
         <v>1.2706</v>
       </c>
       <c r="D523" t="n">
-        <v>2.8913</v>
+        <v>2.8594</v>
       </c>
       <c r="E523" t="n">
         <v>6.765500068664551</v>
       </c>
       <c r="F523" t="n">
-        <v>6.777470111846924</v>
+        <v>6.777100086212158</v>
       </c>
       <c r="G523" t="n">
         <v>6.7603</v>
       </c>
       <c r="H523" t="n">
-        <v>0.01197004318237305</v>
+        <v>0.01160001754760742</v>
       </c>
       <c r="I523" t="n">
         <v>100.0500030517578</v>
@@ -80956,28 +80956,28 @@
         <v>0</v>
       </c>
       <c r="K523" t="n">
-        <v>2.8913</v>
+        <v>2.8594</v>
       </c>
       <c r="L523" t="n">
-        <v>2.81591</v>
+        <v>2.814315</v>
       </c>
       <c r="M523" t="n">
-        <v>2.634503333333333</v>
+        <v>2.633971666666667</v>
       </c>
       <c r="N523" t="n">
         <v/>
       </c>
       <c r="O523" t="n">
-        <v>99.40000000000001</v>
+        <v>98</v>
       </c>
       <c r="P523" t="n">
-        <v>87.32534930139721</v>
+        <v>85.42914171656686</v>
       </c>
       <c r="Q523" t="n">
         <v>1.46</v>
       </c>
       <c r="R523" t="n">
-        <v>-5.53612850894153</v>
+        <v>-5.576672545643703</v>
       </c>
       <c r="S523" t="n">
         <v>6.5945</v>
@@ -80986,7 +80986,7 @@
         <v>-2.527530366255759</v>
       </c>
       <c r="U523" t="n">
-        <v>0.05757712354463873</v>
+        <v>0.03808262961786379</v>
       </c>
       <c r="V523" t="n">
         <v>3.21285140562249</v>
@@ -81012,19 +81012,19 @@
         <v>4.563492063492063</v>
       </c>
       <c r="AC523" t="n">
-        <v>-0.1324228764553625</v>
+        <v>-0.1519173703821375</v>
       </c>
       <c r="AD523" t="n">
-        <v>7.140046846738348</v>
+        <v>7.142789853569273</v>
       </c>
       <c r="AE523" t="n">
-        <v>-0.374546778073797</v>
+        <v>-0.3772897849047219</v>
       </c>
       <c r="AF523" t="n">
-        <v>6.835218810322361</v>
+        <v>6.84372974060455</v>
       </c>
       <c r="AG523" t="n">
-        <v>-0.06971874165781067</v>
+        <v>-0.07822967193999908</v>
       </c>
       <c r="AH523" t="n">
         <v>6.849407886968131</v>
@@ -81042,10 +81042,10 @@
         <v>0.2456601220977567</v>
       </c>
       <c r="AM523" t="n">
-        <v>0.4841164455449952</v>
+        <v>0.3947161230837788</v>
       </c>
       <c r="AN523" t="n">
-        <v>48.4</v>
+        <v>46</v>
       </c>
       <c r="AO523" t="n">
         <v>-0.02086501094564525</v>
@@ -81072,10 +81072,10 @@
         <v>50</v>
       </c>
       <c r="AW523" t="n">
-        <v>66.81</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="AX523" t="n">
-        <v>65.658</v>
+        <v>65.41600000000001</v>
       </c>
     </row>
   </sheetData>
@@ -81302,7 +81302,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -81317,17 +81317,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>2.86</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>98</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>85</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -81352,7 +81352,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -81392,17 +81392,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>-0.15</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.37</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.08</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -81427,7 +81427,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.39</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -81462,7 +81462,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>65</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-10 13:54 EDT
Score: 62/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81097,13 +81097,13 @@
         <v>6.765500068664551</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7801</v>
+        <v>6.7802</v>
       </c>
       <c r="G524" t="n">
         <v>6.7636</v>
       </c>
       <c r="H524" t="n">
-        <v>0.01459993133544923</v>
+        <v>0.014699931335449</v>
       </c>
       <c r="I524" t="n">
         <v>99.91000366210938</v>

</xml_diff>

<commit_message>
auto: data update 2026-06-11 17:25 EDT
Score: 66/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81089,25 +81089,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.13</v>
+        <v>4.05</v>
       </c>
       <c r="C524" t="n">
         <v>1.2881</v>
       </c>
       <c r="D524" t="n">
-        <v>2.85</v>
+        <v>2.7619</v>
       </c>
       <c r="E524" t="n">
         <v>6.772500038146973</v>
       </c>
       <c r="F524" t="n">
-        <v>6.761769771575928</v>
+        <v>6.764050006866455</v>
       </c>
       <c r="G524" t="n">
         <v>6.7652</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01073026657104492</v>
+        <v>-0.008450031280517578</v>
       </c>
       <c r="I524" t="n">
         <v>99.94999694824219</v>
@@ -81116,28 +81116,28 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>2.85</v>
+        <v>2.7619</v>
       </c>
       <c r="L524" t="n">
-        <v>2.827615</v>
+        <v>2.82321</v>
       </c>
       <c r="M524" t="n">
-        <v>2.64699</v>
+        <v>2.645521666666666</v>
       </c>
       <c r="N524" t="n">
         <v/>
       </c>
       <c r="O524" t="n">
-        <v>97.40000000000001</v>
+        <v>93.2</v>
       </c>
       <c r="P524" t="n">
-        <v>85.12974051896208</v>
+        <v>77.64471057884232</v>
       </c>
       <c r="Q524" t="n">
         <v>1.463</v>
       </c>
       <c r="R524" t="n">
-        <v>-5.053151574334762</v>
+        <v>-5.214756244730081</v>
       </c>
       <c r="S524" t="n">
         <v>6.604</v>
@@ -81146,10 +81146,10 @@
         <v>-2.48800350236803</v>
       </c>
       <c r="U524" t="n">
-        <v>0.07624195298416847</v>
+        <v>-0.001767644213934716</v>
       </c>
       <c r="V524" t="n">
-        <v>4.016064257028113</v>
+        <v>2.811244979919679</v>
       </c>
       <c r="W524" t="inlineStr">
         <is>
@@ -81172,19 +81172,19 @@
         <v>3.174603174603174</v>
       </c>
       <c r="AC524" t="n">
-        <v>-0.1107580470158354</v>
+        <v>-0.1887676442139385</v>
       </c>
       <c r="AD524" t="n">
-        <v>7.114724730446419</v>
+        <v>7.125669406810589</v>
       </c>
       <c r="AE524" t="n">
-        <v>-0.3422246922994461</v>
+        <v>-0.3531693686636164</v>
       </c>
       <c r="AF524" t="n">
-        <v>6.838008652840204</v>
+        <v>6.862565363470972</v>
       </c>
       <c r="AG524" t="n">
-        <v>-0.06550861469323088</v>
+        <v>-0.0900653253239998</v>
       </c>
       <c r="AH524" t="n">
         <v>6.850973969550408</v>
@@ -81202,10 +81202,10 @@
         <v>0.2758112468611972</v>
       </c>
       <c r="AM524" t="n">
-        <v>0.5364628789273158</v>
+        <v>0.2773018968561238</v>
       </c>
       <c r="AN524" t="n">
-        <v>55.8</v>
+        <v>50</v>
       </c>
       <c r="AO524" t="n">
         <v>-0.02268959371609924</v>
@@ -81232,10 +81232,10 @@
         <v>50</v>
       </c>
       <c r="AW524" t="n">
-        <v>68.33</v>
+        <v>65.12</v>
       </c>
       <c r="AX524" t="n">
-        <v>66.934</v>
+        <v>66.292</v>
       </c>
     </row>
   </sheetData>
@@ -81462,7 +81462,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.05</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -81477,17 +81477,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>2.76</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>93</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>78</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -81512,12 +81512,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>-0.00</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -81552,17 +81552,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.11</t>
+          <t>-0.19</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.34</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -81587,7 +81587,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -81622,7 +81622,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>66</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-12 16:22 EDT
Score: 67/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81101,13 +81101,13 @@
         <v>6.772500038146973</v>
       </c>
       <c r="F524" t="n">
-        <v>6.762479782104492</v>
+        <v>6.763579845428467</v>
       </c>
       <c r="G524" t="n">
         <v>6.752000000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01002025604248047</v>
+        <v>-0.008920192718505859</v>
       </c>
       <c r="I524" t="n">
         <v>99.86000061035156</v>
@@ -81140,16 +81140,16 @@
         <v>-5.094303117933674</v>
       </c>
       <c r="S524" t="n">
-        <v>6.5986</v>
+        <v>6.5915</v>
       </c>
       <c r="T524" t="n">
-        <v>-2.567737721188013</v>
+        <v>-2.672573453340232</v>
       </c>
       <c r="U524" t="n">
-        <v>-0.08673109889614228</v>
+        <v>-0.1958126782005243</v>
       </c>
       <c r="V524" t="n">
-        <v>1.204819277108434</v>
+        <v>0.4016064257028112</v>
       </c>
       <c r="W524" t="inlineStr">
         <is>
@@ -81172,7 +81172,7 @@
         <v>2.777777777777778</v>
       </c>
       <c r="AC524" t="n">
-        <v>-0.271731098896133</v>
+        <v>-0.380812678200515</v>
       </c>
       <c r="AD524" t="n">
         <v>7.117511718752353</v>
@@ -81507,17 +81507,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.60</t>
+          <t>6.59</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.09</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -81552,7 +81552,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.27</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-12 17:06 EDT
Score: 68/100
USD/CNY: 6.78
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81089,25 +81089,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.05</v>
+        <v>4.09</v>
       </c>
       <c r="C524" t="n">
         <v>1.2937</v>
       </c>
       <c r="D524" t="n">
-        <v>2.7619</v>
+        <v>2.7963</v>
       </c>
       <c r="E524" t="n">
-        <v>6.772500038146973</v>
+        <v>6.775499820709229</v>
       </c>
       <c r="F524" t="n">
-        <v>6.763579845428467</v>
+        <v>6.760039806365967</v>
       </c>
       <c r="G524" t="n">
         <v>6.752000000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.008920192718505859</v>
+        <v>-0.01546001434326172</v>
       </c>
       <c r="I524" t="n">
         <v>99.86000061035156</v>
@@ -81116,37 +81116,37 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>2.7619</v>
+        <v>2.7963</v>
       </c>
       <c r="L524" t="n">
-        <v>2.82047</v>
+        <v>2.82219</v>
       </c>
       <c r="M524" t="n">
-        <v>2.648698333333333</v>
+        <v>2.649271666666666</v>
       </c>
       <c r="N524" t="n">
         <v/>
       </c>
       <c r="O524" t="n">
-        <v>93</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="P524" t="n">
-        <v>77.74451097804391</v>
+        <v>79.44111776447106</v>
       </c>
       <c r="Q524" t="n">
         <v>1.465</v>
       </c>
       <c r="R524" t="n">
-        <v>-5.094303117933674</v>
+        <v>-4.967053101505541</v>
       </c>
       <c r="S524" t="n">
         <v>6.5915</v>
       </c>
       <c r="T524" t="n">
-        <v>-2.672573453340232</v>
+        <v>-2.715664166159892</v>
       </c>
       <c r="U524" t="n">
-        <v>-0.1958126782005243</v>
+        <v>-0.2017348305558331</v>
       </c>
       <c r="V524" t="n">
         <v>0.4016064257028112</v>
@@ -81172,25 +81172,25 @@
         <v>2.777777777777778</v>
       </c>
       <c r="AC524" t="n">
-        <v>-0.380812678200515</v>
+        <v>-0.3867348305558238</v>
       </c>
       <c r="AD524" t="n">
-        <v>7.117511718752353</v>
+        <v>7.112042494696269</v>
       </c>
       <c r="AE524" t="n">
-        <v>-0.3450116806053805</v>
+        <v>-0.3365426739870401</v>
       </c>
       <c r="AF524" t="n">
-        <v>6.861247837162044</v>
+        <v>6.851520987708294</v>
       </c>
       <c r="AG524" t="n">
-        <v>-0.08874779901507157</v>
+        <v>-0.07602116699906514</v>
       </c>
       <c r="AH524" t="n">
         <v>6.873527983489107</v>
       </c>
       <c r="AI524" t="n">
-        <v>-0.1010279453421346</v>
+        <v>-0.09802816277987869</v>
       </c>
       <c r="AJ524" t="n">
         <v>-0.2827572515625072</v>
@@ -81202,13 +81202,13 @@
         <v>0.2854425463774819</v>
       </c>
       <c r="AM524" t="n">
-        <v>0.2953205820410048</v>
+        <v>0.4299825318573854</v>
       </c>
       <c r="AN524" t="n">
-        <v>51.8</v>
+        <v>55.4</v>
       </c>
       <c r="AO524" t="n">
-        <v>-0.02328093440495399</v>
+        <v>-0.0232937615129034</v>
       </c>
       <c r="AP524" t="n">
         <v>6.7778000831604</v>
@@ -81232,10 +81232,10 @@
         <v>70</v>
       </c>
       <c r="AW524" t="n">
-        <v>72.59</v>
+        <v>74.16</v>
       </c>
       <c r="AX524" t="n">
-        <v>67.23800000000001</v>
+        <v>67.55199999999999</v>
       </c>
     </row>
   </sheetData>
@@ -81447,7 +81447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.77</t>
+          <t>6.78</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -81462,7 +81462,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.05</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -81477,17 +81477,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.76</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>79</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -81552,17 +81552,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.38</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.35</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.09</t>
+          <t>-0.08</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -81587,7 +81587,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.30</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -81622,7 +81622,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>68</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-13 16:20 EDT
Score: 67/100
USD/CNY: 6.76
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -80984,16 +80984,16 @@
         <v>-5.175053069294153</v>
       </c>
       <c r="S523" t="n">
-        <v>6.5986</v>
+        <v>6.5915</v>
       </c>
       <c r="T523" t="n">
-        <v>-2.417891105038572</v>
+        <v>-2.52288807002421</v>
       </c>
       <c r="U523" t="n">
-        <v>0.1082171487653438</v>
+        <v>-0.001074192088212911</v>
       </c>
       <c r="V523" t="n">
-        <v>5.220883534136546</v>
+        <v>3.21285140562249</v>
       </c>
       <c r="W523" t="inlineStr">
         <is>
@@ -81016,7 +81016,7 @@
         <v>9.126984126984127</v>
       </c>
       <c r="AC523" t="n">
-        <v>-0.09345285123465441</v>
+        <v>-0.2027441920882112</v>
       </c>
       <c r="AD523" t="n">
         <v>7.112042494696269</v>
@@ -81351,17 +81351,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.60</t>
+          <t>6.59</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.11</t>
+          <t>-0.00</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -81396,7 +81396,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.09</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-15 17:15 EDT
Score: 68/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -80777,25 +80777,25 @@
         </is>
       </c>
       <c r="B522" t="n">
-        <v>4.09</v>
+        <v>4.07</v>
       </c>
       <c r="C522" t="n">
         <v>1.3012</v>
       </c>
       <c r="D522" t="n">
-        <v>2.7963</v>
+        <v>2.768800000000001</v>
       </c>
       <c r="E522" t="n">
-        <v>6.775499820709229</v>
+        <v>6.765999794006348</v>
       </c>
       <c r="F522" t="n">
-        <v>6.759250164031982</v>
+        <v>6.757299900054932</v>
       </c>
       <c r="G522" t="n">
         <v>6.745</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.01624965667724609</v>
+        <v>-0.008699893951416016</v>
       </c>
       <c r="I522" t="n">
         <v>99.75</v>
@@ -80804,40 +80804,40 @@
         <v>0</v>
       </c>
       <c r="K522" t="n">
-        <v>2.7963</v>
+        <v>2.768800000000001</v>
       </c>
       <c r="L522" t="n">
-        <v>2.821925</v>
+        <v>2.82055</v>
       </c>
       <c r="M522" t="n">
-        <v>2.653981666666667</v>
+        <v>2.653523333333333</v>
       </c>
       <c r="N522" t="n">
         <v/>
       </c>
       <c r="O522" t="n">
-        <v>94.2</v>
+        <v>93.60000000000001</v>
       </c>
       <c r="P522" t="n">
-        <v>79.54091816367266</v>
+        <v>78.64271457085829</v>
       </c>
       <c r="Q522" t="n">
         <v>1.472</v>
       </c>
       <c r="R522" t="n">
-        <v>-4.981439310224391</v>
+        <v>-5.169252842083079</v>
       </c>
       <c r="S522" t="n">
         <v>6.5895</v>
       </c>
       <c r="T522" t="n">
-        <v>-2.745182283685144</v>
+        <v>-2.60862842713504</v>
       </c>
       <c r="U522" t="n">
-        <v>-0.2394602390878742</v>
+        <v>-0.1167996041194552</v>
       </c>
       <c r="V522" t="n">
-        <v>0.4016064257028112</v>
+        <v>0.8032128514056225</v>
       </c>
       <c r="W522" t="inlineStr">
         <is>
@@ -80860,25 +80860,25 @@
         <v>6.349206349206349</v>
       </c>
       <c r="AC522" t="n">
-        <v>-0.434130239087871</v>
+        <v>-0.311469604119452</v>
       </c>
       <c r="AD522" t="n">
-        <v>7.113017232242221</v>
+        <v>7.115751430653356</v>
       </c>
       <c r="AE522" t="n">
-        <v>-0.3375174115329926</v>
+        <v>-0.3497516366470084</v>
       </c>
       <c r="AF522" t="n">
-        <v>6.85080956240254</v>
+        <v>6.858689007310963</v>
       </c>
       <c r="AG522" t="n">
-        <v>-0.07530974169331106</v>
+        <v>-0.09268921330461577</v>
       </c>
       <c r="AH522" t="n">
         <v>6.860464582220349</v>
       </c>
       <c r="AI522" t="n">
-        <v>-0.0849647615111202</v>
+        <v>-0.09446478821400106</v>
       </c>
       <c r="AJ522" t="n">
         <v>-0.2865252693972555</v>
@@ -80890,13 +80890,13 @@
         <v>0.2945802259112972</v>
       </c>
       <c r="AM522" t="n">
-        <v>0.4419882241595692</v>
+        <v>0.2575822725658247</v>
       </c>
       <c r="AN522" t="n">
-        <v>55.6</v>
+        <v>50.40000000000001</v>
       </c>
       <c r="AO522" t="n">
-        <v>-0.02213175137108842</v>
+        <v>-0.02208330338555479</v>
       </c>
       <c r="AP522" t="n">
         <v>6.7778000831604</v>
@@ -80920,10 +80920,10 @@
         <v>58.06451612903226</v>
       </c>
       <c r="AW522" t="n">
-        <v>69.97258064516129</v>
+        <v>68.20258064516129</v>
       </c>
       <c r="AX522" t="n">
-        <v>68.05718279569892</v>
+        <v>67.70318279569892</v>
       </c>
     </row>
   </sheetData>
@@ -81135,7 +81135,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.78</t>
+          <t>6.77</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -81150,7 +81150,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>4.07</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -81165,7 +81165,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -81175,7 +81175,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>79</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -81200,12 +81200,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -81240,22 +81240,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.43</t>
+          <t>-0.31</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.34</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -81275,7 +81275,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-18 17:24 EDT
Score: 73/100
USD/CNY: 6.76
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85802,25 +85802,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.2</v>
+        <v>4.19</v>
       </c>
       <c r="C524" t="n">
         <v>1.2437</v>
       </c>
       <c r="D524" t="n">
-        <v>2.9338</v>
+        <v>2.9463</v>
       </c>
       <c r="E524" t="n">
         <v>6.757199764251709</v>
       </c>
       <c r="F524" t="n">
-        <v>6.777140140533447</v>
+        <v>6.777100086212158</v>
       </c>
       <c r="G524" t="n">
         <v>6.7577</v>
       </c>
       <c r="H524" t="n">
-        <v>0.01994037628173828</v>
+        <v>0.01990032196044922</v>
       </c>
       <c r="I524" t="n">
         <v>100.0899963378906</v>
@@ -85829,22 +85829,22 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>2.9338</v>
+        <v>2.9463</v>
       </c>
       <c r="L524" t="n">
-        <v>2.82853</v>
+        <v>2.829155</v>
       </c>
       <c r="M524" t="n">
-        <v>2.66786</v>
+        <v>2.668068333333333</v>
       </c>
       <c r="N524" t="n">
         <v/>
       </c>
       <c r="O524" t="n">
-        <v>99.80000000000001</v>
+        <v>100</v>
       </c>
       <c r="P524" t="n">
-        <v>91.71656686626747</v>
+        <v>92.01596806387225</v>
       </c>
       <c r="Q524" t="n">
         <v>1.48</v>
@@ -85859,7 +85859,7 @@
         <v>2.5</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.907198609603871</v>
+        <v>-4.927337247290302</v>
       </c>
       <c r="V524" t="n">
         <v>6.5888</v>
@@ -85897,16 +85897,16 @@
         <v>-0.2780108065170372</v>
       </c>
       <c r="AG524" t="n">
-        <v>7.088788977131225</v>
+        <v>7.090149785109496</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3315892128795159</v>
+        <v>-0.3329500208577869</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.800848487526014</v>
+        <v>6.797114622073084</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.04364872327430547</v>
+        <v>-0.03991485782137527</v>
       </c>
       <c r="AK524" t="n">
         <v>6.809671190627447</v>
@@ -85924,10 +85924,10 @@
         <v>0.3212764901162176</v>
       </c>
       <c r="AP524" t="n">
-        <v>0.7900583668523539</v>
+        <v>0.8297740745378822</v>
       </c>
       <c r="AQ524" t="n">
-        <v>65.40000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="AR524" t="n">
         <v>-0.01886246161065713</v>
@@ -85954,10 +85954,10 @@
         <v>73.52941176470588</v>
       </c>
       <c r="AZ524" t="n">
-        <v>80.28529411764706</v>
+        <v>80.47529411764705</v>
       </c>
       <c r="BA524" t="n">
-        <v>72.83628707377379</v>
+        <v>72.87428707377379</v>
       </c>
     </row>
   </sheetData>
@@ -86184,7 +86184,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.20</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86199,7 +86199,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.93</t>
+          <t>2.95</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-20 12:12 EDT
Score: 76/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85493,10 +85493,10 @@
         <v>0.02060031890869141</v>
       </c>
       <c r="I522" t="n">
-        <v>100.8499984741211</v>
+        <v>100.0899963378906</v>
       </c>
       <c r="J522" t="n">
-        <v>0.007593187771381293</v>
+        <v>0</v>
       </c>
       <c r="K522" t="n">
         <v>2.9463</v>
@@ -85573,10 +85573,10 @@
         <v>-0.3329500208577869</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.789283666813434</v>
+        <v>6.797114622073084</v>
       </c>
       <c r="AJ522" t="n">
-        <v>-0.032083902561725</v>
+        <v>-0.03991485782137527</v>
       </c>
       <c r="AK522" t="n">
         <v>6.809671190627447</v>
@@ -85594,25 +85594,25 @@
         <v>0.3212764901162176</v>
       </c>
       <c r="AP522" t="n">
-        <v>0.9130165331270262</v>
+        <v>0.8297740745378823</v>
       </c>
       <c r="AQ522" t="n">
-        <v>68.40000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.01800843067043562</v>
+        <v>-0.0188624616106571</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.77687327731828</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.01917327731828067</v>
+        <v>-0.02010008316040057</v>
       </c>
       <c r="AU522" t="n">
         <v>-0.02010008316040057</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.03630913890309846</v>
+        <v>-0.03635547919520445</v>
       </c>
       <c r="AW522" t="n">
         <v/>
@@ -85624,10 +85624,10 @@
         <v>73.52941176470588</v>
       </c>
       <c r="AZ522" t="n">
-        <v>81.25529411764705</v>
+        <v>80.47529411764705</v>
       </c>
       <c r="BA522" t="n">
-        <v>73.03028707377379</v>
+        <v>72.87428707377379</v>
       </c>
     </row>
     <row r="523">
@@ -85646,7 +85646,7 @@
         <v>2.9463</v>
       </c>
       <c r="E523" t="n">
-        <v>6.768099784851074</v>
+        <v>6.768599987030029</v>
       </c>
       <c r="F523" t="n">
         <v>6.7778000831604</v>
@@ -85655,13 +85655,13 @@
         <v>6.7647</v>
       </c>
       <c r="H523" t="n">
-        <v>0.009700298309326172</v>
+        <v>0.009200096130371094</v>
       </c>
       <c r="I523" t="n">
         <v>100.8489990234375</v>
       </c>
       <c r="J523" t="n">
-        <v>-9.910269694768381e-06</v>
+        <v>0.007583202251147947</v>
       </c>
       <c r="K523" t="n">
         <v>2.9463</v>
@@ -85694,19 +85694,19 @@
         <v>2.5</v>
       </c>
       <c r="U523" t="n">
-        <v>-4.787436242365851</v>
+        <v>-4.77969240995797</v>
       </c>
       <c r="V523" t="n">
         <v>6.5888</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.649189440918087</v>
+        <v>-2.656383703787513</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2546271806666223</v>
+        <v>-0.2621077751982392</v>
       </c>
       <c r="Y523" t="n">
-        <v>2.811244979919679</v>
+        <v>2.008032128514056</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,55 +85729,55 @@
         <v>4.166666666666666</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4422071806666317</v>
+        <v>-0.4496877751982487</v>
       </c>
       <c r="AG523" t="n">
         <v>7.09211824687052</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3240184620194455</v>
+        <v>-0.3235182598404904</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.789261345933951</v>
+        <v>6.789228834098362</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.02116156108287726</v>
+        <v>-0.02062884706833223</v>
       </c>
       <c r="AK523" t="n">
         <v>6.802840448144932</v>
       </c>
       <c r="AL523" t="n">
-        <v>-0.03474066329385739</v>
+        <v>-0.03424046111490231</v>
       </c>
       <c r="AM523" t="n">
-        <v>-0.3027504956929284</v>
+        <v>-0.3031231825467917</v>
       </c>
       <c r="AN523" t="n">
-        <v>-0.008812786025409525</v>
+        <v>-0.00871021199524602</v>
       </c>
       <c r="AO523" t="n">
-        <v>0.3322271170679635</v>
+        <v>0.3321305540852062</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.029607407155507</v>
+        <v>1.035900222957083</v>
       </c>
       <c r="AQ523" t="n">
         <v>70.40000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.01804805112348658</v>
+        <v>-0.01413372847627263</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.777801295444869</v>
+        <v>6.777073645856678</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.01310129544486838</v>
+        <v>-0.01237364585667766</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.01310008316040001</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.03469781788882886</v>
+        <v>-0.03470777570152532</v>
       </c>
       <c r="AW523" t="n">
         <v/>
@@ -85786,13 +85786,13 @@
         <v/>
       </c>
       <c r="AY523" t="n">
-        <v>82.85714285714286</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="AZ523" t="n">
-        <v>85.05</v>
+        <v>86.05</v>
       </c>
       <c r="BA523" t="n">
-        <v>75.46562040710712</v>
+        <v>75.50962040710712</v>
       </c>
     </row>
   </sheetData>
@@ -86069,12 +86069,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.26</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86109,7 +86109,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.44</t>
+          <t>-0.45</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86134,7 +86134,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>-0.0088</t>
+          <t>-0.0087</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -86144,17 +86144,17 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>-0.018</t>
+          <t>-0.014</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.7778</t>
+          <t>6.7771</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -86179,7 +86179,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>76</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-21 12:30 EDT
Score: 75/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85367,16 +85367,16 @@
         <v>-4.927337247290302</v>
       </c>
       <c r="V521" t="n">
-        <v>6.5888</v>
+        <v>6.5986</v>
       </c>
       <c r="W521" t="n">
-        <v>-2.492153112634188</v>
+        <v>-2.347122621574171</v>
       </c>
       <c r="X521" t="n">
-        <v>-0.09134080651702625</v>
+        <v>0.05946189808718749</v>
       </c>
       <c r="Y521" t="n">
-        <v>6.42570281124498</v>
+        <v>6.827309236947791</v>
       </c>
       <c r="Z521" t="inlineStr">
         <is>
@@ -85399,7 +85399,7 @@
         <v>3.968253968253968</v>
       </c>
       <c r="AF521" t="n">
-        <v>-0.2789208065170357</v>
+        <v>-0.1281181019128219</v>
       </c>
       <c r="AG521" t="n">
         <v>7.090149785109496</v>
@@ -85532,16 +85532,16 @@
         <v>-4.77969240995797</v>
       </c>
       <c r="V522" t="n">
-        <v>6.5888</v>
+        <v>6.5986</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.656383703787513</v>
+        <v>-2.511597484794237</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.2621077751982392</v>
+        <v>-0.1115590646890263</v>
       </c>
       <c r="Y522" t="n">
-        <v>2.008032128514056</v>
+        <v>6.024096385542169</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,7 +85564,7 @@
         <v>4.166666666666666</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.4496877751982487</v>
+        <v>-0.2991390646890357</v>
       </c>
       <c r="AG522" t="n">
         <v>7.09211824687052</v>
@@ -85899,17 +85899,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.59</t>
+          <t>6.60</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.11</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85944,7 +85944,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-22 17:33 EDT
Score: 79/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85472,25 +85472,25 @@
         </is>
       </c>
       <c r="B522" t="n">
-        <v>4.19</v>
+        <v>4.24</v>
       </c>
       <c r="C522" t="n">
         <v>1.2462</v>
       </c>
       <c r="D522" t="n">
-        <v>2.9463</v>
+        <v>2.9938</v>
       </c>
       <c r="E522" t="n">
         <v>6.768599987030029</v>
       </c>
       <c r="F522" t="n">
-        <v>6.777339935302734</v>
+        <v>6.77685022354126</v>
       </c>
       <c r="G522" t="n">
         <v>6.762899999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>0.008739948272705078</v>
+        <v>0.008250236511230469</v>
       </c>
       <c r="I522" t="n">
         <v>100.8499984741211</v>
@@ -85499,22 +85499,22 @@
         <v>0</v>
       </c>
       <c r="K522" t="n">
-        <v>2.9463</v>
+        <v>2.9938</v>
       </c>
       <c r="L522" t="n">
-        <v>2.837015</v>
+        <v>2.83939</v>
       </c>
       <c r="M522" t="n">
-        <v>2.680671666666667</v>
+        <v>2.681463333333333</v>
       </c>
       <c r="N522" t="n">
         <v/>
       </c>
       <c r="O522" t="n">
-        <v>99.60000000000001</v>
+        <v>100</v>
       </c>
       <c r="P522" t="n">
-        <v>91.81636726546907</v>
+        <v>93.01397205588822</v>
       </c>
       <c r="Q522" t="n">
         <v>1.48</v>
@@ -85529,7 +85529,7 @@
         <v>2.52</v>
       </c>
       <c r="U522" t="n">
-        <v>-4.987577336020991</v>
+        <v>-4.886884321781088</v>
       </c>
       <c r="V522" t="n">
         <v>6.6001</v>
@@ -85567,16 +85567,16 @@
         <v>-0.2565937819789088</v>
       </c>
       <c r="AG522" t="n">
-        <v>7.106189145949059</v>
+        <v>7.099373638600277</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.3375891589190294</v>
+        <v>-0.3307736515702473</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.789777073311202</v>
+        <v>6.775203601329934</v>
       </c>
       <c r="AJ522" t="n">
-        <v>-0.02117708628117221</v>
+        <v>-0.006603614299904415</v>
       </c>
       <c r="AK522" t="n">
         <v>6.800260207803535</v>
@@ -85594,10 +85594,10 @@
         <v>0.3427146952658529</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.027988339780894</v>
+        <v>1.182405408260665</v>
       </c>
       <c r="AQ522" t="n">
-        <v>69</v>
+        <v>73.2</v>
       </c>
       <c r="AR522" t="n">
         <v>-0.01848658309162282</v>
@@ -85624,10 +85624,10 @@
         <v>77.77777777777779</v>
       </c>
       <c r="AZ522" t="n">
-        <v>82.78222222222223</v>
+        <v>84.18222222222222</v>
       </c>
       <c r="BA522" t="n">
-        <v>78.41754872251931</v>
+        <v>78.69754872251931</v>
       </c>
     </row>
   </sheetData>
@@ -85854,7 +85854,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.19</t>
+          <t>4.24</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -85869,7 +85869,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -85879,7 +85879,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -85949,12 +85949,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.34</t>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -85979,7 +85979,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86014,7 +86014,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-23 16:16 EDT
Score: 84/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.768599987030029</v>
       </c>
       <c r="F523" t="n">
-        <v>6.797200202941895</v>
+        <v>6.794929981231689</v>
       </c>
       <c r="G523" t="n">
         <v>6.778300000000001</v>
       </c>
       <c r="H523" t="n">
-        <v>0.02860021591186523</v>
+        <v>0.02632999420166016</v>
       </c>
       <c r="I523" t="n">
         <v>101.0199966430664</v>
@@ -86009,7 +86009,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.80</t>
+          <t>6.79</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-23 17:02 EDT
Score: 83/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85520,13 +85520,13 @@
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="S522" t="n">
-        <v>2.52</v>
+        <v>2.56</v>
       </c>
       <c r="T522" t="n">
-        <v>2.52</v>
+        <v>2.56</v>
       </c>
       <c r="U522" t="n">
         <v>-4.886884321781088</v>
@@ -85538,10 +85538,10 @@
         <v>-2.511597484794237</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.09206138418600407</v>
+        <v>-0.05306602317991516</v>
       </c>
       <c r="Y522" t="n">
-        <v>6.626506024096385</v>
+        <v>7.228915662650603</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,7 +85564,7 @@
         <v>5.952380952380952</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.2819113841860066</v>
+        <v>-0.2429160231799177</v>
       </c>
       <c r="AG522" t="n">
         <v>7.099373638600277</v>
@@ -85637,25 +85637,25 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>4.24</v>
+        <v>4.16</v>
       </c>
       <c r="C523" t="n">
         <v>1.2637</v>
       </c>
       <c r="D523" t="n">
-        <v>2.9938</v>
+        <v>2.8963</v>
       </c>
       <c r="E523" t="n">
-        <v>6.768599987030029</v>
+        <v>6.774499893188477</v>
       </c>
       <c r="F523" t="n">
-        <v>6.794929981231689</v>
+        <v>6.793159961700439</v>
       </c>
       <c r="G523" t="n">
         <v>6.778300000000001</v>
       </c>
       <c r="H523" t="n">
-        <v>0.02632999420166016</v>
+        <v>0.01866006851196289</v>
       </c>
       <c r="I523" t="n">
         <v>101.0199966430664</v>
@@ -85664,49 +85664,49 @@
         <v>0</v>
       </c>
       <c r="K523" t="n">
-        <v>2.9938</v>
+        <v>2.8963</v>
       </c>
       <c r="L523" t="n">
-        <v>2.851145</v>
+        <v>2.84627</v>
       </c>
       <c r="M523" t="n">
-        <v>2.689436666666666</v>
+        <v>2.687811666666667</v>
       </c>
       <c r="N523" t="n">
         <v/>
       </c>
       <c r="O523" t="n">
-        <v>99.80000000000001</v>
+        <v>98</v>
       </c>
       <c r="P523" t="n">
-        <v>92.91417165668663</v>
+        <v>87.82435129740519</v>
       </c>
       <c r="Q523" t="n">
         <v>1.482</v>
       </c>
       <c r="R523" t="n">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="S523" t="n">
-        <v>2.518</v>
+        <v>2.558</v>
       </c>
       <c r="T523" t="n">
-        <v>2.518</v>
+        <v>2.558</v>
       </c>
       <c r="U523" t="n">
-        <v>-4.939089016379318</v>
+        <v>-5.008815874384545</v>
       </c>
       <c r="V523" t="n">
         <v>6.612</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.313624491476907</v>
+        <v>-2.398699472294097</v>
       </c>
       <c r="X523" t="n">
-        <v>0.1118305288640098</v>
+        <v>0.0623930690252239</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.835341365461847</v>
+        <v>8.032128514056225</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,25 +85729,25 @@
         <v>4.761904761904762</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.07601947113597962</v>
+        <v>-0.1254569309747655</v>
       </c>
       <c r="AG523" t="n">
-        <v>7.102907165552081</v>
+        <v>7.113822119248665</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3343071785220522</v>
+        <v>-0.3393222260601885</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.774183190518288</v>
+        <v>6.804618466352278</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.005583203488258803</v>
+        <v>-0.03011857316380162</v>
       </c>
       <c r="AK523" t="n">
         <v>6.781970485204615</v>
       </c>
       <c r="AL523" t="n">
-        <v>-0.01337049817458524</v>
+        <v>-0.007470592016137978</v>
       </c>
       <c r="AM523" t="n">
         <v>-0.3121566752204096</v>
@@ -85759,13 +85759,13 @@
         <v>0.3560731605465752</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.190252106428963</v>
+        <v>0.9304925970779739</v>
       </c>
       <c r="AQ523" t="n">
-        <v>73.2</v>
+        <v>67.2</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.01835732393593754</v>
+        <v>-0.01840023488955626</v>
       </c>
       <c r="AS523" t="n">
         <v>6.7778000831604</v>
@@ -85789,10 +85789,10 @@
         <v>100</v>
       </c>
       <c r="AZ523" t="n">
-        <v>91.89</v>
+        <v>89.45999999999999</v>
       </c>
       <c r="BA523" t="n">
-        <v>83.83004872251931</v>
+        <v>83.3440487225193</v>
       </c>
     </row>
   </sheetData>
@@ -86019,7 +86019,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.24</t>
+          <t>4.16</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86034,17 +86034,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.99</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>98</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>88</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86054,12 +86054,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.00</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.52</t>
+          <t>2.56</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86069,12 +86069,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.11</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86109,24 +86109,24 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.13</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.33</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>-0.01</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
-      </c>
       <c r="AA2" t="inlineStr">
         <is>
           <t>-0.312</t>
@@ -86144,7 +86144,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86179,7 +86179,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>83</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-24 12:08 EDT
Score: 86/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85649,19 +85649,19 @@
         <v>6.774499893188477</v>
       </c>
       <c r="F523" t="n">
-        <v>6.793159961700439</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="G523" t="n">
         <v>6.778300000000001</v>
       </c>
       <c r="H523" t="n">
-        <v>0.01866006851196289</v>
+        <v>0.003300189971923828</v>
       </c>
       <c r="I523" t="n">
-        <v>101.0199966430664</v>
+        <v>101.4100036621094</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>0.003860691269085947</v>
       </c>
       <c r="K523" t="n">
         <v>2.8963</v>
@@ -85697,16 +85697,16 @@
         <v>-5.008815874384545</v>
       </c>
       <c r="V523" t="n">
-        <v>6.612</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.398699472294097</v>
+        <v>-2.596500051101003</v>
       </c>
       <c r="X523" t="n">
-        <v>0.0623930690252239</v>
+        <v>-0.1433986531654829</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.032128514056225</v>
+        <v>5.220883534136546</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85714,22 +85714,22 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.66985</v>
+        <v>1.70273</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.63606</v>
+        <v>1.68515</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.54212</v>
+        <v>1.65788</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.1878500000000001</v>
+        <v>0.2207300000000001</v>
       </c>
       <c r="AE523" t="n">
-        <v>4.761904761904762</v>
+        <v>18.25396825396825</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.1254569309747655</v>
+        <v>-0.3641286531654853</v>
       </c>
       <c r="AG523" t="n">
         <v>7.113822119248665</v>
@@ -85738,10 +85738,10 @@
         <v>-0.3393222260601885</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.804618466352278</v>
+        <v>6.802628307046305</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.03011857316380162</v>
+        <v>-0.0281284138578286</v>
       </c>
       <c r="AK523" t="n">
         <v>6.781970485204615</v>
@@ -85759,25 +85759,25 @@
         <v>0.3560731605465752</v>
       </c>
       <c r="AP523" t="n">
-        <v>0.9304925970779739</v>
+        <v>0.9515940158218971</v>
       </c>
       <c r="AQ523" t="n">
         <v>67.2</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.01840023488955626</v>
+        <v>-0.0170334136218979</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7778000831604</v>
+        <v>6.77735436993509</v>
       </c>
       <c r="AT523" t="n">
-        <v>0.0004999168396002673</v>
+        <v>0.0009456300649102189</v>
       </c>
       <c r="AU523" t="n">
         <v>0.0004999168396002673</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.0296790995789523</v>
+        <v>-0.0296568139176868</v>
       </c>
       <c r="AW523" t="n">
         <v/>
@@ -85793,6 +85793,171 @@
       </c>
       <c r="BA523" t="n">
         <v>83.3440487225193</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2562</v>
+      </c>
+      <c r="D524" t="n">
+        <v>2.8963</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.774499893188477</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.81443977355957</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.7989</v>
+      </c>
+      <c r="H524" t="n">
+        <v>0.03993988037109375</v>
+      </c>
+      <c r="I524" t="n">
+        <v>101.4100036621094</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>2.8963</v>
+      </c>
+      <c r="L524" t="n">
+        <v>2.852975</v>
+      </c>
+      <c r="M524" t="n">
+        <v>2.694</v>
+      </c>
+      <c r="N524" t="n">
+        <v/>
+      </c>
+      <c r="O524" t="n">
+        <v>97.80000000000001</v>
+      </c>
+      <c r="P524" t="n">
+        <v>87.72455089820359</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.484</v>
+      </c>
+      <c r="R524" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.556</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.556</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-5.039083284728484</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.6285</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-2.155139058091571</v>
+      </c>
+      <c r="X524" t="n">
+        <v>0.3137933239615309</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>10.8433734939759</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.70273</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.68515</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.65788</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.2187300000000001</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>18.25396825396825</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>0.09506332396151951</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>7.115872584930086</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.3413726917416096</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.803087339410362</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>-0.02858744622188514</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.809638458820509</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>-0.03513856563203266</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.3181413841564625</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>-0.003317316385138602</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.3690689225934927</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>0.9458453748694567</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>-0.01728680009510248</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.7778000831604</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>0.02109991683959933</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>0.02109991683959933</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.02549515336567576</v>
+      </c>
+      <c r="AW524" t="n">
+        <v/>
+      </c>
+      <c r="AX524" t="n">
+        <v/>
+      </c>
+      <c r="AY524" t="n">
+        <v>100</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>89.27000000000001</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>85.87950326797386</v>
       </c>
     </row>
   </sheetData>
@@ -85999,7 +86164,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86009,12 +86174,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.79</t>
+          <t>6.81</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.78</t>
+          <t>6.80</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -86029,7 +86194,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>101.02</t>
+          <t>101.41</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86064,17 +86229,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.61</t>
+          <t>6.63</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86084,32 +86249,32 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>0.19</t>
+          <t>0.22</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>18</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86124,32 +86289,32 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.01</t>
+          <t>-0.04</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.312</t>
+          <t>-0.318</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>-0.0051</t>
+          <t>-0.0033</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.356</t>
+          <t>0.369</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>-0.018</t>
+          <t>-0.017</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -86159,12 +86324,12 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
@@ -86179,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>86</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-06-24 16:51 EDT
Score: 86/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.482</v>
       </c>
       <c r="R523" t="n">
-        <v>4.04</v>
+        <v>4.01</v>
       </c>
       <c r="S523" t="n">
-        <v>2.558</v>
+        <v>2.528</v>
       </c>
       <c r="T523" t="n">
-        <v>2.558</v>
+        <v>2.528</v>
       </c>
       <c r="U523" t="n">
         <v>-5.008815874384545</v>
@@ -85703,10 +85703,10 @@
         <v>-2.596500051101003</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.1433986531654829</v>
+        <v>-0.1726197031501453</v>
       </c>
       <c r="Y523" t="n">
-        <v>5.220883534136546</v>
+        <v>4.016064257028113</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>18.25396825396825</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.3641286531654853</v>
+        <v>-0.3933497031501476</v>
       </c>
       <c r="AG523" t="n">
         <v>7.113822119248665</v>
@@ -85811,16 +85811,16 @@
         <v>2.8963</v>
       </c>
       <c r="E524" t="n">
-        <v>6.774499893188477</v>
+        <v>6.789999961853027</v>
       </c>
       <c r="F524" t="n">
-        <v>6.814010143280029</v>
+        <v>6.812910079956055</v>
       </c>
       <c r="G524" t="n">
         <v>6.7989</v>
       </c>
       <c r="H524" t="n">
-        <v>0.03951025009155273</v>
+        <v>0.02291011810302734</v>
       </c>
       <c r="I524" t="n">
         <v>101.4100036621094</v>
@@ -85850,28 +85850,28 @@
         <v>1.484</v>
       </c>
       <c r="R524" t="n">
-        <v>4.04</v>
+        <v>4.01</v>
       </c>
       <c r="S524" t="n">
-        <v>2.556</v>
+        <v>2.526</v>
       </c>
       <c r="T524" t="n">
-        <v>2.556</v>
+        <v>2.526</v>
       </c>
       <c r="U524" t="n">
-        <v>-5.039083284728484</v>
+        <v>-4.799302281411595</v>
       </c>
       <c r="V524" t="n">
         <v>6.6285</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.155139058091571</v>
+        <v>-2.378497242420508</v>
       </c>
       <c r="X524" t="n">
-        <v>0.3137933239615309</v>
+        <v>0.05212501815843318</v>
       </c>
       <c r="Y524" t="n">
-        <v>10.8433734939759</v>
+        <v>8.032128514056225</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>18.25396825396825</v>
       </c>
       <c r="AF524" t="n">
-        <v>0.09506332396151951</v>
+        <v>-0.1666049818415782</v>
       </c>
       <c r="AG524" t="n">
         <v>7.115872584930086</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3413726917416096</v>
+        <v>-0.3258726230770588</v>
       </c>
       <c r="AI524" t="n">
         <v>6.803087339410362</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.02858744622188514</v>
+        <v>-0.01308737755733436</v>
       </c>
       <c r="AK524" t="n">
         <v>6.809638458820509</v>
       </c>
       <c r="AL524" t="n">
-        <v>-0.03513856563203266</v>
+        <v>-0.01963849696748188</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3181413841564625</v>
@@ -85924,13 +85924,13 @@
         <v>0.3690689225934927</v>
       </c>
       <c r="AP524" t="n">
-        <v>0.9458453748694567</v>
+        <v>1.109947206004787</v>
       </c>
       <c r="AQ524" t="n">
-        <v>66.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.01728680009510248</v>
+        <v>-0.01740141359052104</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85954,10 +85954,10 @@
         <v>100</v>
       </c>
       <c r="AZ524" t="n">
-        <v>89.27000000000001</v>
+        <v>90.95</v>
       </c>
       <c r="BA524" t="n">
-        <v>85.87950326797386</v>
+        <v>86.21550326797386</v>
       </c>
     </row>
   </sheetData>
@@ -86169,7 +86169,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.77</t>
+          <t>6.79</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>4.01</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.56</t>
+          <t>2.53</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,22 +86274,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.34</t>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.03</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-0.04</t>
+          <t>-0.02</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-26 12:57 EDT
Score: 88/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.789999961853027</v>
       </c>
       <c r="F524" t="n">
-        <v>6.801270008087158</v>
+        <v>6.801459789276123</v>
       </c>
       <c r="G524" t="n">
         <v>6.7878</v>
       </c>
       <c r="H524" t="n">
-        <v>0.01127004623413086</v>
+        <v>0.0114598274230957</v>
       </c>
       <c r="I524" t="n">
         <v>101.4300003051758</v>

</xml_diff>

<commit_message>
auto: data update 2026-06-26 16:01 EDT
Score: 88/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.789999961853027</v>
       </c>
       <c r="F524" t="n">
-        <v>6.801459789276123</v>
+        <v>6.801740169525146</v>
       </c>
       <c r="G524" t="n">
         <v>6.7878</v>
       </c>
       <c r="H524" t="n">
-        <v>0.0114598274230957</v>
+        <v>0.01174020767211914</v>
       </c>
       <c r="I524" t="n">
         <v>101.4300003051758</v>

</xml_diff>

<commit_message>
auto: data update 2026-06-27 12:00 EDT
Score: 73/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85658,10 +85658,10 @@
         <v>0.01450003814697265</v>
       </c>
       <c r="I523" t="n">
-        <v>101.4300003051758</v>
+        <v>101.3600006103516</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>-0.0006901281141044047</v>
       </c>
       <c r="K523" t="n">
         <v>2.8238</v>
@@ -85738,10 +85738,10 @@
         <v>-0.3364383256526304</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.826408025492162</v>
+        <v>6.826413262727742</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.03640806363913462</v>
+        <v>-0.03641330087471495</v>
       </c>
       <c r="AK523" t="n">
         <v>6.822087900644207</v>
@@ -85759,40 +85759,40 @@
         <v>0.3960788710418811</v>
       </c>
       <c r="AP523" t="n">
-        <v>0.8639251684625331</v>
+        <v>0.8638695859060854</v>
       </c>
       <c r="AQ523" t="n">
         <v>66.60000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.01603797197385831</v>
+        <v>-0.01608028461035975</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.8015</v>
+        <v>6.801575479350333</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.01370000000000005</v>
+        <v>-0.01377547935033352</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.01370000000000005</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01289635640003279</v>
+        <v>-0.01290013036754947</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01347598678887955</v>
+        <v>-0.01347724477805177</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01353511290781563</v>
+        <v>0.01353530160619146</v>
       </c>
       <c r="AY523" t="n">
-        <v>49.2063492063492</v>
+        <v>48.80952380952381</v>
       </c>
       <c r="AZ523" t="n">
-        <v>70.10222222222221</v>
+        <v>69.96333333333332</v>
       </c>
       <c r="BA523" t="n">
-        <v>72.97088888888888</v>
+        <v>72.94311111111111</v>
       </c>
     </row>
   </sheetData>
@@ -86029,7 +86029,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>101.43</t>
+          <t>101.36</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86154,7 +86154,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.8015</t>
+          <t>6.8016</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-06-29 16:09 EDT
Score: 88/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.789999961853027</v>
       </c>
       <c r="F522" t="n">
-        <v>6.798580169677734</v>
+        <v>6.799769878387451</v>
       </c>
       <c r="G522" t="n">
         <v>6.7855</v>
       </c>
       <c r="H522" t="n">
-        <v>0.008580207824707031</v>
+        <v>0.009769916534423828</v>
       </c>
       <c r="I522" t="n">
         <v>101.3600006103516</v>

</xml_diff>

<commit_message>
auto: data update 2026-06-30 16:08 EDT
Score: 67/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.797999858856201</v>
       </c>
       <c r="F523" t="n">
-        <v>6.7922</v>
+        <v>6.791</v>
       </c>
       <c r="G523" t="n">
         <v>6.7749</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.005799858856200935</v>
+        <v>-0.006999858856200802</v>
       </c>
       <c r="I523" t="n">
         <v>101.1100006103516</v>

</xml_diff>

<commit_message>
auto: data update 2026-07-01 13:11 EDT
Score: 65/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.793600082397461</v>
       </c>
       <c r="F524" t="n">
-        <v>6.794</v>
+        <v>6.795</v>
       </c>
       <c r="G524" t="n">
         <v>6.7784</v>
       </c>
       <c r="H524" t="n">
-        <v>0.0003999176025386575</v>
+        <v>0.001399917602538991</v>
       </c>
       <c r="I524" t="n">
         <v>101.1900024414062</v>
@@ -85862,16 +85862,16 @@
         <v>-4.704522407705351</v>
       </c>
       <c r="V524" t="n">
-        <v>6.6126</v>
+        <v>6.5986</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.664273436795916</v>
+        <v>-2.870349741409051</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2800450922366915</v>
+        <v>-0.4943026261429839</v>
       </c>
       <c r="Y524" t="n">
-        <v>3.614457831325301</v>
+        <v>1.004016064257028</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,7 +85894,7 @@
         <v>61.7063492063492</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.5536850922366998</v>
+        <v>-0.7679426261429922</v>
       </c>
       <c r="AG524" t="n">
         <v>7.113206520563739</v>
@@ -86229,17 +86229,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.61</t>
+          <t>6.60</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.55</t>
+          <t>-0.77</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-01 16:05 EDT
Score: 65/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.793600082397461</v>
       </c>
       <c r="F524" t="n">
-        <v>6.795</v>
+        <v>6.7953</v>
       </c>
       <c r="G524" t="n">
         <v>6.7784</v>
       </c>
       <c r="H524" t="n">
-        <v>0.001399917602538991</v>
+        <v>0.00169991760253918</v>
       </c>
       <c r="I524" t="n">
         <v>101.1900024414062</v>
@@ -85862,16 +85862,16 @@
         <v>-4.704522407705351</v>
       </c>
       <c r="V524" t="n">
-        <v>6.5986</v>
+        <v>6.6126</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.870349741409051</v>
+        <v>-2.664273436795916</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.4943026261429839</v>
+        <v>-0.2800450922366915</v>
       </c>
       <c r="Y524" t="n">
-        <v>1.004016064257028</v>
+        <v>3.614457831325301</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,7 +85894,7 @@
         <v>61.7063492063492</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.7679426261429922</v>
+        <v>-0.5536850922366998</v>
       </c>
       <c r="AG524" t="n">
         <v>7.113206520563739</v>
@@ -86174,7 +86174,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.79</t>
+          <t>6.80</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -86229,17 +86229,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.60</t>
+          <t>6.61</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.49</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.77</t>
+          <t>-0.55</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-01 16:49 EDT
Score: 65/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>3.97</v>
+        <v>3.98</v>
       </c>
       <c r="S523" t="n">
-        <v>2.49</v>
+        <v>2.5</v>
       </c>
       <c r="T523" t="n">
-        <v>2.49</v>
+        <v>2.5</v>
       </c>
       <c r="U523" t="n">
         <v>-4.808351947122741</v>
@@ -85703,7 +85703,7 @@
         <v>-2.870349741409051</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.4943026261429839</v>
+        <v>-0.4845896611171074</v>
       </c>
       <c r="Y523" t="n">
         <v>0.8032128514056225</v>
@@ -85729,7 +85729,7 @@
         <v>61.9047619047619</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.7679426261429922</v>
+        <v>-0.7582296611171158</v>
       </c>
       <c r="AG523" t="n">
         <v>7.120260284239151</v>
@@ -85814,13 +85814,13 @@
         <v>6.793600082397461</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7953</v>
+        <v>6.7948</v>
       </c>
       <c r="G524" t="n">
         <v>6.7784</v>
       </c>
       <c r="H524" t="n">
-        <v>0.00169991760253918</v>
+        <v>0.001199917602539458</v>
       </c>
       <c r="I524" t="n">
         <v>101.1900024414062</v>
@@ -85850,13 +85850,13 @@
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>3.97</v>
+        <v>3.98</v>
       </c>
       <c r="S524" t="n">
-        <v>2.49</v>
+        <v>2.5</v>
       </c>
       <c r="T524" t="n">
-        <v>2.49</v>
+        <v>2.5</v>
       </c>
       <c r="U524" t="n">
         <v>-4.704522407705351</v>
@@ -85868,10 +85868,10 @@
         <v>-2.664273436795916</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2800450922366915</v>
+        <v>-0.2703115195803907</v>
       </c>
       <c r="Y524" t="n">
-        <v>3.614457831325301</v>
+        <v>4.016064257028113</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,7 +85894,7 @@
         <v>61.7063492063492</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.5536850922366998</v>
+        <v>-0.543951519580399</v>
       </c>
       <c r="AG524" t="n">
         <v>7.113206520563739</v>
@@ -86174,7 +86174,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.80</t>
+          <t>6.79</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.97</t>
+          <t>3.98</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.49</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,7 +86234,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.55</t>
+          <t>-0.54</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-02 15:43 EDT
Score: 87/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.793600082397461</v>
       </c>
       <c r="F524" t="n">
-        <v>6.787280082702637</v>
+        <v>6.788370132446289</v>
       </c>
       <c r="G524" t="n">
         <v>6.7735</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.006319999694824219</v>
+        <v>-0.005229949951171875</v>
       </c>
       <c r="I524" t="n">
         <v>101.3899993896484</v>

</xml_diff>

<commit_message>
auto: data update 2026-07-02 16:22 EDT
Score: 86/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>3.98</v>
+        <v>4</v>
       </c>
       <c r="S523" t="n">
-        <v>2.5</v>
+        <v>2.52</v>
       </c>
       <c r="T523" t="n">
-        <v>2.5</v>
+        <v>2.52</v>
       </c>
       <c r="U523" t="n">
         <v>-4.644223216706636</v>
@@ -85703,10 +85703,10 @@
         <v>-2.870349741409051</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.4845896611171074</v>
+        <v>-0.4651637310653989</v>
       </c>
       <c r="Y523" t="n">
-        <v>1.004016064257028</v>
+        <v>1.606425702811245</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>61.7063492063492</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.7582296611171158</v>
+        <v>-0.7388037310654072</v>
       </c>
       <c r="AG523" t="n">
         <v>7.109110034674365</v>
@@ -85802,25 +85802,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.17</v>
+        <v>4.14</v>
       </c>
       <c r="C524" t="n">
         <v>1.2471</v>
       </c>
       <c r="D524" t="n">
-        <v>2.913</v>
+        <v>2.8929</v>
       </c>
       <c r="E524" t="n">
-        <v>6.793600082397461</v>
+        <v>6.79419994354248</v>
       </c>
       <c r="F524" t="n">
-        <v>6.788370132446289</v>
+        <v>6.787069797515869</v>
       </c>
       <c r="G524" t="n">
         <v>6.7735</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.005229949951171875</v>
+        <v>-0.007130146026611328</v>
       </c>
       <c r="I524" t="n">
         <v>101.3899993896484</v>
@@ -85829,46 +85829,46 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>2.913</v>
+        <v>2.8929</v>
       </c>
       <c r="L524" t="n">
-        <v>2.87207</v>
+        <v>2.871065</v>
       </c>
       <c r="M524" t="n">
-        <v>2.730643333333333</v>
+        <v>2.730308333333333</v>
       </c>
       <c r="N524" t="n">
         <v/>
       </c>
       <c r="O524" t="n">
-        <v>97.80000000000001</v>
+        <v>96.80000000000001</v>
       </c>
       <c r="P524" t="n">
-        <v>89.12175648702595</v>
+        <v>87.42514970059881</v>
       </c>
       <c r="Q524" t="n">
         <v>1.479</v>
       </c>
       <c r="R524" t="n">
-        <v>3.98</v>
+        <v>4</v>
       </c>
       <c r="S524" t="n">
-        <v>2.501</v>
+        <v>2.521</v>
       </c>
       <c r="T524" t="n">
-        <v>2.501</v>
+        <v>2.521</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.750962877716808</v>
+        <v>-4.802069764597548</v>
       </c>
       <c r="V524" t="n">
         <v>6.6074</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.74081606422365</v>
+        <v>-2.749403095209524</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.3489005435797443</v>
+        <v>-0.3383792190179147</v>
       </c>
       <c r="Y524" t="n">
         <v>2.811244979919679</v>
@@ -85894,25 +85894,25 @@
         <v>63.09523809523809</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.623540543579737</v>
+        <v>-0.6130192190179073</v>
       </c>
       <c r="AG524" t="n">
-        <v>7.116361500372703</v>
+        <v>7.120462164777638</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3227614179752418</v>
+        <v>-0.3262622212351571</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.796014117276787</v>
+        <v>6.803054954182924</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.00241403487932601</v>
+        <v>-0.008855010640443695</v>
       </c>
       <c r="AK524" t="n">
         <v>6.78726841810145</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.006331664296010509</v>
+        <v>0.00693152544103004</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3502903933401412</v>
@@ -85924,13 +85924,13 @@
         <v>0.4450018361960529</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.221585213247868</v>
+        <v>1.153579065576432</v>
       </c>
       <c r="AQ524" t="n">
-        <v>76</v>
+        <v>73.8</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.01719824269810831</v>
+        <v>-0.01720141545016146</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85954,10 +85954,10 @@
         <v>79.54545454545455</v>
       </c>
       <c r="AZ524" t="n">
-        <v>84.87090909090909</v>
+        <v>83.86090909090909</v>
       </c>
       <c r="BA524" t="n">
-        <v>86.65036654119183</v>
+        <v>86.44836654119183</v>
       </c>
     </row>
   </sheetData>
@@ -86184,7 +86184,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86199,17 +86199,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>2.89</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>97</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>87</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.98</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.52</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,7 +86234,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.35</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86274,64 +86274,64 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.62</t>
+          <t>-0.61</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.32</t>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>-0.350</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>0.0054</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>0.445</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>-0.017</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>6.7778</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
           <t>-0.00</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>-0.350</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>0.0054</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>0.445</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>1.22</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>-0.017</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>6.7778</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>-0.00</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>-0.00</t>
-        </is>
-      </c>
       <c r="AI2" t="inlineStr">
         <is>
           <t>-0.01</t>
@@ -86344,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>86</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-07-07 16:52 EDT
Score: 85/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85520,13 +85520,13 @@
         <v>1.4775</v>
       </c>
       <c r="R522" t="n">
-        <v>3.96</v>
+        <v>3.95</v>
       </c>
       <c r="S522" t="n">
-        <v>2.4825</v>
+        <v>2.4725</v>
       </c>
       <c r="T522" t="n">
-        <v>2.4825</v>
+        <v>2.4725</v>
       </c>
       <c r="U522" t="n">
         <v>-5.013559261659041</v>
@@ -85538,10 +85538,10 @@
         <v>-2.798809310511419</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.4271421592076718</v>
+        <v>-0.4368622782766174</v>
       </c>
       <c r="Y522" t="n">
-        <v>3.21285140562249</v>
+        <v>2.811244979919679</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,7 +85564,7 @@
         <v>48.01587301587301</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.68479215920767</v>
+        <v>-0.6945122782766155</v>
       </c>
       <c r="AG522" t="n">
         <v>7.128950450387011</v>
@@ -85649,13 +85649,13 @@
         <v>6.79580020904541</v>
       </c>
       <c r="F523" t="n">
-        <v>6.802899837493896</v>
+        <v>6.802710056304932</v>
       </c>
       <c r="G523" t="n">
         <v>6.7835</v>
       </c>
       <c r="H523" t="n">
-        <v>0.007099628448486328</v>
+        <v>0.006909847259521484</v>
       </c>
       <c r="I523" t="n">
         <v>100.8499984741211</v>
@@ -85685,13 +85685,13 @@
         <v>1.4742</v>
       </c>
       <c r="R523" t="n">
-        <v>3.96</v>
+        <v>3.95</v>
       </c>
       <c r="S523" t="n">
-        <v>2.4858</v>
+        <v>2.4758</v>
       </c>
       <c r="T523" t="n">
-        <v>2.4858</v>
+        <v>2.4758</v>
       </c>
       <c r="U523" t="n">
         <v>-4.921134333451794</v>
@@ -85703,7 +85703,7 @@
         <v>-2.622210829685956</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2402503785415178</v>
+        <v>-0.2499881574585361</v>
       </c>
       <c r="Y523" t="n">
         <v>6.42570281124498</v>
@@ -85729,7 +85729,7 @@
         <v>50</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.5012003785415109</v>
+        <v>-0.5109381574585292</v>
       </c>
       <c r="AG523" t="n">
         <v>7.130230666365533</v>
@@ -86054,12 +86054,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.96</t>
+          <t>3.95</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.49</t>
+          <t>2.48</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86069,7 +86069,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86109,7 +86109,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.50</t>
+          <t>-0.51</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-08 16:23 EDT
Score: 75/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.4742</v>
       </c>
       <c r="R523" t="n">
-        <v>3.95</v>
+        <v>4.06</v>
       </c>
       <c r="S523" t="n">
-        <v>2.4758</v>
+        <v>2.5858</v>
       </c>
       <c r="T523" t="n">
-        <v>2.4758</v>
+        <v>2.5858</v>
       </c>
       <c r="U523" t="n">
         <v>-4.800327050049622</v>
@@ -85703,10 +85703,10 @@
         <v>-2.901795270304308</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.5406161834813128</v>
+        <v>-0.4338081582786701</v>
       </c>
       <c r="Y523" t="n">
-        <v>0.8032128514056225</v>
+        <v>3.21285140562249</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>34.92063492063492</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.786266183481299</v>
+        <v>-0.6794581582786563</v>
       </c>
       <c r="AG523" t="n">
         <v>7.122020844747546</v>
@@ -85811,16 +85811,16 @@
         <v>2.9411</v>
       </c>
       <c r="E524" t="n">
-        <v>6.79580020904541</v>
+        <v>6.793399810791016</v>
       </c>
       <c r="F524" t="n">
-        <v>6.8041</v>
+        <v>6.8055</v>
       </c>
       <c r="G524" t="n">
         <v>6.7926</v>
       </c>
       <c r="H524" t="n">
-        <v>0.008299790954589881</v>
+        <v>0.0121001892089847</v>
       </c>
       <c r="I524" t="n">
         <v>101.1399993896484</v>
@@ -85850,28 +85850,28 @@
         <v>1.4739</v>
       </c>
       <c r="R524" t="n">
-        <v>3.95</v>
+        <v>4.06</v>
       </c>
       <c r="S524" t="n">
-        <v>2.4761</v>
+        <v>2.5861</v>
       </c>
       <c r="T524" t="n">
-        <v>2.4761</v>
+        <v>2.5861</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.638140639053372</v>
+        <v>-4.675113762545102</v>
       </c>
       <c r="V524" t="n">
         <v>6.6185</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.60896735618299</v>
+        <v>-2.574554945422103</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2359215667522063</v>
+        <v>-0.09298187620625509</v>
       </c>
       <c r="Y524" t="n">
-        <v>6.827309236947791</v>
+        <v>10.8433734939759</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>34.92063492063492</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.48187156675219</v>
+        <v>-0.3389318762062388</v>
       </c>
       <c r="AG524" t="n">
         <v>7.110998980290019</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3151987712446092</v>
+        <v>-0.3175991694990037</v>
       </c>
       <c r="AI524" t="n">
         <v>6.777782796571369</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.01801741247404109</v>
+        <v>0.01561701421964656</v>
       </c>
       <c r="AK524" t="n">
         <v>6.767889899932765</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.02791030911264514</v>
+        <v>0.02550991085825061</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3660007866474812</v>
@@ -85924,13 +85924,13 @@
         <v>0.4997690914082398</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.431925132075766</v>
+        <v>1.406729556864538</v>
       </c>
       <c r="AQ524" t="n">
-        <v>79.8</v>
+        <v>78.8</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.01740534829500343</v>
+        <v>-0.01739019580162808</v>
       </c>
       <c r="AS524" t="n">
         <v>6.8035</v>
@@ -85954,10 +85954,10 @@
         <v>63.09523809523809</v>
       </c>
       <c r="AZ524" t="n">
-        <v>80.53333333333333</v>
+        <v>80.23333333333332</v>
       </c>
       <c r="BA524" t="n">
-        <v>74.87</v>
+        <v>74.80999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -86169,12 +86169,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.80</t>
+          <t>6.79</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.80</t>
+          <t>6.81</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.95</t>
+          <t>4.06</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.48</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-09 16:49 EDT
Score: 88/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85811,16 +85811,16 @@
         <v>2.961</v>
       </c>
       <c r="E524" t="n">
-        <v>6.793399810791016</v>
+        <v>6.802499771118164</v>
       </c>
       <c r="F524" t="n">
-        <v>6.796879768371582</v>
+        <v>6.79596996307373</v>
       </c>
       <c r="G524" t="n">
         <v>6.7813</v>
       </c>
       <c r="H524" t="n">
-        <v>0.003479957580566406</v>
+        <v>-0.006529808044433594</v>
       </c>
       <c r="I524" t="n">
         <v>101.0500030517578</v>
@@ -85859,19 +85859,19 @@
         <v>2.587499999999999</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.56713146402871</v>
+        <v>-4.42724807117856</v>
       </c>
       <c r="V524" t="n">
         <v>6.6144</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.634907642366091</v>
+        <v>-2.765156596061824</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.1543848926461644</v>
+        <v>-0.2899219538619491</v>
       </c>
       <c r="Y524" t="n">
-        <v>9.236947791164658</v>
+        <v>6.024096385542169</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>35.71428571428572</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.401274892646164</v>
+        <v>-0.5368119538619487</v>
       </c>
       <c r="AG524" t="n">
         <v>7.103663311026919</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3102635002359033</v>
+        <v>-0.3011635399087549</v>
       </c>
       <c r="AI524" t="n">
         <v>6.769987309553778</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.02341250123723793</v>
+        <v>0.03251246156438636</v>
       </c>
       <c r="AK524" t="n">
         <v>6.759766754404358</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.03363305638665715</v>
+        <v>0.04273301671380558</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3700034659576358</v>
@@ -85924,13 +85924,13 @@
         <v>0.5120623436103316</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.484715684815194</v>
+        <v>1.579874079083509</v>
       </c>
       <c r="AQ524" t="n">
-        <v>80.2</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.01762154256789362</v>
+        <v>-0.01768577082363138</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85954,10 +85954,10 @@
         <v>85.71428571428571</v>
       </c>
       <c r="AZ524" t="n">
-        <v>88.84999999999999</v>
+        <v>89.20999999999999</v>
       </c>
       <c r="BA524" t="n">
-        <v>87.85950411141945</v>
+        <v>87.93150411141946</v>
       </c>
     </row>
   </sheetData>
@@ -86169,7 +86169,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.79</t>
+          <t>6.80</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,22 +86274,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.40</t>
+          <t>-0.54</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.48</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-10 15:48 EDT
Score: 87/100
USD/CNY: 6.80
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.802499771118164</v>
       </c>
       <c r="F524" t="n">
-        <v>6.779240131378174</v>
+        <v>6.781529903411865</v>
       </c>
       <c r="G524" t="n">
         <v>6.7644</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.02325963973999023</v>
+        <v>-0.02096986770629883</v>
       </c>
       <c r="I524" t="n">
         <v>100.9400024414062</v>

</xml_diff>

<commit_message>
auto: data update 2026-07-11 15:19 EDT
Score: 87/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85697,16 +85697,16 @@
         <v>-4.654726879307909</v>
       </c>
       <c r="V523" t="n">
-        <v>6.6003</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.823868229759674</v>
+        <v>-2.848897307833309</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.3901877325960257</v>
+        <v>-0.4162229796082162</v>
       </c>
       <c r="Y523" t="n">
-        <v>5.220883534136546</v>
+        <v>4.819277108433734</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>34.92063492063492</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.6367777325960278</v>
+        <v>-0.6628129796082183</v>
       </c>
       <c r="AG523" t="n">
         <v>7.108253654865436</v>
@@ -86069,7 +86069,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.39</t>
+          <t>-0.42</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86109,7 +86109,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.64</t>
+          <t>-0.66</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-13 15:39 EDT
Score: 86/100
USD/CNY: 6.79
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.792099952697754</v>
       </c>
       <c r="F522" t="n">
-        <v>6.784910202026367</v>
+        <v>6.784470081329346</v>
       </c>
       <c r="G522" t="n">
         <v>6.7683</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.007189750671386719</v>
+        <v>-0.007629871368408203</v>
       </c>
       <c r="I522" t="n">
         <v>100.9700012207031</v>

</xml_diff>

<commit_message>
auto: data update 2026-07-13 16:18 EDT
Score: 86/100
USD/CNY: 6.78
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85355,13 +85355,13 @@
         <v>1.4728</v>
       </c>
       <c r="R521" t="n">
-        <v>4.02</v>
+        <v>4.06</v>
       </c>
       <c r="S521" t="n">
-        <v>2.547199999999999</v>
+        <v>2.587199999999999</v>
       </c>
       <c r="T521" t="n">
-        <v>2.547199999999999</v>
+        <v>2.587199999999999</v>
       </c>
       <c r="U521" t="n">
         <v>-4.654726879307909</v>
@@ -85373,10 +85373,10 @@
         <v>-2.848897307833309</v>
       </c>
       <c r="X521" t="n">
-        <v>-0.4162229796082162</v>
+        <v>-0.3773625385313562</v>
       </c>
       <c r="Y521" t="n">
-        <v>4.819277108433734</v>
+        <v>5.220883534136546</v>
       </c>
       <c r="Z521" t="inlineStr">
         <is>
@@ -85399,7 +85399,7 @@
         <v>34.92063492063492</v>
       </c>
       <c r="AF521" t="n">
-        <v>-0.6628129796082183</v>
+        <v>-0.6239525385313582</v>
       </c>
       <c r="AG521" t="n">
         <v>7.108253654865436</v>
@@ -85481,16 +85481,16 @@
         <v>2.9485</v>
       </c>
       <c r="E522" t="n">
-        <v>6.792099952697754</v>
+        <v>6.776599884033203</v>
       </c>
       <c r="F522" t="n">
-        <v>6.784470081329346</v>
+        <v>6.784500122070312</v>
       </c>
       <c r="G522" t="n">
         <v>6.7683</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.007629871368408203</v>
+        <v>0.007900238037109375</v>
       </c>
       <c r="I522" t="n">
         <v>100.9700012207031</v>
@@ -85520,28 +85520,28 @@
         <v>1.4735</v>
       </c>
       <c r="R522" t="n">
-        <v>4.02</v>
+        <v>4.06</v>
       </c>
       <c r="S522" t="n">
-        <v>2.5465</v>
+        <v>2.5865</v>
       </c>
       <c r="T522" t="n">
-        <v>2.5465</v>
+        <v>2.5865</v>
       </c>
       <c r="U522" t="n">
-        <v>-4.413088187676177</v>
+        <v>-4.651911500854224</v>
       </c>
       <c r="V522" t="n">
         <v>6.6014</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.807672943947326</v>
+        <v>-2.585365626292957</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.3740413962940004</v>
+        <v>-0.1038314707204391</v>
       </c>
       <c r="Y522" t="n">
-        <v>5.622489959839357</v>
+        <v>12.04819277108434</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,25 +85564,25 @@
         <v>34.12698412698413</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.6199313962940156</v>
+        <v>-0.3497214707204543</v>
       </c>
       <c r="AG522" t="n">
         <v>7.091841313405418</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.2997413607076638</v>
+        <v>-0.3152414293722146</v>
       </c>
       <c r="AI522" t="n">
         <v>6.775018791664189</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.01708116103356527</v>
+        <v>0.001581092369014492</v>
       </c>
       <c r="AK522" t="n">
         <v>6.761698703407076</v>
       </c>
       <c r="AL522" t="n">
-        <v>0.03040124929067822</v>
+        <v>0.01490118062612744</v>
       </c>
       <c r="AM522" t="n">
         <v>-0.3816350905604304</v>
@@ -85594,13 +85594,13 @@
         <v>0.537958310473289</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.410596659939346</v>
+        <v>1.248514126271823</v>
       </c>
       <c r="AQ522" t="n">
-        <v>80.80000000000001</v>
+        <v>77</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.01735653601348189</v>
+        <v>-0.01724891280684824</v>
       </c>
       <c r="AS522" t="n">
         <v>6.7778000831604</v>
@@ -85624,10 +85624,10 @@
         <v>64.70588235294117</v>
       </c>
       <c r="AZ522" t="n">
-        <v>81.53705882352941</v>
+        <v>80.39705882352941</v>
       </c>
       <c r="BA522" t="n">
-        <v>86.39383375052148</v>
+        <v>86.16583375052149</v>
       </c>
     </row>
   </sheetData>
@@ -85839,7 +85839,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.79</t>
+          <t>6.78</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -85889,12 +85889,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.02</t>
+          <t>4.06</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.55</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -85904,12 +85904,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.37</t>
+          <t>-0.10</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>12</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85944,22 +85944,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.62</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -85979,7 +85979,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-14 16:15 EDT
Score: 68/100
USD/CNY: 6.78
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85646,16 +85646,16 @@
         <v>2.9934</v>
       </c>
       <c r="E523" t="n">
-        <v>6.776599884033203</v>
+        <v>6.779500007629395</v>
       </c>
       <c r="F523" t="n">
-        <v>6.7737</v>
+        <v>6.7739</v>
       </c>
       <c r="G523" t="n">
         <v>6.7576</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.002899884033203293</v>
+        <v>-0.005600007629394277</v>
       </c>
       <c r="I523" t="n">
         <v>101.2799987792969</v>
@@ -85694,19 +85694,19 @@
         <v>2.5866</v>
       </c>
       <c r="U523" t="n">
-        <v>-4.511948999669444</v>
+        <v>-4.467241046422626</v>
       </c>
       <c r="V523" t="n">
         <v>6.595</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.679808268761485</v>
+        <v>-2.721439743664955</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.202008484473204</v>
+        <v>-0.2453301972577648</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.433734939759036</v>
+        <v>8.032128514056225</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,25 +85729,25 @@
         <v>34.12698412698413</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.447998484473211</v>
+        <v>-0.4913201972577719</v>
       </c>
       <c r="AG523" t="n">
         <v>7.08235661471244</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3057567306792368</v>
+        <v>-0.3028566070830454</v>
       </c>
       <c r="AI523" t="n">
         <v>6.76332928403141</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.01327060000179348</v>
+        <v>0.01617072359798488</v>
       </c>
       <c r="AK523" t="n">
         <v>6.744939020214936</v>
       </c>
       <c r="AL523" t="n">
-        <v>0.03166086381826716</v>
+        <v>0.03456098741445857</v>
       </c>
       <c r="AM523" t="n">
         <v>-0.3872393091179336</v>
@@ -85759,13 +85759,13 @@
         <v>0.5511317941481411</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.365699136480587</v>
+        <v>1.39593084714911</v>
       </c>
       <c r="AQ523" t="n">
-        <v>79</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.01873119790987359</v>
+        <v>-0.01875152901911802</v>
       </c>
       <c r="AS523" t="n">
         <v>6.7857</v>
@@ -85789,10 +85789,10 @@
         <v>8.730158730158729</v>
       </c>
       <c r="AZ523" t="n">
-        <v>61.54555555555555</v>
+        <v>61.96555555555555</v>
       </c>
       <c r="BA523" t="n">
-        <v>68.39022222222222</v>
+        <v>68.47422222222221</v>
       </c>
     </row>
   </sheetData>
@@ -86069,7 +86069,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.20</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86109,17 +86109,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86144,7 +86144,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-15 12:14 EDT
Score: 79/100
USD/CNY: 6.78
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85658,10 +85658,10 @@
         <v>-0.001699924468994141</v>
       </c>
       <c r="I523" t="n">
-        <v>101.2799987792969</v>
+        <v>100.9400024414062</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>-0.003356993897990934</v>
       </c>
       <c r="K523" t="n">
         <v>2.9102</v>
@@ -85738,10 +85738,10 @@
         <v>-0.3137378908481967</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.795547594550022</v>
+        <v>6.789815280543246</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.01604758692062713</v>
+        <v>-0.01031527291385181</v>
       </c>
       <c r="AK523" t="n">
         <v>6.744939020214936</v>
@@ -85759,40 +85759,40 @@
         <v>0.5511317941481411</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.059279406782159</v>
+        <v>1.11929705519035</v>
       </c>
       <c r="AQ523" t="n">
-        <v>73.59999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.01875152901911802</v>
+        <v>-0.01935177719733854</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7778000831604</v>
+        <v>6.778240394795662</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.02020008316040034</v>
+        <v>-0.02064039479566215</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.02020008316040034</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.002838790261682789</v>
+        <v>-0.002860805843445879</v>
       </c>
       <c r="AW523" t="n">
         <v/>
       </c>
       <c r="AX523" t="n">
-        <v>0.01624649551193112</v>
+        <v>0.01624759629101927</v>
       </c>
       <c r="AY523" t="n">
         <v>48.07692307692308</v>
       </c>
       <c r="AZ523" t="n">
-        <v>72.50692307692307</v>
+        <v>72.74692307692307</v>
       </c>
       <c r="BA523" t="n">
-        <v>82.80496304675715</v>
+        <v>82.85296304675715</v>
       </c>
     </row>
     <row r="524">
@@ -85814,16 +85814,16 @@
         <v>6.779500007629395</v>
       </c>
       <c r="F524" t="n">
-        <v>6.771689891815186</v>
+        <v>6.770559787750244</v>
       </c>
       <c r="G524" t="n">
-        <v>6.756799999999999</v>
+        <v>6.756699999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.007810115814208984</v>
+        <v>-0.008940219879150391</v>
       </c>
       <c r="I524" t="n">
-        <v>101.2799987792969</v>
+        <v>100.9400024414062</v>
       </c>
       <c r="J524" t="n">
         <v>0</v>
@@ -85903,10 +85903,10 @@
         <v>-0.3167040309578999</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.795595880328118</v>
+        <v>6.789416822421766</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.01609587269872392</v>
+        <v>-0.009916814792371831</v>
       </c>
       <c r="AK524" t="n">
         <v>6.772636231606738</v>
@@ -85915,49 +85915,49 @@
         <v>0.006863776022656864</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.3930613027465069</v>
+        <v>-0.393020019860339</v>
       </c>
       <c r="AN524" t="n">
-        <v>0.01867862727572794</v>
+        <v>0.01873686412955489</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.5644108856084985</v>
+        <v>0.5644439393662184</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.057052712032486</v>
+        <v>1.121156336523879</v>
       </c>
       <c r="AQ524" t="n">
-        <v>72.8</v>
+        <v>73.8</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.02009779819294918</v>
+        <v>-0.02071481787523424</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
       </c>
       <c r="AT524" t="n">
-        <v>-0.02100008316040114</v>
+        <v>-0.02110008316040091</v>
       </c>
       <c r="AU524" t="n">
-        <v>-0.02100008316040114</v>
+        <v>-0.02110008316040091</v>
       </c>
       <c r="AV524" t="n">
-        <v>-0.002403665783411579</v>
+        <v>-0.002430681365174658</v>
       </c>
       <c r="AW524" t="n">
         <v/>
       </c>
       <c r="AX524" t="n">
-        <v>0.01450932895130501</v>
+        <v>0.01451178050948132</v>
       </c>
       <c r="AY524" t="n">
         <v>47.16981132075472</v>
       </c>
       <c r="AZ524" t="n">
-        <v>71.87943396226416</v>
+        <v>72.17943396226416</v>
       </c>
       <c r="BA524" t="n">
-        <v>78.54268317254332</v>
+        <v>78.65068317254332</v>
       </c>
     </row>
   </sheetData>
@@ -86194,7 +86194,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>101.28</t>
+          <t>100.94</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86284,7 +86284,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86309,12 +86309,12 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>-0.020</t>
+          <t>-0.021</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-21 15:42 EDT
Score: 72/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.772500038146973</v>
       </c>
       <c r="F523" t="n">
-        <v>6.767950057983398</v>
+        <v>6.767970085144043</v>
       </c>
       <c r="G523" t="n">
         <v>6.755</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.004549980163574219</v>
+        <v>-0.004529953002929688</v>
       </c>
       <c r="I523" t="n">
         <v>100.9899978637695</v>

</xml_diff>

<commit_message>
auto: data update 2026-07-22 11:26 EDT
Score: 76/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85637,49 +85637,49 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>4.21</v>
+        <v>4.26</v>
       </c>
       <c r="C523" t="n">
         <v>1.2689</v>
       </c>
       <c r="D523" t="n">
-        <v>2.9409</v>
+        <v>2.9911</v>
       </c>
       <c r="E523" t="n">
         <v>6.772500038146973</v>
       </c>
       <c r="F523" t="n">
-        <v>6.769</v>
+        <v>6.7689</v>
       </c>
       <c r="G523" t="n">
         <v>6.755</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.003500038146972528</v>
+        <v>-0.003600038146972295</v>
       </c>
       <c r="I523" t="n">
-        <v>100.9899978637695</v>
+        <v>101.1800003051758</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>0.001881398608033935</v>
       </c>
       <c r="K523" t="n">
-        <v>2.9409</v>
+        <v>2.9911</v>
       </c>
       <c r="L523" t="n">
-        <v>2.90292</v>
+        <v>2.90543</v>
       </c>
       <c r="M523" t="n">
-        <v>2.823651666666666</v>
+        <v>2.824488333333333</v>
       </c>
       <c r="N523" t="n">
         <v/>
       </c>
       <c r="O523" t="n">
-        <v>97</v>
+        <v>99.2</v>
       </c>
       <c r="P523" t="n">
-        <v>90.51896207584831</v>
+        <v>92.41516966067864</v>
       </c>
       <c r="Q523" t="n">
         <v>1.474</v>
@@ -85694,19 +85694,19 @@
         <v>2.556</v>
       </c>
       <c r="U523" t="n">
-        <v>-4.931482159984864</v>
+        <v>-4.830862247124208</v>
       </c>
       <c r="V523" t="n">
-        <v>6.5873</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.73458895686689</v>
+        <v>-2.567737721188013</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2887928918286153</v>
+        <v>-0.1152175513518872</v>
       </c>
       <c r="Y523" t="n">
-        <v>6.827309236947791</v>
+        <v>12.85140562248996</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85714,34 +85714,34 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.71485</v>
+        <v>1.65409</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.60818</v>
+        <v>1.60409</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.43939</v>
+        <v>1.32121</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.24085</v>
+        <v>0.1800900000000001</v>
       </c>
       <c r="AE523" t="n">
-        <v>26.98412698412698</v>
+        <v>0.7936507936507936</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.5296428918286189</v>
+        <v>-0.2953075513518977</v>
       </c>
       <c r="AG523" t="n">
-        <v>7.106484669313159</v>
+        <v>7.099670185676287</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.333984631166186</v>
+        <v>-0.3271701475293147</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.768336774052734</v>
+        <v>6.751667781721844</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.004163264094239061</v>
+        <v>0.02083225642512865</v>
       </c>
       <c r="AK523" t="n">
         <v>6.753855191419989</v>
@@ -85759,40 +85759,205 @@
         <v>0.6129676701055393</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.275593056723391</v>
+        <v>1.449851053645146</v>
       </c>
       <c r="AQ523" t="n">
-        <v>75.2</v>
+        <v>79.2</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.007003369303381743</v>
+        <v>-0.006834851647461732</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7692</v>
+        <v>6.769112954313121</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.01419999999999977</v>
+        <v>-0.01411295431312087</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.01419999999999977</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01621120085361394</v>
+        <v>-0.01620684856927</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01464163897419126</v>
+        <v>-0.01464018821274327</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01473421387743528</v>
+        <v>0.01473399626321808</v>
       </c>
       <c r="AY523" t="n">
-        <v>46.42857142857143</v>
+        <v>46.82539682539682</v>
       </c>
       <c r="AZ523" t="n">
-        <v>72.75999999999999</v>
+        <v>74.86888888888889</v>
       </c>
       <c r="BA523" t="n">
-        <v>71.77888888888889</v>
+        <v>72.20066666666666</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2649</v>
+      </c>
+      <c r="D524" t="n">
+        <v>2.9911</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.772500038146973</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.7747</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.760800000000001</v>
+      </c>
+      <c r="H524" t="n">
+        <v>0.00219996185302751</v>
+      </c>
+      <c r="I524" t="n">
+        <v>101.1800003051758</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>2.9911</v>
+      </c>
+      <c r="L524" t="n">
+        <v>2.912295</v>
+      </c>
+      <c r="M524" t="n">
+        <v>2.829948333333333</v>
+      </c>
+      <c r="N524" t="n">
+        <v/>
+      </c>
+      <c r="O524" t="n">
+        <v>99</v>
+      </c>
+      <c r="P524" t="n">
+        <v>92.31536926147704</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.4755</v>
+      </c>
+      <c r="R524" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.5545</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.5545</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-4.989576934418969</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.5918</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-2.668143774516896</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.2211699686299307</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>8.835341365461847</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.65409</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.60409</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.32121</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.17859</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>0.3968253968253968</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.3997599686299314</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>7.11041913793387</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.3379190997868973</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.751845244455401</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>0.02065479369157153</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.736226026398153</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>0.03627401174881939</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.3964908591695859</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>0.01740130648959376</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.6198907013195262</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>1.452450192364421</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>77</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>-0.007368533431474942</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.7689</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>-0.008099999999999774</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>-0.008099999999999774</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.01682248444114012</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.01458303701557822</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.01494834029962992</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>74.20634920634922</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>83.72222222222223</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>76.46111111111111</v>
       </c>
     </row>
   </sheetData>
@@ -85999,7 +86164,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86014,42 +86179,42 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.75</t>
+          <t>6.76</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.21</t>
+          <t>4.26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>100.99</t>
+          <t>101.18</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.94</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>99</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -86059,7 +86224,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.56</t>
+          <t>2.55</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86069,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.29</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86084,67 +86249,67 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.71</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.53</t>
+          <t>-0.40</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.33</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.398</t>
+          <t>-0.396</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0173</t>
+          <t>0.0174</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.613</t>
+          <t>0.620</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86154,7 +86319,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.7692</t>
+          <t>6.7689</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -86179,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>76</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-07-22 12:15 EDT
Score: 76/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.772500038146973</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7747</v>
+        <v>6.7742</v>
       </c>
       <c r="G524" t="n">
         <v>6.760800000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>0.00219996185302751</v>
+        <v>0.001699961853027787</v>
       </c>
       <c r="I524" t="n">
         <v>101.1800003051758</v>

</xml_diff>

<commit_message>
auto: data update 2026-07-22 15:37 EDT
Score: 76/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.772500038146973</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7742</v>
+        <v>6.7752</v>
       </c>
       <c r="G524" t="n">
         <v>6.760800000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>0.001699961853027787</v>
+        <v>0.002699961853027233</v>
       </c>
       <c r="I524" t="n">
         <v>101.1800003051758</v>
@@ -86174,7 +86174,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.77</t>
+          <t>6.78</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-22 16:18 EDT
Score: 76/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85811,16 +85811,16 @@
         <v>2.9911</v>
       </c>
       <c r="E524" t="n">
-        <v>6.772500038146973</v>
+        <v>6.765600204467773</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7752</v>
+        <v>6.775</v>
       </c>
       <c r="G524" t="n">
         <v>6.760800000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>0.002699961853027233</v>
+        <v>0.009399795532226918</v>
       </c>
       <c r="I524" t="n">
         <v>101.1800003051758</v>
@@ -85859,19 +85859,19 @@
         <v>2.5545</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.989576934418969</v>
+        <v>-5.096649566115209</v>
       </c>
       <c r="V524" t="n">
         <v>6.5918</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.668143774516896</v>
+        <v>-2.568880797198181</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2211699686299307</v>
+        <v>-0.1179066933252759</v>
       </c>
       <c r="Y524" t="n">
-        <v>8.835341365461847</v>
+        <v>12.85140562248996</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>0.3968253968253968</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.3997599686299314</v>
+        <v>-0.2964966933252766</v>
       </c>
       <c r="AG524" t="n">
         <v>7.11041913793387</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3379190997868973</v>
+        <v>-0.3448189334660965</v>
       </c>
       <c r="AI524" t="n">
         <v>6.751845244455401</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.02065479369157153</v>
+        <v>0.01375496001237231</v>
       </c>
       <c r="AK524" t="n">
         <v>6.736226026398153</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.03627401174881939</v>
+        <v>0.02937417806962017</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3964908591695859</v>
@@ -85924,13 +85924,13 @@
         <v>0.6198907013195262</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.452450192364421</v>
+        <v>1.380226358427129</v>
       </c>
       <c r="AQ524" t="n">
-        <v>77</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.007368533431474942</v>
+        <v>-0.0073321786938442</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7689</v>
@@ -85954,10 +85954,10 @@
         <v>74.20634920634922</v>
       </c>
       <c r="AZ524" t="n">
-        <v>83.72222222222223</v>
+        <v>82.70222222222222</v>
       </c>
       <c r="BA524" t="n">
-        <v>76.46111111111111</v>
+        <v>76.25711111111112</v>
       </c>
     </row>
   </sheetData>
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.40</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86284,12 +86284,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-27 15:45 EDT
Score: 77/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85328,10 +85328,10 @@
         <v>0.005300045013427734</v>
       </c>
       <c r="I521" t="n">
-        <v>101.4700012207031</v>
+        <v>101.4300003051758</v>
       </c>
       <c r="J521" t="n">
-        <v>0.000394369667820138</v>
+        <v>0</v>
       </c>
       <c r="K521" t="n">
         <v>3.0607</v>
@@ -85408,10 +85408,10 @@
         <v>-0.3026099231499435</v>
       </c>
       <c r="AI521" t="n">
-        <v>6.731179671396989</v>
+        <v>6.730473016530254</v>
       </c>
       <c r="AJ521" t="n">
-        <v>0.04132036674998396</v>
+        <v>0.04202702161671823</v>
       </c>
       <c r="AK521" t="n">
         <v>6.699415101064979</v>
@@ -85429,31 +85429,31 @@
         <v>0.6334129699358579</v>
       </c>
       <c r="AP521" t="n">
-        <v>1.659142843632353</v>
+        <v>1.666476021183947</v>
       </c>
       <c r="AQ521" t="n">
         <v>83.59999999999999</v>
       </c>
       <c r="AR521" t="n">
-        <v>-0.004023434406281946</v>
+        <v>-0.004056261939140153</v>
       </c>
       <c r="AS521" t="n">
-        <v>6.777789328686129</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="AT521" t="n">
-        <v>-0.01858932868612939</v>
+        <v>-0.01860008316040052</v>
       </c>
       <c r="AU521" t="n">
         <v>-0.01860008316040052</v>
       </c>
       <c r="AV521" t="n">
-        <v>-0.008163438475363893</v>
+        <v>-0.008163976199077449</v>
       </c>
       <c r="AW521" t="n">
-        <v>-0.02279946196507197</v>
+        <v>-0.02279964120630983</v>
       </c>
       <c r="AX521" t="n">
-        <v>0.006200241951505226</v>
+        <v>0.006200268837690903</v>
       </c>
       <c r="AY521" t="n">
         <v>50</v>
@@ -85484,16 +85484,16 @@
         <v>6.772500038146973</v>
       </c>
       <c r="F522" t="n">
-        <v>6.763539791107178</v>
+        <v>6.76471996307373</v>
       </c>
       <c r="G522" t="n">
         <v>6.7524</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.008960247039794922</v>
+        <v>-0.007780075073242188</v>
       </c>
       <c r="I522" t="n">
-        <v>101.4700012207031</v>
+        <v>101.4300003051758</v>
       </c>
       <c r="J522" t="n">
         <v>0</v>
@@ -85573,10 +85573,10 @@
         <v>-0.3074391409091621</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.732547738986348</v>
+        <v>6.731823957437258</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.0399522991606247</v>
+        <v>0.04067608070971485</v>
       </c>
       <c r="AK522" t="n">
         <v>6.714685154719483</v>
@@ -85585,22 +85585,22 @@
         <v>0.05781488342748986</v>
       </c>
       <c r="AM522" t="n">
-        <v>-0.3929423394238508</v>
+        <v>-0.3929111188475297</v>
       </c>
       <c r="AN522" t="n">
-        <v>0.01842070378092631</v>
+        <v>0.0184160223266695</v>
       </c>
       <c r="AO522" t="n">
-        <v>0.640374511165978</v>
+        <v>0.6403625127842805</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.641224027314495</v>
+        <v>1.648613895812288</v>
       </c>
       <c r="AQ522" t="n">
         <v>82.80000000000001</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.004152980915098716</v>
+        <v>-0.004185826460177477</v>
       </c>
       <c r="AS522" t="n">
         <v>6.7778000831604</v>
@@ -85612,13 +85612,13 @@
         <v>-0.02540008316040065</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.009803613606400585</v>
+        <v>-0.009804151330114141</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02311295786935557</v>
+        <v>-0.02311313711059343</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.006016948192040539</v>
+        <v>0.006017001964411894</v>
       </c>
       <c r="AY522" t="n">
         <v>40.98360655737705</v>
@@ -85864,7 +85864,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>101.47</t>
+          <t>101.43</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -85979,7 +85979,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-28 16:18 EDT
Score: 77/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85328,10 +85328,10 @@
         <v>-0.0008000381469726037</v>
       </c>
       <c r="I521" t="n">
-        <v>101.4700012207031</v>
+        <v>101.4300003051758</v>
       </c>
       <c r="J521" t="n">
-        <v>0.000394369667820138</v>
+        <v>0</v>
       </c>
       <c r="K521" t="n">
         <v>3.0607</v>
@@ -85408,10 +85408,10 @@
         <v>-0.3026099231499435</v>
       </c>
       <c r="AI521" t="n">
-        <v>6.731179671396997</v>
+        <v>6.730473016530262</v>
       </c>
       <c r="AJ521" t="n">
-        <v>0.04132036674997597</v>
+        <v>0.04202702161671112</v>
       </c>
       <c r="AK521" t="n">
         <v>6.699415101064979</v>
@@ -85429,31 +85429,31 @@
         <v>0.6334129699358579</v>
       </c>
       <c r="AP521" t="n">
-        <v>1.659142843632271</v>
+        <v>1.666476021183875</v>
       </c>
       <c r="AQ521" t="n">
         <v>83.59999999999999</v>
       </c>
       <c r="AR521" t="n">
-        <v>-0.004023434406281946</v>
+        <v>-0.004056261939140153</v>
       </c>
       <c r="AS521" t="n">
-        <v>6.77778924552586</v>
+        <v>6.7778</v>
       </c>
       <c r="AT521" t="n">
-        <v>-0.0185892455258605</v>
+        <v>-0.01860000000000017</v>
       </c>
       <c r="AU521" t="n">
         <v>-0.01860000000000017</v>
       </c>
       <c r="AV521" t="n">
-        <v>-0.01616849012092603</v>
+        <v>-0.01616902784463301</v>
       </c>
       <c r="AW521" t="n">
-        <v>-0.01436512198313518</v>
+        <v>-0.01436530122437085</v>
       </c>
       <c r="AX521" t="n">
-        <v>0.01525119053772384</v>
+        <v>0.01525121742390918</v>
       </c>
       <c r="AY521" t="n">
         <v>25</v>
@@ -85493,10 +85493,10 @@
         <v>-0.006500041198730599</v>
       </c>
       <c r="I522" t="n">
-        <v>101.4700012207031</v>
+        <v>101.5100021362305</v>
       </c>
       <c r="J522" t="n">
-        <v>0</v>
+        <v>0.0007887393356402761</v>
       </c>
       <c r="K522" t="n">
         <v>3.0412</v>
@@ -85573,10 +85573,10 @@
         <v>-0.3108543589941197</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.74021011460511</v>
+        <v>6.740959039761663</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.03158992659362081</v>
+        <v>0.03084100143706703</v>
       </c>
       <c r="AK522" t="n">
         <v>6.714685154719483</v>
@@ -85585,49 +85585,49 @@
         <v>0.05711488647924767</v>
       </c>
       <c r="AM522" t="n">
-        <v>-0.392942339423851</v>
+        <v>-0.3929111188475297</v>
       </c>
       <c r="AN522" t="n">
-        <v>0.0184207037809263</v>
+        <v>0.01841602232666951</v>
       </c>
       <c r="AO522" t="n">
-        <v>0.6403745111659787</v>
+        <v>0.6403625127842802</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.554475762548375</v>
+        <v>1.546593094679171</v>
       </c>
       <c r="AQ522" t="n">
         <v>81.8</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.004148262386322705</v>
+        <v>-0.004144098042268884</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.7717</v>
+        <v>6.771677865932422</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.01930000000000032</v>
+        <v>-0.01927786593242242</v>
       </c>
       <c r="AU522" t="n">
         <v>-0.01930000000000032</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.01616860685207428</v>
+        <v>-0.01616803787240238</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.01455528240688933</v>
+        <v>-0.0145550927469987</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01538783972232463</v>
+        <v>0.01538783815952639</v>
       </c>
       <c r="AY522" t="n">
-        <v>23.80952380952381</v>
+        <v>24.20634920634921</v>
       </c>
       <c r="AZ522" t="n">
-        <v>67.45333333333333</v>
+        <v>67.59222222222222</v>
       </c>
       <c r="BA522" t="n">
-        <v>75.98177777777778</v>
+        <v>76.00955555555556</v>
       </c>
     </row>
     <row r="523">
@@ -85646,19 +85646,19 @@
         <v>3.0412</v>
       </c>
       <c r="E523" t="n">
-        <v>6.77180004119873</v>
+        <v>6.765699863433838</v>
       </c>
       <c r="F523" t="n">
-        <v>6.7708</v>
+        <v>6.7711</v>
       </c>
       <c r="G523" t="n">
         <v>6.756</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.001000041198730095</v>
+        <v>0.005400136566161784</v>
       </c>
       <c r="I523" t="n">
-        <v>101.4700012207031</v>
+        <v>101.5100021362305</v>
       </c>
       <c r="J523" t="n">
         <v>0</v>
@@ -85694,19 +85694,19 @@
         <v>2.66</v>
       </c>
       <c r="U523" t="n">
-        <v>-4.665736110508692</v>
+        <v>-4.760106184419033</v>
       </c>
       <c r="V523" t="n">
         <v>6.5824</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.796893588801297</v>
+        <v>-2.709252067543044</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.252684983377649</v>
+        <v>-0.1614151031393174</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.032128514056225</v>
+        <v>10.44176706827309</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,43 +85729,43 @@
         <v>8.928571428571429</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4578349833776585</v>
+        <v>-0.3665651031393269</v>
       </c>
       <c r="AG523" t="n">
         <v>7.087754361052382</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3159543198536516</v>
+        <v>-0.3220544976185442</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.740909840959077</v>
+        <v>6.741668983377259</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.03089020023965361</v>
+        <v>0.02403088005657938</v>
       </c>
       <c r="AK523" t="n">
         <v>6.722064699270507</v>
       </c>
       <c r="AL523" t="n">
-        <v>0.0497353419282236</v>
+        <v>0.04363516416333102</v>
       </c>
       <c r="AM523" t="n">
-        <v>-0.3931146518891239</v>
+        <v>-0.3931090237000185</v>
       </c>
       <c r="AN523" t="n">
-        <v>0.01902481078771318</v>
+        <v>0.01902261654170435</v>
       </c>
       <c r="AO523" t="n">
-        <v>0.6484763062471188</v>
+        <v>0.6484734929758087</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.544012672016944</v>
+        <v>1.472839619605213</v>
       </c>
       <c r="AQ523" t="n">
-        <v>81</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.004183427886888702</v>
+        <v>-0.004134826640182815</v>
       </c>
       <c r="AS523" t="n">
         <v>6.7653</v>
@@ -85777,22 +85777,22 @@
         <v>-0.009299999999999642</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01533832677469102</v>
+        <v>-0.01533775779501911</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01456727726885478</v>
+        <v>-0.01456708760896414</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01545413923320929</v>
+        <v>0.01545410922142745</v>
       </c>
       <c r="AY523" t="n">
         <v>67.06349206349206</v>
       </c>
       <c r="AZ523" t="n">
-        <v>82.28222222222223</v>
+        <v>82.16222222222223</v>
       </c>
       <c r="BA523" t="n">
-        <v>77.46444444444444</v>
+        <v>77.46822222222222</v>
       </c>
     </row>
   </sheetData>
@@ -86029,7 +86029,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>101.47</t>
+          <t>101.51</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86069,12 +86069,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86109,7 +86109,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.46</t>
+          <t>-0.37</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86119,12 +86119,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86144,7 +86144,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-29 12:16 EDT
Score: 75/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85328,10 +85328,10 @@
         <v>-0.0008000381469726037</v>
       </c>
       <c r="I521" t="n">
-        <v>101.4300003051758</v>
+        <v>101.4700012207031</v>
       </c>
       <c r="J521" t="n">
-        <v>0</v>
+        <v>0.000394369667820138</v>
       </c>
       <c r="K521" t="n">
         <v>3.0607</v>
@@ -85408,10 +85408,10 @@
         <v>-0.3026099231499435</v>
       </c>
       <c r="AI521" t="n">
-        <v>6.730473016530254</v>
+        <v>6.731179671396989</v>
       </c>
       <c r="AJ521" t="n">
-        <v>0.04202702161671823</v>
+        <v>0.04132036674998396</v>
       </c>
       <c r="AK521" t="n">
         <v>6.699415101064979</v>
@@ -85429,31 +85429,31 @@
         <v>0.6334129699358579</v>
       </c>
       <c r="AP521" t="n">
-        <v>1.666476021183947</v>
+        <v>1.659142843632353</v>
       </c>
       <c r="AQ521" t="n">
         <v>83.59999999999999</v>
       </c>
       <c r="AR521" t="n">
-        <v>-0.004056261939140153</v>
+        <v>-0.004023434406281946</v>
       </c>
       <c r="AS521" t="n">
-        <v>6.7778</v>
+        <v>6.77778924552586</v>
       </c>
       <c r="AT521" t="n">
-        <v>-0.01860000000000017</v>
+        <v>-0.0185892455258605</v>
       </c>
       <c r="AU521" t="n">
         <v>-0.01860000000000017</v>
       </c>
       <c r="AV521" t="n">
-        <v>-0.01616902784463301</v>
+        <v>-0.01616849012092603</v>
       </c>
       <c r="AW521" t="n">
-        <v>-0.01436530122437085</v>
+        <v>-0.01436512198313518</v>
       </c>
       <c r="AX521" t="n">
-        <v>0.01525121742390918</v>
+        <v>0.01525119053772384</v>
       </c>
       <c r="AY521" t="n">
         <v>25</v>
@@ -85493,10 +85493,10 @@
         <v>-0.006500041198730599</v>
       </c>
       <c r="I522" t="n">
-        <v>101.5100021362305</v>
+        <v>101.4700012207031</v>
       </c>
       <c r="J522" t="n">
-        <v>0.0007887393356402761</v>
+        <v>0</v>
       </c>
       <c r="K522" t="n">
         <v>3.0412</v>
@@ -85573,10 +85573,10 @@
         <v>-0.3108543589941197</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.740959039761663</v>
+        <v>6.740210114605112</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.03084100143706792</v>
+        <v>0.03158992659361815</v>
       </c>
       <c r="AK522" t="n">
         <v>6.714685154719483</v>
@@ -85585,49 +85585,49 @@
         <v>0.05711488647924767</v>
       </c>
       <c r="AM522" t="n">
-        <v>-0.3929111188475297</v>
+        <v>-0.3929423394238508</v>
       </c>
       <c r="AN522" t="n">
-        <v>0.0184160223266695</v>
+        <v>0.01842070378092631</v>
       </c>
       <c r="AO522" t="n">
-        <v>0.6403625127842805</v>
+        <v>0.640374511165978</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.546593094679178</v>
+        <v>1.554475762548346</v>
       </c>
       <c r="AQ522" t="n">
         <v>81.8</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.004144098042268884</v>
+        <v>-0.004148262386322705</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.771677865932422</v>
+        <v>6.7717</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.01927786593242242</v>
+        <v>-0.01930000000000032</v>
       </c>
       <c r="AU522" t="n">
         <v>-0.01930000000000032</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.01616803787240238</v>
+        <v>-0.01616860685207428</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.0145550927469987</v>
+        <v>-0.01455528240688933</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01538783815952639</v>
+        <v>0.01538783972232463</v>
       </c>
       <c r="AY522" t="n">
-        <v>24.20634920634921</v>
+        <v>23.80952380952381</v>
       </c>
       <c r="AZ522" t="n">
-        <v>67.59222222222222</v>
+        <v>67.45333333333333</v>
       </c>
       <c r="BA522" t="n">
-        <v>76.00955555555556</v>
+        <v>75.98177777777778</v>
       </c>
     </row>
     <row r="523">
@@ -85658,10 +85658,10 @@
         <v>0.005500136566162439</v>
       </c>
       <c r="I523" t="n">
-        <v>101.5100021362305</v>
+        <v>101.379997253418</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>-0.000887000750984468</v>
       </c>
       <c r="K523" t="n">
         <v>2.9909</v>
@@ -85738,10 +85738,10 @@
         <v>-0.3288542807561932</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.76144236726937</v>
+        <v>6.758971199501358</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.004257496164467689</v>
+        <v>0.006728663932479506</v>
       </c>
       <c r="AK523" t="n">
         <v>6.722064699270507</v>
@@ -85750,40 +85750,40 @@
         <v>0.04363516416333102</v>
       </c>
       <c r="AM523" t="n">
-        <v>-0.3931090237000187</v>
+        <v>-0.3931146518891241</v>
       </c>
       <c r="AN523" t="n">
-        <v>0.01902261654170434</v>
+        <v>0.01902481078771323</v>
       </c>
       <c r="AO523" t="n">
-        <v>0.6484734929758089</v>
+        <v>0.6484763062471189</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.267170832868127</v>
+        <v>1.292910986116276</v>
       </c>
       <c r="AQ523" t="n">
         <v>76.40000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.004134826640182815</v>
+        <v>-0.003925942751382671</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7653</v>
+        <v>6.765323558900046</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.009299999999999642</v>
+        <v>-0.009323558900045548</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.009299999999999642</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01533775779501911</v>
+        <v>-0.01533950471969332</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01456708760896414</v>
+        <v>-0.01456766991718888</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01545410922142745</v>
+        <v>0.01545419813045941</v>
       </c>
       <c r="AY523" t="n">
         <v>67.06349206349206</v>
@@ -85792,7 +85792,7 @@
         <v>80.41222222222223</v>
       </c>
       <c r="BA523" t="n">
-        <v>77.11822222222222</v>
+        <v>77.09044444444444</v>
       </c>
     </row>
     <row r="524">
@@ -85814,16 +85814,16 @@
         <v>6.765699863433838</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7714</v>
+        <v>6.7717</v>
       </c>
       <c r="G524" t="n">
-        <v>6.7566</v>
+        <v>6.757400000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>0.005700136566161973</v>
+        <v>0.006000136566162162</v>
       </c>
       <c r="I524" t="n">
-        <v>101.5100021362305</v>
+        <v>101.379997253418</v>
       </c>
       <c r="J524" t="n">
         <v>0</v>
@@ -85903,10 +85903,10 @@
         <v>-0.3273571420905625</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.761606601153161</v>
+        <v>6.759074965934392</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.004093262280676413</v>
+        <v>0.006624897499445837</v>
       </c>
       <c r="AK524" t="n">
         <v>6.739235851443908</v>
@@ -85915,49 +85915,49 @@
         <v>0.02646401198992976</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.3951800081326278</v>
+        <v>-0.3951474775499479</v>
       </c>
       <c r="AN524" t="n">
-        <v>0.01994916658150125</v>
+        <v>0.01996181116265461</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.6590726151904053</v>
+        <v>0.6590699534979907</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.265943023774732</v>
+        <v>1.29204279075324</v>
       </c>
       <c r="AQ524" t="n">
         <v>76.80000000000001</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.004444447970427436</v>
+        <v>-0.004234709439972656</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7712</v>
       </c>
       <c r="AT524" t="n">
-        <v>-0.01460000000000061</v>
+        <v>-0.01379999999999981</v>
       </c>
       <c r="AU524" t="n">
-        <v>-0.01460000000000061</v>
+        <v>-0.01379999999999981</v>
       </c>
       <c r="AV524" t="n">
-        <v>-0.0154341287746206</v>
+        <v>-0.01539587569929477</v>
       </c>
       <c r="AW524" t="n">
-        <v>-0.01433729360326819</v>
+        <v>-0.01432454257815957</v>
       </c>
       <c r="AX524" t="n">
-        <v>0.01548935862423207</v>
+        <v>0.01548753487949774</v>
       </c>
       <c r="AY524" t="n">
-        <v>43.65079365079365</v>
+        <v>48.41269841269841</v>
       </c>
       <c r="AZ524" t="n">
-        <v>72.26777777777777</v>
+        <v>73.93444444444444</v>
       </c>
       <c r="BA524" t="n">
-        <v>74.72133333333333</v>
+        <v>75.02688888888889</v>
       </c>
     </row>
   </sheetData>
@@ -86194,7 +86194,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>101.51</t>
+          <t>101.38</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86284,7 +86284,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86299,7 +86299,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0199</t>
+          <t>0.0200</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-07-30 16:17 EDT
Score: 73/100
USD/CNY: 6.77
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.481</v>
       </c>
       <c r="R523" t="n">
-        <v>4.09</v>
+        <v>4.04</v>
       </c>
       <c r="S523" t="n">
-        <v>2.609</v>
+        <v>2.559</v>
       </c>
       <c r="T523" t="n">
-        <v>2.609</v>
+        <v>2.559</v>
       </c>
       <c r="U523" t="n">
         <v>-4.836845760641702</v>
@@ -85703,10 +85703,10 @@
         <v>-2.546151392384233</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.04128898433275463</v>
+        <v>-0.09001590863655373</v>
       </c>
       <c r="Y523" t="n">
-        <v>16.06425702811245</v>
+        <v>14.05622489959839</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>13.88888888888889</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.2593789843327476</v>
+        <v>-0.3081059086365467</v>
       </c>
       <c r="AG523" t="n">
         <v>7.098502730472051</v>
@@ -85811,16 +85811,16 @@
         <v>2.9511</v>
       </c>
       <c r="E524" t="n">
-        <v>6.770999908447266</v>
+        <v>6.76609992980957</v>
       </c>
       <c r="F524" t="n">
-        <v>6.747230052947998</v>
+        <v>6.747620105743408</v>
       </c>
       <c r="G524" t="n">
         <v>6.7413</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.02376985549926758</v>
+        <v>-0.01847982406616211</v>
       </c>
       <c r="I524" t="n">
         <v>100.8000030517578</v>
@@ -85850,28 +85850,28 @@
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>4.09</v>
+        <v>4.04</v>
       </c>
       <c r="S524" t="n">
-        <v>2.61</v>
+        <v>2.56</v>
       </c>
       <c r="T524" t="n">
-        <v>2.61</v>
+        <v>2.56</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.834102736870547</v>
+        <v>-4.910023114819662</v>
       </c>
       <c r="V524" t="n">
         <v>6.5742</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.906511757617136</v>
+        <v>-2.836197097298432</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.4153880885036765</v>
+        <v>-0.390779460029278</v>
       </c>
       <c r="Y524" t="n">
-        <v>4.819277108433734</v>
+        <v>5.220883534136546</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>14.28571428571428</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.634478088503676</v>
+        <v>-0.6098694600292776</v>
       </c>
       <c r="AG524" t="n">
         <v>7.098317000335017</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.3273170918877515</v>
+        <v>-0.3322170705254468</v>
       </c>
       <c r="AI524" t="n">
         <v>6.762721699397421</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.008278209049844776</v>
+        <v>0.003378230412149463</v>
       </c>
       <c r="AK524" t="n">
         <v>6.75259493782903</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.01840497061823587</v>
+        <v>0.01350499198054056</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3960001863323608</v>
@@ -85924,13 +85924,13 @@
         <v>0.6685846444009622</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.310927996341253</v>
+        <v>1.259843246390136</v>
       </c>
       <c r="AQ524" t="n">
-        <v>77.59999999999999</v>
+        <v>76</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.004395360887880053</v>
+        <v>-0.004365999690989386</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85954,10 +85954,10 @@
         <v>26.5625</v>
       </c>
       <c r="AZ524" t="n">
-        <v>66.246875</v>
+        <v>65.766875</v>
       </c>
       <c r="BA524" t="n">
-        <v>72.69105900023503</v>
+        <v>72.59505900023503</v>
       </c>
     </row>
   </sheetData>
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.61</t>
+          <t>2.56</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,7 +86234,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.42</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.63</t>
+          <t>-0.61</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86284,14 +86284,14 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
       <c r="AA2" t="inlineStr">
         <is>
           <t>-0.396</t>
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-08-03 16:28 EDT
Score: 71/100
USD/CNY: 6.76
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85355,13 +85355,13 @@
         <v>1.48</v>
       </c>
       <c r="R521" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="S521" t="n">
-        <v>2.56</v>
+        <v>2.6</v>
       </c>
       <c r="T521" t="n">
-        <v>2.56</v>
+        <v>2.6</v>
       </c>
       <c r="U521" t="n">
         <v>-4.742037037916409</v>
@@ -85373,7 +85373,7 @@
         <v>-2.315323638656408</v>
       </c>
       <c r="X521" t="n">
-        <v>0.1511372863418847</v>
+        <v>0.1902111568864218</v>
       </c>
       <c r="Y521" t="n">
         <v>20.48192771084337</v>
@@ -85399,7 +85399,7 @@
         <v>15.07936507936508</v>
       </c>
       <c r="AF521" t="n">
-        <v>-0.0725027136581291</v>
+        <v>-0.03342884311359207</v>
       </c>
       <c r="AG521" t="n">
         <v>7.075324721779002</v>
@@ -85484,13 +85484,13 @@
         <v>6.755000114440918</v>
       </c>
       <c r="F522" t="n">
-        <v>6.758049964904785</v>
+        <v>6.758170127868652</v>
       </c>
       <c r="G522" t="n">
         <v>6.7451</v>
       </c>
       <c r="H522" t="n">
-        <v>0.003049850463867188</v>
+        <v>0.003170013427734375</v>
       </c>
       <c r="I522" t="n">
         <v>99.80000305175781</v>
@@ -85520,13 +85520,13 @@
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="S522" t="n">
-        <v>2.56</v>
+        <v>2.6</v>
       </c>
       <c r="T522" t="n">
-        <v>2.56</v>
+        <v>2.6</v>
       </c>
       <c r="U522" t="n">
         <v>-4.824866533557659</v>
@@ -85538,10 +85538,10 @@
         <v>-2.691341396904845</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.2400715893397853</v>
+        <v>-0.2011481258985537</v>
       </c>
       <c r="Y522" t="n">
-        <v>8.032128514056225</v>
+        <v>8.835341365461847</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,7 +85564,7 @@
         <v>15.27777777777778</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.4637115893397992</v>
+        <v>-0.4247881258985675</v>
       </c>
       <c r="AG522" t="n">
         <v>7.080919854304359</v>
@@ -85889,12 +85889,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>4.08</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.56</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -85904,12 +85904,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85944,7 +85944,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.46</t>
+          <t>-0.42</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-08-04 12:47 EDT
Score: 68/100
USD/CNY: 6.75
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85649,13 +85649,13 @@
         <v>6.750899791717529</v>
       </c>
       <c r="F523" t="n">
-        <v>6.747200012207031</v>
+        <v>6.746940135955811</v>
       </c>
       <c r="G523" t="n">
         <v>6.7358</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.003699779510498047</v>
+        <v>-0.00395965576171875</v>
       </c>
       <c r="I523" t="n">
         <v>99.95999908447266</v>

</xml_diff>

<commit_message>
auto: data update 2026-08-07 10:45 EDT
Score: 74/100
USD/CNY: 6.75
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85658,10 +85658,10 @@
         <v>-0.001300069427490058</v>
       </c>
       <c r="I523" t="n">
-        <v>99.96600341796875</v>
+        <v>99.97000122070312</v>
       </c>
       <c r="J523" t="n">
-        <v>0.002768592334268627</v>
+        <v>0.002808694677898682</v>
       </c>
       <c r="K523" t="n">
         <v>2.9952</v>
@@ -85697,16 +85697,16 @@
         <v>-5.066364726372421</v>
       </c>
       <c r="V523" t="n">
-        <v>6.5711</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.646044529244373</v>
+        <v>-2.238619018227073</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2026801237729137</v>
+        <v>0.2211646353383889</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.835341365461847</v>
+        <v>22.08835341365462</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85717,10 +85717,10 @@
         <v>1.70364</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.6</v>
+        <v>1.60091</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.3</v>
+        <v>1.27879</v>
       </c>
       <c r="AD523" t="n">
         <v>0.2236400000000001</v>
@@ -85729,7 +85729,7 @@
         <v>15.47619047619047</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4263201237729275</v>
+        <v>-0.002475364661624901</v>
       </c>
       <c r="AG523" t="n">
         <v>7.091664492880899</v>
@@ -85738,10 +85738,10 @@
         <v>-0.3419644234534092</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.72489075280469</v>
+        <v>6.724989986752571</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.02480931662280028</v>
+        <v>0.02471008267491914</v>
       </c>
       <c r="AK523" t="n">
         <v>6.75925064743029</v>
@@ -85759,31 +85759,31 @@
         <v>0.7172988664983253</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.477057463073161</v>
+        <v>1.476029071691014</v>
       </c>
       <c r="AQ523" t="n">
         <v>76</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.002672567282273163</v>
+        <v>-0.002676225531211763</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.748150068385938</v>
+        <v>6.748149275802318</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.009350068385937327</v>
+        <v>-0.009349275802317258</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.009399999999999409</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01477242863187094</v>
+        <v>-0.01477238900268993</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01418294443912817</v>
+        <v>-0.01418293122940117</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01561145107407074</v>
+        <v>0.01561144909261169</v>
       </c>
       <c r="AY523" t="n">
         <v>65.87301587301587</v>
@@ -85805,7 +85805,7 @@
         <v>4.25</v>
       </c>
       <c r="C524" t="n">
-        <v>1.2548</v>
+        <v>1.2523</v>
       </c>
       <c r="D524" t="n">
         <v>2.9952</v>
@@ -85814,16 +85814,16 @@
         <v>6.74970006942749</v>
       </c>
       <c r="F524" t="n">
-        <v>6.7478</v>
+        <v>6.7434</v>
       </c>
       <c r="G524" t="n">
-        <v>6.743099999999999</v>
+        <v>6.734299999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.001900069427490436</v>
+        <v>-0.006300069427489952</v>
       </c>
       <c r="I524" t="n">
-        <v>99.96600341796875</v>
+        <v>99.97000122070312</v>
       </c>
       <c r="J524" t="n">
         <v>0</v>
@@ -85859,19 +85859,19 @@
         <v>2.55</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.98075992220646</v>
+        <v>-4.975575996904917</v>
       </c>
       <c r="V524" t="n">
-        <v>6.5711</v>
+        <v>6.5688</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.646044529244373</v>
+        <v>-2.680120117438545</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2026801237729137</v>
+        <v>-0.238128958171302</v>
       </c>
       <c r="Y524" t="n">
-        <v>9.036144578313253</v>
+        <v>8.032128514056225</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85882,10 +85882,10 @@
         <v>1.70364</v>
       </c>
       <c r="AB524" t="n">
-        <v>1.6</v>
+        <v>1.60091</v>
       </c>
       <c r="AC524" t="n">
-        <v>1.3</v>
+        <v>1.27879</v>
       </c>
       <c r="AD524" t="n">
         <v>0.2236400000000001</v>
@@ -85894,19 +85894,19 @@
         <v>15.67460317460317</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4263201237729275</v>
+        <v>-0.4617689581713158</v>
       </c>
       <c r="AG524" t="n">
-        <v>7.085886425354676</v>
+        <v>7.085536525944999</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.336186355927186</v>
+        <v>-0.3358364565175087</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.724422856194913</v>
+        <v>6.724522580384015</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.02527721323257737</v>
+        <v>0.02517748904347528</v>
       </c>
       <c r="AK524" t="n">
         <v>6.734775445902895</v>
@@ -85915,49 +85915,49 @@
         <v>0.01492462352459523</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.4022255514809761</v>
+        <v>-0.4022294042554291</v>
       </c>
       <c r="AN524" t="n">
-        <v>0.02545717031874362</v>
+        <v>0.02545790195722747</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.7273298677763016</v>
+        <v>0.7273309315128231</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.480458223051945</v>
+        <v>1.479438795429824</v>
       </c>
       <c r="AQ524" t="n">
         <v>78</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.00270628660431744</v>
+        <v>-0.002709964033465996</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7484</v>
       </c>
       <c r="AT524" t="n">
-        <v>-0.005300000000000971</v>
+        <v>-0.01410000000000089</v>
       </c>
       <c r="AU524" t="n">
-        <v>-0.005300000000000971</v>
+        <v>-0.01410000000000089</v>
       </c>
       <c r="AV524" t="n">
-        <v>-0.0134392728074074</v>
+        <v>-0.01387923317822639</v>
       </c>
       <c r="AW524" t="n">
-        <v>-0.01450049258921028</v>
+        <v>-0.01464714604614995</v>
       </c>
       <c r="AX524" t="n">
-        <v>0.01551196477937654</v>
+        <v>0.01553396081645844</v>
       </c>
       <c r="AY524" t="n">
-        <v>80.55555555555556</v>
+        <v>46.03174603174603</v>
       </c>
       <c r="AZ524" t="n">
-        <v>85.82444444444445</v>
+        <v>73.74111111111111</v>
       </c>
       <c r="BA524" t="n">
-        <v>76.74711111111111</v>
+        <v>74.33044444444445</v>
       </c>
     </row>
   </sheetData>
@@ -86174,12 +86174,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.75</t>
+          <t>6.74</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.74</t>
+          <t>6.73</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.20</t>
+          <t>-0.24</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86259,7 +86259,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.43</t>
+          <t>-0.46</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86344,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-08-10 11:51 EDT
Score: 62/100
USD/CNY: 6.75
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.748799800872803</v>
       </c>
       <c r="F522" t="n">
-        <v>6.745550155639648</v>
+        <v>6.745850086212158</v>
       </c>
       <c r="G522" t="n">
-        <v>6.7339</v>
+        <v>6.7336</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.003249645233154297</v>
+        <v>-0.002949714660644531</v>
       </c>
       <c r="I522" t="n">
         <v>99.59999847412109</v>
@@ -85606,28 +85606,28 @@
         <v>6.7778000831604</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.04390008316040017</v>
+        <v>-0.04420008316040036</v>
       </c>
       <c r="AU522" t="n">
-        <v>-0.04390008316040017</v>
+        <v>-0.04420008316040036</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.02723784725808111</v>
+        <v>-0.02725284725808113</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02272681965260244</v>
+        <v>-0.02273181965260244</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01159700812457607</v>
+        <v>0.01159775812457607</v>
       </c>
       <c r="AY522" t="n">
-        <v>18.30985915492958</v>
+        <v>16.90140845070422</v>
       </c>
       <c r="AZ522" t="n">
-        <v>60.43845070422535</v>
+        <v>59.94549295774648</v>
       </c>
       <c r="BA522" t="n">
-        <v>62.1355224880604</v>
+        <v>62.03693093876463</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: data update 2026-08-10 15:06 EDT
Score: 62/100
USD/CNY: 6.75
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.748799800872803</v>
       </c>
       <c r="F522" t="n">
-        <v>6.745850086212158</v>
+        <v>6.746560096740723</v>
       </c>
       <c r="G522" t="n">
-        <v>6.7336</v>
+        <v>6.733099999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.002949714660644531</v>
+        <v>-0.002239704132080078</v>
       </c>
       <c r="I522" t="n">
         <v>99.59999847412109</v>
@@ -85606,19 +85606,19 @@
         <v>6.7778000831604</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.04420008316040036</v>
+        <v>-0.04470008316040097</v>
       </c>
       <c r="AU522" t="n">
-        <v>-0.04420008316040036</v>
+        <v>-0.04470008316040097</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.02725284725808113</v>
+        <v>-0.02727784725808115</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02273181965260244</v>
+        <v>-0.02274015298593578</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01159775812457607</v>
+        <v>0.01159900812457607</v>
       </c>
       <c r="AY522" t="n">
         <v>16.90140845070422</v>

</xml_diff>

<commit_message>
auto: data update 2026-08-10 16:01 EDT
Score: 62/100
USD/CNY: 6.75
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.748799800872803</v>
       </c>
       <c r="F522" t="n">
-        <v>6.746560096740723</v>
+        <v>6.7463698387146</v>
       </c>
       <c r="G522" t="n">
         <v>6.733099999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.002239704132080078</v>
+        <v>-0.002429962158203125</v>
       </c>
       <c r="I522" t="n">
         <v>99.59999847412109</v>
@@ -85532,16 +85532,16 @@
         <v>-5.123330151365641</v>
       </c>
       <c r="V522" t="n">
-        <v>6.5647</v>
+        <v>6.5986</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.727889495981095</v>
+        <v>-2.225577959111746</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.2586418095179122</v>
+        <v>0.2640635757483301</v>
       </c>
       <c r="Y522" t="n">
-        <v>7.630522088353414</v>
+        <v>23.49397590361446</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,7 +85564,7 @@
         <v>13.69047619047619</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.4786418095179101</v>
+        <v>0.04406357574833208</v>
       </c>
       <c r="AG522" t="n">
         <v>7.094563095926223</v>
@@ -85899,17 +85899,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.56</t>
+          <t>6.60</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85944,7 +85944,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.48</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-08-17 14:50 EDT
Score: 61/100
USD/CNY: 6.74
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.742800235748291</v>
       </c>
       <c r="F522" t="n">
-        <v>6.740749835968018</v>
+        <v>6.743150234222412</v>
       </c>
       <c r="G522" t="n">
-        <v>6.728300000000001</v>
+        <v>6.7286</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.002050399780273438</v>
+        <v>0.0003499984741210938</v>
       </c>
       <c r="I522" t="n">
         <v>99.66999816894531</v>
@@ -85606,19 +85606,19 @@
         <v>6.7778000831604</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.04950008316039956</v>
+        <v>-0.04920008316040025</v>
       </c>
       <c r="AU522" t="n">
-        <v>-0.04950008316039956</v>
+        <v>-0.04920008316040025</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.03433778995864811</v>
+        <v>-0.03432278995864815</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02314630184459926</v>
+        <v>-0.02314130184459928</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01879992551607207</v>
+        <v>0.01879917551607207</v>
       </c>
       <c r="AY522" t="n">
         <v>13.1578947368421</v>

</xml_diff>

<commit_message>
auto: data update 2026-08-18 11:22 EDT
Score: 62/100
USD/CNY: 6.74
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -82358,10 +82358,10 @@
         <v>0.005300045013427734</v>
       </c>
       <c r="I503" t="n">
-        <v>101.1800003051758</v>
+        <v>100.9899978637695</v>
       </c>
       <c r="J503" t="n">
-        <v>0.001881398608033935</v>
+        <v>0</v>
       </c>
       <c r="K503" t="n">
         <v>2.9911</v>
@@ -82438,10 +82438,10 @@
         <v>-0.3271701475293147</v>
       </c>
       <c r="AI503" t="n">
-        <v>6.751667781721844</v>
+        <v>6.748378446675487</v>
       </c>
       <c r="AJ503" t="n">
-        <v>0.02083225642512865</v>
+        <v>0.02412159147148518</v>
       </c>
       <c r="AK503" t="n">
         <v>6.753855191419989</v>
@@ -82459,40 +82459,40 @@
         <v>0.6129676701055393</v>
       </c>
       <c r="AP503" t="n">
-        <v>1.471879255561614</v>
+        <v>1.506409891093108</v>
       </c>
       <c r="AQ503" t="n">
-        <v>79.63709677419355</v>
+        <v>80.24193548387098</v>
       </c>
       <c r="AR503" t="n">
-        <v>-0.006834851647461727</v>
+        <v>-0.007003369303381739</v>
       </c>
       <c r="AS503" t="n">
-        <v>6.777712926884361</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="AT503" t="n">
-        <v>-0.02271292688436155</v>
+        <v>-0.0228000831604005</v>
       </c>
       <c r="AU503" t="n">
         <v>-0.0228000831604005</v>
       </c>
       <c r="AV503" t="n">
-        <v>-0.003801761499381939</v>
+        <v>-0.003806119313183887</v>
       </c>
       <c r="AW503" t="n">
         <v/>
       </c>
       <c r="AX503" t="n">
-        <v>0.008409381195421756</v>
+        <v>0.008409599086111854</v>
       </c>
       <c r="AY503" t="n">
         <v>43.85964912280701</v>
       </c>
       <c r="AZ503" t="n">
-        <v>73.96200622524051</v>
+        <v>74.14345783814375</v>
       </c>
       <c r="BA503" t="n">
-        <v>73.06543549125743</v>
+        <v>73.10172581383809</v>
       </c>
     </row>
     <row r="504">
@@ -82523,10 +82523,10 @@
         <v>0.01219987869262695</v>
       </c>
       <c r="I504" t="n">
-        <v>101.1399993896484</v>
+        <v>100.9899978637695</v>
       </c>
       <c r="J504" t="n">
-        <v>-0.000395344093760519</v>
+        <v>0</v>
       </c>
       <c r="K504" t="n">
         <v>3.0451</v>
@@ -82603,10 +82603,10 @@
         <v>-0.3380039445079355</v>
       </c>
       <c r="AI504" t="n">
-        <v>6.729738669869288</v>
+        <v>6.727199502804298</v>
       </c>
       <c r="AJ504" t="n">
-        <v>0.03586153459848518</v>
+        <v>0.03840070166347509</v>
       </c>
       <c r="AK504" t="n">
         <v>6.736226026398153</v>
@@ -82615,40 +82615,40 @@
         <v>0.02937417806962017</v>
       </c>
       <c r="AM504" t="n">
-        <v>-0.3964908591695859</v>
+        <v>-0.3963830856482191</v>
       </c>
       <c r="AN504" t="n">
-        <v>0.01740130648959376</v>
+        <v>0.0173931510924123</v>
       </c>
       <c r="AO504" t="n">
-        <v>0.6198907013195262</v>
+        <v>0.6198612076146387</v>
       </c>
       <c r="AP504" t="n">
-        <v>1.619810543945891</v>
+        <v>1.645848973056612</v>
       </c>
       <c r="AQ504" t="n">
         <v>77.71084337349397</v>
       </c>
       <c r="AR504" t="n">
-        <v>-0.007224318615641342</v>
+        <v>-0.00750820718856422</v>
       </c>
       <c r="AS504" t="n">
-        <v>6.777819441178935</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="AT504" t="n">
-        <v>-0.01701944117893461</v>
+        <v>-0.0170000831603998</v>
       </c>
       <c r="AU504" t="n">
         <v>-0.0170000831603998</v>
       </c>
       <c r="AV504" t="n">
-        <v>-0.005718338506144782</v>
+        <v>-0.005721728419019989</v>
       </c>
       <c r="AW504" t="n">
         <v/>
       </c>
       <c r="AX504" t="n">
-        <v>0.007421070907737014</v>
+        <v>0.007421458294070871</v>
       </c>
       <c r="AY504" t="n">
         <v>53.44827586206896</v>
@@ -82657,7 +82657,7 @@
         <v>77.02014956377232</v>
       </c>
       <c r="BA504" t="n">
-        <v>74.58207041483776</v>
+        <v>74.6183607374184</v>
       </c>
     </row>
     <row r="505">
@@ -82691,7 +82691,7 @@
         <v>101.4300003051758</v>
       </c>
       <c r="J505" t="n">
-        <v>0.002867321705333437</v>
+        <v>0.004356891283429754</v>
       </c>
       <c r="K505" t="n">
         <v>3.1009</v>
@@ -82768,10 +82768,10 @@
         <v>-0.2945538086312354</v>
       </c>
       <c r="AI505" t="n">
-        <v>6.713320364291503</v>
+        <v>6.713441687447537</v>
       </c>
       <c r="AJ505" t="n">
-        <v>0.05917967385546952</v>
+        <v>0.05905835069943599</v>
       </c>
       <c r="AK505" t="n">
         <v>6.717723214958548</v>
@@ -82780,40 +82780,40 @@
         <v>0.05477682318842447</v>
       </c>
       <c r="AM505" t="n">
-        <v>-0.394760534481672</v>
+        <v>-0.3945367333325842</v>
       </c>
       <c r="AN505" t="n">
-        <v>0.01742962324324016</v>
+        <v>0.01740213766857585</v>
       </c>
       <c r="AO505" t="n">
-        <v>0.6272835381163622</v>
+        <v>0.6272161240534573</v>
       </c>
       <c r="AP505" t="n">
-        <v>1.850399549334671</v>
+        <v>1.848197986779916</v>
       </c>
       <c r="AQ505" t="n">
         <v>84</v>
       </c>
       <c r="AR505" t="n">
-        <v>-0.006140390830400942</v>
+        <v>-0.005732026124068678</v>
       </c>
       <c r="AS505" t="n">
-        <v>6.777680749986533</v>
+        <v>6.777630815637345</v>
       </c>
       <c r="AT505" t="n">
-        <v>-0.01178074998653234</v>
+        <v>-0.01173081563734524</v>
       </c>
       <c r="AU505" t="n">
         <v>-0.01190008316040014</v>
       </c>
       <c r="AV505" t="n">
-        <v>-0.006737737016154322</v>
+        <v>-0.006738630211570174</v>
       </c>
       <c r="AW505" t="n">
         <v/>
       </c>
       <c r="AX505" t="n">
-        <v>0.00666926220474588</v>
+        <v>0.00666969425085053</v>
       </c>
       <c r="AY505" t="n">
         <v>67.79661016949152</v>
@@ -82822,7 +82822,7 @@
         <v>83.92881355932204</v>
       </c>
       <c r="BA505" t="n">
-        <v>76.95804325519801</v>
+        <v>76.99433357777866</v>
       </c>
     </row>
     <row r="506">
@@ -82933,10 +82933,10 @@
         <v>-0.3026099231499435</v>
       </c>
       <c r="AI506" t="n">
-        <v>6.731179671396989</v>
+        <v>6.731291413833156</v>
       </c>
       <c r="AJ506" t="n">
-        <v>0.04132036674998396</v>
+        <v>0.04120862431381678</v>
       </c>
       <c r="AK506" t="n">
         <v>6.699415101064979</v>
@@ -82945,40 +82945,40 @@
         <v>0.07308493708199393</v>
       </c>
       <c r="AM506" t="n">
-        <v>-0.3930396958464927</v>
+        <v>-0.3928212926594107</v>
       </c>
       <c r="AN506" t="n">
-        <v>0.01766596732646103</v>
+        <v>0.0176401990086969</v>
       </c>
       <c r="AO506" t="n">
-        <v>0.6334129699358579</v>
+        <v>0.63334722370496</v>
       </c>
       <c r="AP506" t="n">
-        <v>1.659142843632353</v>
+        <v>1.65713401518142</v>
       </c>
       <c r="AQ506" t="n">
         <v>83.59999999999999</v>
       </c>
       <c r="AR506" t="n">
-        <v>-0.004023434406281946</v>
+        <v>-0.003614816218188609</v>
       </c>
       <c r="AS506" t="n">
-        <v>6.777789328686129</v>
+        <v>6.777790420905697</v>
       </c>
       <c r="AT506" t="n">
-        <v>-0.01858932868612939</v>
+        <v>-0.01859042090569751</v>
       </c>
       <c r="AU506" t="n">
         <v>-0.01860008316040052</v>
       </c>
       <c r="AV506" t="n">
-        <v>-0.008163438475363893</v>
+        <v>-0.008164386281758151</v>
       </c>
       <c r="AW506" t="n">
-        <v>-0.02279946196507197</v>
+        <v>-0.02279977790053673</v>
       </c>
       <c r="AX506" t="n">
-        <v>0.006200241951505226</v>
+        <v>0.006200721387929589</v>
       </c>
       <c r="AY506" t="n">
         <v>50</v>
@@ -82987,7 +82987,7 @@
         <v>77.44</v>
       </c>
       <c r="BA506" t="n">
-        <v>76.88451775630665</v>
+        <v>76.92080807888729</v>
       </c>
     </row>
     <row r="507">
@@ -83098,10 +83098,10 @@
         <v>-0.3108543589941197</v>
       </c>
       <c r="AI507" t="n">
-        <v>6.740946959621007</v>
+        <v>6.741058756412103</v>
       </c>
       <c r="AJ507" t="n">
-        <v>0.03085308157772371</v>
+        <v>0.03074128478662708</v>
       </c>
       <c r="AK507" t="n">
         <v>6.714685154719483</v>
@@ -83110,40 +83110,40 @@
         <v>0.05711488647924767</v>
       </c>
       <c r="AM507" t="n">
-        <v>-0.3929423394238508</v>
+        <v>-0.3927252921266378</v>
       </c>
       <c r="AN507" t="n">
-        <v>0.01842070378092631</v>
+        <v>0.01839707693354764</v>
       </c>
       <c r="AO507" t="n">
-        <v>0.640374511165978</v>
+        <v>0.6403084753775724</v>
       </c>
       <c r="AP507" t="n">
-        <v>1.546825022153</v>
+        <v>1.544874484275931</v>
       </c>
       <c r="AQ507" t="n">
         <v>81.8</v>
       </c>
       <c r="AR507" t="n">
-        <v>-0.00412996822745609</v>
+        <v>-0.003720442266642405</v>
       </c>
       <c r="AS507" t="n">
-        <v>6.777789048277441</v>
+        <v>6.777790142491924</v>
       </c>
       <c r="AT507" t="n">
-        <v>-0.02538904827744126</v>
+        <v>-0.02539014249192384</v>
       </c>
       <c r="AU507" t="n">
         <v>-0.02540008316040065</v>
       </c>
       <c r="AV507" t="n">
-        <v>-0.009803061862252615</v>
+        <v>-0.009804064379371003</v>
       </c>
       <c r="AW507" t="n">
-        <v>-0.02311277395463958</v>
+        <v>-0.02311310812701238</v>
       </c>
       <c r="AX507" t="n">
-        <v>0.00601692060483314</v>
+        <v>0.006017450167113423</v>
       </c>
       <c r="AY507" t="n">
         <v>40.98360655737705</v>
@@ -83152,7 +83152,7 @@
         <v>73.46426229508197</v>
       </c>
       <c r="BA507" t="n">
-        <v>77.16304632868336</v>
+        <v>77.19933665126402</v>
       </c>
     </row>
     <row r="508">
@@ -83263,10 +83263,10 @@
         <v>-0.3288542807561932</v>
       </c>
       <c r="AI508" t="n">
-        <v>6.7589577577717</v>
+        <v>6.759064466295768</v>
       </c>
       <c r="AJ508" t="n">
-        <v>0.006742105662137732</v>
+        <v>0.006635397138070154</v>
       </c>
       <c r="AK508" t="n">
         <v>6.722064699270507</v>
@@ -83275,40 +83275,40 @@
         <v>0.04363516416333102</v>
       </c>
       <c r="AM508" t="n">
-        <v>-0.3931401656438959</v>
+        <v>-0.3929227883143734</v>
       </c>
       <c r="AN508" t="n">
-        <v>0.01902711841846483</v>
+        <v>0.01900432654710715</v>
       </c>
       <c r="AO508" t="n">
-        <v>0.648485714148394</v>
+        <v>0.6484185000485352</v>
       </c>
       <c r="AP508" t="n">
-        <v>1.29314447754431</v>
+        <v>1.291348423746136</v>
       </c>
       <c r="AQ508" t="n">
         <v>76.40000000000001</v>
       </c>
       <c r="AR508" t="n">
-        <v>-0.003811905170718655</v>
+        <v>-0.003402651081290551</v>
       </c>
       <c r="AS508" t="n">
-        <v>6.77783317201014</v>
+        <v>6.77782961952222</v>
       </c>
       <c r="AT508" t="n">
-        <v>-0.02183317201013946</v>
+        <v>-0.02182961952221962</v>
       </c>
       <c r="AU508" t="n">
         <v>-0.02180008316040016</v>
       </c>
       <c r="AV508" t="n">
-        <v>-0.01075442019568116</v>
+        <v>-0.01075524508840355</v>
       </c>
       <c r="AW508" t="n">
-        <v>-0.02335865732252871</v>
+        <v>-0.02335893228676951</v>
       </c>
       <c r="AX508" t="n">
-        <v>0.006071829453409399</v>
+        <v>0.006072400260325801</v>
       </c>
       <c r="AY508" t="n">
         <v>43.54838709677419</v>
@@ -83428,10 +83428,10 @@
         <v>-0.3275028220247851</v>
       </c>
       <c r="AI509" t="n">
-        <v>6.763209774497792</v>
+        <v>6.763325216522089</v>
       </c>
       <c r="AJ509" t="n">
-        <v>0.007790133949473699</v>
+        <v>0.007674691925176447</v>
       </c>
       <c r="AK509" t="n">
         <v>6.739235851443908</v>
@@ -83440,40 +83440,40 @@
         <v>0.03176405700335749</v>
       </c>
       <c r="AM509" t="n">
-        <v>-0.3951733572725242</v>
+        <v>-0.394950414749964</v>
       </c>
       <c r="AN509" t="n">
-        <v>0.019963995720711</v>
+        <v>0.01994113462732905</v>
       </c>
       <c r="AO509" t="n">
-        <v>0.6590798145480943</v>
+        <v>0.6590084916407786</v>
       </c>
       <c r="AP509" t="n">
-        <v>1.304270996662537</v>
+        <v>1.302392211302197</v>
       </c>
       <c r="AQ509" t="n">
         <v>77.2</v>
       </c>
       <c r="AR509" t="n">
-        <v>-0.006169407306945165</v>
+        <v>-0.005757564598953703</v>
       </c>
       <c r="AS509" t="n">
-        <v>6.778039306514387</v>
+        <v>6.778023337007266</v>
       </c>
       <c r="AT509" t="n">
-        <v>-0.02063930651438639</v>
+        <v>-0.02062333700726526</v>
       </c>
       <c r="AU509" t="n">
         <v>-0.02040008316039987</v>
       </c>
       <c r="AV509" t="n">
-        <v>-0.01182772973946284</v>
+        <v>-0.01182775615682918</v>
       </c>
       <c r="AW509" t="n">
-        <v>-0.0231995169034272</v>
+        <v>-0.02319952570921598</v>
       </c>
       <c r="AX509" t="n">
-        <v>0.006185761652615558</v>
+        <v>0.006186333780400277</v>
       </c>
       <c r="AY509" t="n">
         <v>49.2063492063492</v>
@@ -83593,10 +83593,10 @@
         <v>-0.3308550871256273</v>
       </c>
       <c r="AI510" t="n">
-        <v>6.740243824085885</v>
+        <v>6.740382201199143</v>
       </c>
       <c r="AJ510" t="n">
-        <v>0.02585610572368502</v>
+        <v>0.02571772861042732</v>
       </c>
       <c r="AK510" t="n">
         <v>6.75259493782903</v>
@@ -83605,40 +83605,40 @@
         <v>0.01350499198054056</v>
       </c>
       <c r="AM510" t="n">
-        <v>-0.3960001863323608</v>
+        <v>-0.3957745806072295</v>
       </c>
       <c r="AN510" t="n">
-        <v>0.02043272610569408</v>
+        <v>0.0204092996144366</v>
       </c>
       <c r="AO510" t="n">
-        <v>0.6685846444009622</v>
+        <v>0.6685102590632164</v>
       </c>
       <c r="AP510" t="n">
-        <v>1.493832689756023</v>
+        <v>1.491667939420019</v>
       </c>
       <c r="AQ510" t="n">
         <v>79</v>
       </c>
       <c r="AR510" t="n">
-        <v>-0.00293773457574891</v>
+        <v>-0.002540174468858687</v>
       </c>
       <c r="AS510" t="n">
-        <v>6.7779561348082</v>
+        <v>6.777935016525326</v>
       </c>
       <c r="AT510" t="n">
-        <v>-0.03665613480819996</v>
+        <v>-0.03663501652532641</v>
       </c>
       <c r="AU510" t="n">
         <v>-0.03650008316040054</v>
       </c>
       <c r="AV510" t="n">
-        <v>-0.01341447857522717</v>
+        <v>-0.01341344907844983</v>
       </c>
       <c r="AW510" t="n">
-        <v>-0.02317664240037365</v>
+        <v>-0.0231762992347812</v>
       </c>
       <c r="AX510" t="n">
-        <v>0.0064044437523467</v>
+        <v>0.006404964405292553</v>
       </c>
       <c r="AY510" t="n">
         <v>26.5625</v>
@@ -83678,10 +83678,10 @@
         <v>0.02279996871948242</v>
       </c>
       <c r="I511" t="n">
-        <v>99.80000305175781</v>
+        <v>100.0100021362305</v>
       </c>
       <c r="J511" t="n">
-        <v>-0.002099780821788189</v>
+        <v>0</v>
       </c>
       <c r="K511" t="n">
         <v>3.0194</v>
@@ -83758,10 +83758,10 @@
         <v>-0.3203246073380841</v>
       </c>
       <c r="AI511" t="n">
-        <v>6.714622134232894</v>
+        <v>6.719227909990969</v>
       </c>
       <c r="AJ511" t="n">
-        <v>0.04037798020802441</v>
+        <v>0.03577220444994911</v>
       </c>
       <c r="AK511" t="n">
         <v>6.746779913842831</v>
@@ -83770,49 +83770,49 @@
         <v>0.008220200598087146</v>
       </c>
       <c r="AM511" t="n">
-        <v>-0.396740905361911</v>
+        <v>-0.3965158172760009</v>
       </c>
       <c r="AN511" t="n">
-        <v>0.02120763540003751</v>
+        <v>0.02118581013855175</v>
       </c>
       <c r="AO511" t="n">
-        <v>0.6777865296786982</v>
+        <v>0.6777101403370329</v>
       </c>
       <c r="AP511" t="n">
-        <v>1.643209728592377</v>
+        <v>1.594761412423886</v>
       </c>
       <c r="AQ511" t="n">
-        <v>81.59999999999999</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="AR511" t="n">
-        <v>-0.002865452421907258</v>
+        <v>-0.003502047583293221</v>
       </c>
       <c r="AS511" t="n">
-        <v>6.777840863977332</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="AT511" t="n">
-        <v>-0.03564086397733135</v>
+        <v>-0.03560008316039998</v>
       </c>
       <c r="AU511" t="n">
         <v>-0.03560008316039998</v>
       </c>
       <c r="AV511" t="n">
-        <v>-0.0147665176160737</v>
+        <v>-0.0147634490784498</v>
       </c>
       <c r="AW511" t="n">
-        <v>-0.02309349928808775</v>
+        <v>-0.02309247644221311</v>
       </c>
       <c r="AX511" t="n">
-        <v>0.006674615339027361</v>
+        <v>0.006674982565092018</v>
       </c>
       <c r="AY511" t="n">
         <v>29.23076923076923</v>
       </c>
       <c r="AZ511" t="n">
-        <v>69.15076923076923</v>
+        <v>69.09076923076923</v>
       </c>
       <c r="BA511" t="n">
-        <v>71.15921284638887</v>
+        <v>71.14721284638887</v>
       </c>
     </row>
     <row r="512">
@@ -83846,7 +83846,7 @@
         <v>99.95999908447266</v>
       </c>
       <c r="J512" t="n">
-        <v>0.00160316661144666</v>
+        <v>-0.0004999805088464759</v>
       </c>
       <c r="K512" t="n">
         <v>2.9854</v>
@@ -83923,10 +83923,10 @@
         <v>-0.3340959985244947</v>
       </c>
       <c r="AI512" t="n">
-        <v>6.731570059394423</v>
+        <v>6.731608564083782</v>
       </c>
       <c r="AJ512" t="n">
-        <v>0.01932973232310609</v>
+        <v>0.01929122763374735</v>
       </c>
       <c r="AK512" t="n">
         <v>6.728823425344638</v>
@@ -83935,40 +83935,40 @@
         <v>0.02207636637289134</v>
       </c>
       <c r="AM512" t="n">
-        <v>-0.3968575339788111</v>
+        <v>-0.3968707490690719</v>
       </c>
       <c r="AN512" t="n">
-        <v>0.0220082962170377</v>
+        <v>0.02204310237142126</v>
       </c>
       <c r="AO512" t="n">
-        <v>0.6856993240123035</v>
+        <v>0.6856948527327844</v>
       </c>
       <c r="AP512" t="n">
-        <v>1.420026821077208</v>
+        <v>1.419585320459278</v>
       </c>
       <c r="AQ512" t="n">
         <v>77.39999999999999</v>
       </c>
       <c r="AR512" t="n">
-        <v>-0.002577229375292126</v>
+        <v>-0.002947463179424533</v>
       </c>
       <c r="AS512" t="n">
-        <v>6.777772079133445</v>
+        <v>6.777810071429111</v>
       </c>
       <c r="AT512" t="n">
-        <v>-0.03267207913344539</v>
+        <v>-0.03271007142911131</v>
       </c>
       <c r="AU512" t="n">
         <v>-0.03270008316040052</v>
       </c>
       <c r="AV512" t="n">
-        <v>-0.01668951675446277</v>
+        <v>-0.01668834783162216</v>
       </c>
       <c r="AW512" t="n">
-        <v>-0.02286406628403812</v>
+        <v>-0.02286367664309125</v>
       </c>
       <c r="AX512" t="n">
-        <v>0.007071727664475771</v>
+        <v>0.007072036444398397</v>
       </c>
       <c r="AY512" t="n">
         <v>33.33333333333333</v>
@@ -83977,7 +83977,7 @@
         <v>68.62666666666667</v>
       </c>
       <c r="BA512" t="n">
-        <v>70.19169372070581</v>
+        <v>70.17969372070581</v>
       </c>
     </row>
     <row r="513">
@@ -84088,10 +84088,10 @@
         <v>-0.3456268937433125</v>
       </c>
       <c r="AI513" t="n">
-        <v>6.748064561399866</v>
+        <v>6.748101272412299</v>
       </c>
       <c r="AJ513" t="n">
-        <v>0.004235224214148126</v>
+        <v>0.004198513201714604</v>
       </c>
       <c r="AK513" t="n">
         <v>6.740096815166266</v>
@@ -84100,40 +84100,40 @@
         <v>0.01220297044774732</v>
       </c>
       <c r="AM513" t="n">
-        <v>-0.3976889317784199</v>
+        <v>-0.3977059644204096</v>
       </c>
       <c r="AN513" t="n">
-        <v>0.02268190844878654</v>
+        <v>0.02271888896632723</v>
       </c>
       <c r="AO513" t="n">
-        <v>0.6953567146475523</v>
+        <v>0.6953537478383294</v>
       </c>
       <c r="AP513" t="n">
-        <v>1.261868708113399</v>
+        <v>1.261451878023444</v>
       </c>
       <c r="AQ513" t="n">
         <v>72</v>
       </c>
       <c r="AR513" t="n">
-        <v>-0.001295276208961911</v>
+        <v>-0.001667844427570213</v>
       </c>
       <c r="AS513" t="n">
-        <v>6.777806230979031</v>
+        <v>6.777807999313707</v>
       </c>
       <c r="AT513" t="n">
-        <v>-0.04200623097903033</v>
+        <v>-0.04200799931370636</v>
       </c>
       <c r="AU513" t="n">
         <v>-0.04200008316040016</v>
       </c>
       <c r="AV513" t="n">
-        <v>-0.01909048262999868</v>
+        <v>-0.01908940212389187</v>
       </c>
       <c r="AW513" t="n">
-        <v>-0.0228285450426347</v>
+        <v>-0.02282818487393242</v>
       </c>
       <c r="AX513" t="n">
-        <v>0.007648168013300609</v>
+        <v>0.007648422767917895</v>
       </c>
       <c r="AY513" t="n">
         <v>20.8955223880597</v>
@@ -84142,7 +84142,7 @@
         <v>61.39343283582089</v>
       </c>
       <c r="BA513" t="n">
-        <v>68.03399319109579</v>
+        <v>68.02199319109579</v>
       </c>
     </row>
     <row r="514">
@@ -84253,10 +84253,10 @@
         <v>-0.3468885181379404</v>
       </c>
       <c r="AI514" t="n">
-        <v>6.747226278872152</v>
+        <v>6.747255722628349</v>
       </c>
       <c r="AJ514" t="n">
-        <v>0.005973775296548745</v>
+        <v>0.00594433154035201</v>
       </c>
       <c r="AK514" t="n">
         <v>6.755554272205931</v>
@@ -84265,40 +84265,40 @@
         <v>-0.002354218037229572</v>
       </c>
       <c r="AM514" t="n">
-        <v>-0.4003515275861345</v>
+        <v>-0.400375027138847</v>
       </c>
       <c r="AN514" t="n">
-        <v>0.02398656672240618</v>
+        <v>0.02402774236102168</v>
       </c>
       <c r="AO514" t="n">
-        <v>0.7067969646460921</v>
+        <v>0.7067971474351272</v>
       </c>
       <c r="AP514" t="n">
-        <v>1.280599476642095</v>
+        <v>1.280261960188511</v>
       </c>
       <c r="AQ514" t="n">
         <v>72</v>
       </c>
       <c r="AR514" t="n">
-        <v>-0.00219780480132725</v>
+        <v>-0.002571042581132642</v>
       </c>
       <c r="AS514" t="n">
-        <v>6.777829908076522</v>
+        <v>6.777834973032914</v>
       </c>
       <c r="AT514" t="n">
-        <v>-0.04082990807652198</v>
+        <v>-0.04083497303291406</v>
       </c>
       <c r="AU514" t="n">
         <v>-0.04080008316040029</v>
       </c>
       <c r="AV514" t="n">
-        <v>-0.02186674294078301</v>
+        <v>-0.02186591568249581</v>
       </c>
       <c r="AW514" t="n">
-        <v>-0.02266077772864999</v>
+        <v>-0.02266050197588759</v>
       </c>
       <c r="AX514" t="n">
-        <v>0.008435519684562156</v>
+        <v>0.008435733076265082</v>
       </c>
       <c r="AY514" t="n">
         <v>23.52941176470588</v>
@@ -84307,7 +84307,7 @@
         <v>61.89529411764705</v>
       </c>
       <c r="BA514" t="n">
-        <v>65.58860757018076</v>
+        <v>65.57660757018077</v>
       </c>
     </row>
     <row r="515">
@@ -84418,10 +84418,10 @@
         <v>-0.3419644234534092</v>
       </c>
       <c r="AI515" t="n">
-        <v>6.724989986752571</v>
+        <v>6.725029661829083</v>
       </c>
       <c r="AJ515" t="n">
-        <v>0.02471008267491914</v>
+        <v>0.024670407598407</v>
       </c>
       <c r="AK515" t="n">
         <v>6.75925064743029</v>
@@ -84430,40 +84430,40 @@
         <v>-0.009550578002800236</v>
       </c>
       <c r="AM515" t="n">
-        <v>-0.4017887258056133</v>
+        <v>-0.4018162797423327</v>
       </c>
       <c r="AN515" t="n">
-        <v>0.02482212216928553</v>
+        <v>0.02486590604389916</v>
       </c>
       <c r="AO515" t="n">
-        <v>0.7172988664983253</v>
+        <v>0.7173010872263644</v>
       </c>
       <c r="AP515" t="n">
-        <v>1.476029071691014</v>
+        <v>1.475588032504229</v>
       </c>
       <c r="AQ515" t="n">
         <v>76</v>
       </c>
       <c r="AR515" t="n">
-        <v>-0.002676225531211754</v>
+        <v>-0.003048533390401407</v>
       </c>
       <c r="AS515" t="n">
-        <v>6.777749136467762</v>
+        <v>6.777742048928296</v>
       </c>
       <c r="AT515" t="n">
-        <v>-0.03894913646776121</v>
+        <v>-0.03894204892829567</v>
       </c>
       <c r="AU515" t="n">
         <v>-0.03900008316040005</v>
       </c>
       <c r="AV515" t="n">
-        <v>-0.02398247898892603</v>
+        <v>-0.02398129735366554</v>
       </c>
       <c r="AW515" t="n">
-        <v>-0.02242578646761387</v>
+        <v>-0.02242539258919371</v>
       </c>
       <c r="AX515" t="n">
-        <v>0.009368919371520569</v>
+        <v>0.009369073681460472</v>
       </c>
       <c r="AY515" t="n">
         <v>26.08695652173913</v>
@@ -84472,7 +84472,7 @@
         <v>66.23043478260868</v>
       </c>
       <c r="BA515" t="n">
-        <v>65.4593195267025</v>
+        <v>65.4473195267025</v>
       </c>
     </row>
     <row r="516">
@@ -84583,10 +84583,10 @@
         <v>-0.3448997849091837</v>
       </c>
       <c r="AI516" t="n">
-        <v>6.738231277482312</v>
+        <v>6.738255595412468</v>
       </c>
       <c r="AJ516" t="n">
-        <v>0.01056852339049108</v>
+        <v>0.01054420546033441</v>
       </c>
       <c r="AK516" t="n">
         <v>6.734775445902895</v>
@@ -84595,40 +84595,40 @@
         <v>0.01402435496990773</v>
       </c>
       <c r="AM516" t="n">
-        <v>-0.4022294042554291</v>
+        <v>-0.4022609316376698</v>
       </c>
       <c r="AN516" t="n">
-        <v>0.02545790195722747</v>
+        <v>0.02550387683415684</v>
       </c>
       <c r="AO516" t="n">
-        <v>0.7273309315128231</v>
+        <v>0.7273351886096061</v>
       </c>
       <c r="AP516" t="n">
-        <v>1.327950493923702</v>
+        <v>1.327674329276297</v>
       </c>
       <c r="AQ516" t="n">
         <v>73.40000000000001</v>
       </c>
       <c r="AR516" t="n">
-        <v>-0.002838978063890906</v>
+        <v>-0.003209446091365256</v>
       </c>
       <c r="AS516" t="n">
-        <v>6.777871300548548</v>
+        <v>6.777880593950862</v>
       </c>
       <c r="AT516" t="n">
-        <v>-0.04367130054854851</v>
+        <v>-0.04368059395086288</v>
       </c>
       <c r="AU516" t="n">
         <v>-0.04360008316040087</v>
       </c>
       <c r="AV516" t="n">
-        <v>-0.02549787898685798</v>
+        <v>-0.02549716202171321</v>
       </c>
       <c r="AW516" t="n">
-        <v>-0.02268459250841133</v>
+        <v>-0.02268435352002974</v>
       </c>
       <c r="AX516" t="n">
-        <v>0.01040961982719224</v>
+        <v>0.0104097382888749</v>
       </c>
       <c r="AY516" t="n">
         <v>18.57142857142857</v>
@@ -84748,10 +84748,10 @@
         <v>-0.3389992354304407</v>
       </c>
       <c r="AI517" t="n">
-        <v>6.718201282169581</v>
+        <v>6.718233131673284</v>
       </c>
       <c r="AJ517" t="n">
-        <v>0.02919852480673768</v>
+        <v>0.02916667530303485</v>
       </c>
       <c r="AK517" t="n">
         <v>6.753996132599221</v>
@@ -84760,40 +84760,40 @@
         <v>-0.00659632562290291</v>
       </c>
       <c r="AM517" t="n">
-        <v>-0.4027953816469058</v>
+        <v>-0.4028302582145923</v>
       </c>
       <c r="AN517" t="n">
-        <v>0.02608258444417638</v>
+        <v>0.02613064267520054</v>
       </c>
       <c r="AO517" t="n">
-        <v>0.736674421029931</v>
+        <v>0.736680621170787</v>
       </c>
       <c r="AP517" t="n">
-        <v>1.519755165509982</v>
+        <v>1.519404100140539</v>
       </c>
       <c r="AQ517" t="n">
         <v>77.40000000000001</v>
       </c>
       <c r="AR517" t="n">
-        <v>-0.001943929707255045</v>
+        <v>-0.002316067232288261</v>
       </c>
       <c r="AS517" t="n">
-        <v>6.77777230347129</v>
+        <v>6.777766985447334</v>
       </c>
       <c r="AT517" t="n">
-        <v>-0.04467230347129014</v>
+        <v>-0.04466698544733472</v>
       </c>
       <c r="AU517" t="n">
         <v>-0.04470008316040097</v>
       </c>
       <c r="AV517" t="n">
-        <v>-0.02727645827362562</v>
+        <v>-0.02727547540728308</v>
       </c>
       <c r="AW517" t="n">
-        <v>-0.02273968999111727</v>
+        <v>-0.02273936236900309</v>
       </c>
       <c r="AX517" t="n">
-        <v>0.01159893867535329</v>
+        <v>0.01159900799371883</v>
       </c>
       <c r="AY517" t="n">
         <v>16.90140845070422</v>
@@ -84913,10 +84913,10 @@
         <v>-0.3329117502755388</v>
       </c>
       <c r="AI518" t="n">
-        <v>6.730898772467414</v>
+        <v>6.730931854936179</v>
       </c>
       <c r="AJ518" t="n">
-        <v>0.01650103450890406</v>
+        <v>0.01646795204013962</v>
       </c>
       <c r="AK518" t="n">
         <v>6.732394407262716</v>
@@ -84925,40 +84925,40 @@
         <v>0.01500539971360215</v>
       </c>
       <c r="AM518" t="n">
-        <v>-0.4025099007694142</v>
+        <v>-0.4025465822999924</v>
       </c>
       <c r="AN518" t="n">
-        <v>0.02634377330607651</v>
+        <v>0.02639266239094257</v>
       </c>
       <c r="AO518" t="n">
-        <v>0.746561519528266</v>
+        <v>0.7465684054287068</v>
       </c>
       <c r="AP518" t="n">
-        <v>1.38684795374353</v>
+        <v>1.38648834307159</v>
       </c>
       <c r="AQ518" t="n">
         <v>78</v>
       </c>
       <c r="AR518" t="n">
-        <v>0.000782692516168381</v>
+        <v>0.0003987308428205903</v>
       </c>
       <c r="AS518" t="n">
-        <v>6.77780061477715</v>
+        <v>6.777800353984499</v>
       </c>
       <c r="AT518" t="n">
-        <v>-0.04510061477715066</v>
+        <v>-0.04510035398449919</v>
       </c>
       <c r="AU518" t="n">
         <v>-0.04510008316040093</v>
       </c>
       <c r="AV518" t="n">
-        <v>-0.02849946927270004</v>
+        <v>-0.02849847336672493</v>
       </c>
       <c r="AW518" t="n">
-        <v>-0.02305884356186635</v>
+        <v>-0.02305851159320798</v>
       </c>
       <c r="AX518" t="n">
-        <v>0.012880871846816</v>
+        <v>0.01288089136988278</v>
       </c>
       <c r="AY518" t="n">
         <v>16.66666666666666</v>
@@ -85078,10 +85078,10 @@
         <v>-0.3335936335657701</v>
       </c>
       <c r="AI519" t="n">
-        <v>6.740580458294252</v>
+        <v>6.740623868728166</v>
       </c>
       <c r="AJ519" t="n">
-        <v>0.004419427264830134</v>
+        <v>0.00437601683091593</v>
       </c>
       <c r="AK519" t="n">
         <v>6.74318350621926</v>
@@ -85090,40 +85090,40 @@
         <v>0.001816379339821594</v>
       </c>
       <c r="AM519" t="n">
-        <v>-0.4034224290251451</v>
+        <v>-0.4034654226643876</v>
       </c>
       <c r="AN519" t="n">
-        <v>0.02736182786837871</v>
+        <v>0.02741459853506639</v>
       </c>
       <c r="AO519" t="n">
-        <v>0.755189863471066</v>
+        <v>0.7552010609216553</v>
       </c>
       <c r="AP519" t="n">
-        <v>1.259334239690847</v>
+        <v>1.258871370070383</v>
       </c>
       <c r="AQ519" t="n">
         <v>76.2</v>
       </c>
       <c r="AR519" t="n">
-        <v>0.004684779010825856</v>
+        <v>0.004293437255601792</v>
       </c>
       <c r="AS519" t="n">
-        <v>6.777860522468127</v>
+        <v>6.777855473686805</v>
       </c>
       <c r="AT519" t="n">
-        <v>-0.04576052246812701</v>
+        <v>-0.0457554736868051</v>
       </c>
       <c r="AU519" t="n">
         <v>-0.04570008316040042</v>
       </c>
       <c r="AV519" t="n">
-        <v>-0.02970460186976949</v>
+        <v>-0.02970335352472828</v>
       </c>
       <c r="AW519" t="n">
-        <v>-0.02310338986639821</v>
+        <v>-0.02310297375138447</v>
       </c>
       <c r="AX519" t="n">
-        <v>0.0142431734036299</v>
+        <v>0.01424313050944462</v>
       </c>
       <c r="AY519" t="n">
         <v>15.06849315068493</v>
@@ -85243,10 +85243,10 @@
         <v>-0.3086955151355042</v>
       </c>
       <c r="AI520" t="n">
-        <v>6.755708466794879</v>
+        <v>6.755750978622371</v>
       </c>
       <c r="AJ520" t="n">
-        <v>-0.01240850570479068</v>
+        <v>-0.01245101753228273</v>
       </c>
       <c r="AK520" t="n">
         <v>6.746865899087779</v>
@@ -85255,40 +85255,40 @@
         <v>-0.003565937997691115</v>
       </c>
       <c r="AM520" t="n">
-        <v>-0.4037073020769307</v>
+        <v>-0.4037527699419104</v>
       </c>
       <c r="AN520" t="n">
-        <v>0.02778289906564352</v>
+        <v>0.02783693810207571</v>
       </c>
       <c r="AO520" t="n">
-        <v>0.7638221248099442</v>
+        <v>0.7638345477935677</v>
       </c>
       <c r="AP520" t="n">
-        <v>1.083564796528327</v>
+        <v>1.083114808402871</v>
       </c>
       <c r="AQ520" t="n">
         <v>78.40000000000001</v>
       </c>
       <c r="AR520" t="n">
-        <v>0.003077728100043848</v>
+        <v>0.002685989934888374</v>
       </c>
       <c r="AS520" t="n">
-        <v>6.777789653454104</v>
+        <v>6.777790980963837</v>
       </c>
       <c r="AT520" t="n">
-        <v>-0.04588965345410401</v>
+        <v>-0.04589098096383637</v>
       </c>
       <c r="AU520" t="n">
         <v>-0.04590008316039995</v>
       </c>
       <c r="AV520" t="n">
-        <v>-0.03115096944061424</v>
+        <v>-0.03114978747105965</v>
       </c>
       <c r="AW520" t="n">
-        <v>-0.02326937677105021</v>
+        <v>-0.02326898278119868</v>
       </c>
       <c r="AX520" t="n">
-        <v>0.01568332077718871</v>
+        <v>0.0156832187845257</v>
       </c>
       <c r="AY520" t="n">
         <v>14.86486486486486</v>
@@ -85316,7 +85316,7 @@
         <v>2.9405</v>
       </c>
       <c r="E521" t="n">
-        <v>6.742800235748291</v>
+        <v>6.743299961090088</v>
       </c>
       <c r="F521" t="n">
         <v>6.7778000831604</v>
@@ -85325,7 +85325,7 @@
         <v>6.7303</v>
       </c>
       <c r="H521" t="n">
-        <v>0.03499984741210938</v>
+        <v>0.0345001220703125</v>
       </c>
       <c r="I521" t="n">
         <v>99.66999816894531</v>
@@ -85364,16 +85364,16 @@
         <v>2.5</v>
       </c>
       <c r="U521" t="n">
-        <v>-4.515716039204559</v>
+        <v>-4.507970699056233</v>
       </c>
       <c r="V521" t="n">
         <v>6.5986</v>
       </c>
       <c r="W521" t="n">
-        <v>-2.138580867097095</v>
+        <v>-2.145833077647874</v>
       </c>
       <c r="X521" t="n">
-        <v>0.2763036143924591</v>
+        <v>0.2687627658617631</v>
       </c>
       <c r="Y521" t="n">
         <v>25.30120481927711</v>
@@ -85399,61 +85399,61 @@
         <v>14.68253968253968</v>
       </c>
       <c r="AF521" t="n">
-        <v>0.05357361439244368</v>
+        <v>0.04603276586174765</v>
       </c>
       <c r="AG521" t="n">
         <v>7.047285947485499</v>
       </c>
       <c r="AH521" t="n">
-        <v>-0.3044857117372084</v>
+        <v>-0.3039859863954115</v>
       </c>
       <c r="AI521" t="n">
-        <v>6.73601646973098</v>
+        <v>6.736041496771461</v>
       </c>
       <c r="AJ521" t="n">
-        <v>0.006783766017311343</v>
+        <v>0.007258464318627311</v>
       </c>
       <c r="AK521" t="n">
         <v>6.761018647414997</v>
       </c>
       <c r="AL521" t="n">
-        <v>-0.01821841166670612</v>
+        <v>-0.01771868632490925</v>
       </c>
       <c r="AM521" t="n">
-        <v>-0.403510818895136</v>
+        <v>-0.4035582267671979</v>
       </c>
       <c r="AN521" t="n">
-        <v>0.02805871830419215</v>
+        <v>0.02811368720091384</v>
       </c>
       <c r="AO521" t="n">
-        <v>0.7683919203573231</v>
+        <v>0.7684053332209008</v>
       </c>
       <c r="AP521" t="n">
-        <v>1.283500676883962</v>
+        <v>1.288416370968192</v>
       </c>
       <c r="AQ521" t="n">
         <v>82.80000000000001</v>
       </c>
       <c r="AR521" t="n">
-        <v>0.002903283150327665</v>
+        <v>0.002431371003544746</v>
       </c>
       <c r="AS521" t="n">
-        <v>6.777742994313127</v>
+        <v>6.777752273780226</v>
       </c>
       <c r="AT521" t="n">
-        <v>-0.04744299431312715</v>
+        <v>-0.04745227378022676</v>
       </c>
       <c r="AU521" t="n">
         <v>-0.04750008316040066</v>
       </c>
       <c r="AV521" t="n">
-        <v>-0.03291463771931293</v>
+        <v>-0.03291391972311333</v>
       </c>
       <c r="AW521" t="n">
-        <v>-0.02330463141409799</v>
+        <v>-0.02330439208203145</v>
       </c>
       <c r="AX521" t="n">
-        <v>0.01721397770073558</v>
+        <v>0.01721383980826259</v>
       </c>
       <c r="AY521" t="n">
         <v>13.33333333333333</v>
@@ -85541,7 +85541,7 @@
         <v>0.2763036143924591</v>
       </c>
       <c r="Y522" t="n">
-        <v>25.50200803212851</v>
+        <v>25.70281124497992</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85573,34 +85573,34 @@
         <v>-0.3058180386269767</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.727923556873627</v>
+        <v>6.727955014350026</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.01487667887466415</v>
+        <v>0.01484522139826527</v>
       </c>
       <c r="AK522" t="n">
-        <v>6.751365564447465</v>
+        <v>6.751372427531023</v>
       </c>
       <c r="AL522" t="n">
-        <v>-0.008565328699174479</v>
+        <v>-0.008572191782731942</v>
       </c>
       <c r="AM522" t="n">
-        <v>-0.4027898636641267</v>
+        <v>-0.4028270972655147</v>
       </c>
       <c r="AN522" t="n">
-        <v>0.02827333203020888</v>
+        <v>0.0283278572240776</v>
       </c>
       <c r="AO522" t="n">
-        <v>0.7726830480787004</v>
+        <v>0.7726869743648852</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.365892657990883</v>
+        <v>1.365509052937986</v>
       </c>
       <c r="AQ522" t="n">
         <v>83.39999999999999</v>
       </c>
       <c r="AR522" t="n">
-        <v>0.003522400618796758</v>
+        <v>0.00304882715731455</v>
       </c>
       <c r="AS522" t="n">
         <v>6.7778000831604</v>
@@ -85612,13 +85612,13 @@
         <v>-0.04920008316040025</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.03432278995864815</v>
+        <v>-0.03432207196244854</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02314130184459928</v>
+        <v>-0.02314106251253274</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01879917551607207</v>
+        <v>0.0187990017237891</v>
       </c>
       <c r="AY522" t="n">
         <v>13.1578947368421</v>
@@ -85649,13 +85649,13 @@
         <v>6.742800235748291</v>
       </c>
       <c r="F523" t="n">
-        <v>6.744699954986572</v>
+        <v>6.74616003036499</v>
       </c>
       <c r="G523" t="n">
         <v>6.730499999999999</v>
       </c>
       <c r="H523" t="n">
-        <v>0.00189971923828125</v>
+        <v>0.003359794616699219</v>
       </c>
       <c r="I523" t="n">
         <v>99.66999816894531</v>
@@ -85738,34 +85738,34 @@
         <v>-0.3032508750781648</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.727698234813079</v>
+        <v>6.727728945732101</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.01510200093521163</v>
+        <v>0.01507129001618956</v>
       </c>
       <c r="AK523" t="n">
-        <v>6.744478107428201</v>
+        <v>6.744485049262728</v>
       </c>
       <c r="AL523" t="n">
-        <v>-0.001677871679909515</v>
+        <v>-0.001684813514437167</v>
       </c>
       <c r="AM523" t="n">
-        <v>-0.4028170403434749</v>
+        <v>-0.402858790327591</v>
       </c>
       <c r="AN523" t="n">
-        <v>0.02891960956825251</v>
+        <v>0.02897682112008632</v>
       </c>
       <c r="AO523" t="n">
-        <v>0.7784413872609752</v>
+        <v>0.7784489548245479</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.366007036968715</v>
+        <v>1.365635379155592</v>
       </c>
       <c r="AQ523" t="n">
         <v>84.19999999999999</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.003558293359634741</v>
+        <v>0.003084674106516256</v>
       </c>
       <c r="AS523" t="n">
         <v>6.7778000831604</v>
@@ -85777,13 +85777,13 @@
         <v>-0.04730008316040113</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.03555214777245012</v>
+        <v>-0.03554707196244857</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.02300357439650629</v>
+        <v>-0.02300333506443975</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.02038669482972548</v>
+        <v>0.02038604935625233</v>
       </c>
       <c r="AY523" t="n">
         <v>15.58441558441558</v>
@@ -86009,7 +86009,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.74</t>
+          <t>6.75</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -86134,7 +86134,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0289</t>
+          <t>0.0290</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -86149,7 +86149,7 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-08-19 10:22 EDT
Score: 70/100
USD/CNY: 6.74
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85520,13 +85520,13 @@
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>3.98</v>
+        <v>4</v>
       </c>
       <c r="S522" t="n">
-        <v>2.5</v>
+        <v>2.52</v>
       </c>
       <c r="T522" t="n">
-        <v>2.5</v>
+        <v>2.52</v>
       </c>
       <c r="U522" t="n">
         <v>-4.535475291194625</v>
@@ -85538,10 +85538,10 @@
         <v>-2.138580867097095</v>
       </c>
       <c r="X522" t="n">
-        <v>0.2763036143924591</v>
+        <v>0.2958758982190224</v>
       </c>
       <c r="Y522" t="n">
-        <v>25.50200803212851</v>
+        <v>25.70281124497992</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,7 +85564,7 @@
         <v>12.8968253968254</v>
       </c>
       <c r="AF522" t="n">
-        <v>0.0553936143924405</v>
+        <v>0.07496589821900379</v>
       </c>
       <c r="AG522" t="n">
         <v>7.048618274375268</v>
@@ -85643,70 +85643,70 @@
         <v>1.2262</v>
       </c>
       <c r="D523" t="n">
-        <v>2.960500000000001</v>
+        <v>2.9638</v>
       </c>
       <c r="E523" t="n">
-        <v>6.742800235748291</v>
+        <v>6.7399001121521</v>
       </c>
       <c r="F523" t="n">
-        <v>6.7468</v>
+        <v>6.7469</v>
       </c>
       <c r="G523" t="n">
         <v>6.732</v>
       </c>
       <c r="H523" t="n">
-        <v>0.003999764251709337</v>
+        <v>0.00699988784790051</v>
       </c>
       <c r="I523" t="n">
-        <v>99.63999938964844</v>
+        <v>99.65000152587891</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>0.0001003827407841662</v>
       </c>
       <c r="K523" t="n">
-        <v>2.960500000000001</v>
+        <v>2.9638</v>
       </c>
       <c r="L523" t="n">
-        <v>2.98268</v>
+        <v>2.982845</v>
       </c>
       <c r="M523" t="n">
-        <v>2.91146</v>
+        <v>2.911515000000001</v>
       </c>
       <c r="N523" t="n">
-        <v>2.726869166666666</v>
+        <v>2.726896666666667</v>
       </c>
       <c r="O523" t="n">
-        <v>93.80000000000001</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="P523" t="n">
-        <v>89.32135728542914</v>
+        <v>89.62075848303394</v>
       </c>
       <c r="Q523" t="n">
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>3.98</v>
+        <v>4</v>
       </c>
       <c r="S523" t="n">
-        <v>2.5</v>
+        <v>2.52</v>
       </c>
       <c r="T523" t="n">
-        <v>2.5</v>
+        <v>2.52</v>
       </c>
       <c r="U523" t="n">
-        <v>-4.497402629109791</v>
+        <v>-4.542367002180986</v>
       </c>
       <c r="V523" t="n">
-        <v>6.5643</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.647271600928292</v>
+        <v>-2.096471903156749</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2526330106452201</v>
+        <v>0.3396692207169982</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.032128514056225</v>
+        <v>26.50602409638554</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85714,40 +85714,40 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.70091</v>
+        <v>1.7</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.61576</v>
+        <v>1.61485</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.36833</v>
+        <v>1.43303</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.2209099999999999</v>
+        <v>0.22</v>
       </c>
       <c r="AE523" t="n">
-        <v>13.09523809523809</v>
+        <v>12.1031746031746</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4735430106452387</v>
+        <v>0.1196692207170003</v>
       </c>
       <c r="AG523" t="n">
         <v>7.046051110826456</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.3032508750781648</v>
+        <v>-0.3061509986743562</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.726846144701057</v>
+        <v>6.725806144687715</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.01595409104723444</v>
+        <v>0.01409396746438496</v>
       </c>
       <c r="AK523" t="n">
         <v>6.744478107428201</v>
       </c>
       <c r="AL523" t="n">
-        <v>-0.001677871679909515</v>
+        <v>-0.004577995276100921</v>
       </c>
       <c r="AM523" t="n">
         <v>-0.4027900432658338</v>
@@ -85759,40 +85759,205 @@
         <v>0.7784357006627721</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.374707959641946</v>
+        <v>1.355489422378677</v>
       </c>
       <c r="AQ523" t="n">
-        <v>84.19999999999999</v>
+        <v>83</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.00353191995001628</v>
+        <v>0.00353753124109526</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7434</v>
+        <v>6.743402394629094</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.01140000000000008</v>
+        <v>-0.01140239462909332</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.01140000000000008</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.0131366710590993</v>
+        <v>-0.01313679079055396</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01432215093025739</v>
+        <v>-0.01432219084074228</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01466385461871044</v>
+        <v>0.01466386060528318</v>
       </c>
       <c r="AY523" t="n">
         <v>60.31746031746032</v>
       </c>
       <c r="AZ523" t="n">
-        <v>79.20111111111112</v>
+        <v>79.05111111111111</v>
       </c>
       <c r="BA523" t="n">
-        <v>72.51466666666667</v>
+        <v>72.48466666666667</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2249</v>
+      </c>
+      <c r="D524" t="n">
+        <v>2.9638</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.7399001121521</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.7299</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.7184</v>
+      </c>
+      <c r="H524" t="n">
+        <v>-0.01000011215209984</v>
+      </c>
+      <c r="I524" t="n">
+        <v>99.65000152587891</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>2.9638</v>
+      </c>
+      <c r="L524" t="n">
+        <v>2.97878</v>
+      </c>
+      <c r="M524" t="n">
+        <v>2.914875</v>
+      </c>
+      <c r="N524" t="n">
+        <v>2.733219166666667</v>
+      </c>
+      <c r="O524" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="P524" t="n">
+        <v>89.52095808383234</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="R524" t="n">
+        <v>4</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-4.219257999202846</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.5594</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-2.678082896609346</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.2652062124737009</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>7.228915662650603</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.61485</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.43303</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>12.3015873015873</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.4852062124736989</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>7.024273886772359</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.284373774620259</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.725613783886462</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>0.01428632826563803</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.743301592583855</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>-0.003401480431755033</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.402742697458547</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>0.02955568036482276</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.7839391318357882</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>1.353055656586767</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>85</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>0.003442048402022131</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.7469</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>-0.02850000000000019</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>-0.02850000000000019</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.01415582416059991</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.01450495964819917</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.01453047925975846</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>6.746031746031746</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>60.83111111111111</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>70.47111111111111</v>
       </c>
     </row>
   </sheetData>
@@ -85999,7 +86164,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86009,12 +86174,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.75</t>
+          <t>6.73</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.73</t>
+          <t>6.72</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -86024,12 +86189,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.64</t>
+          <t>99.65</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86044,7 +86209,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>90</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86054,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.98</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.52</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86069,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86089,12 +86254,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86104,22 +86269,22 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.47</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86134,44 +86299,44 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0289</t>
+          <t>0.0296</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.778</t>
+          <t>0.784</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.7434</t>
+          <t>6.7469</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
           <t>-0.01</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
-      </c>
       <c r="AJ2" t="inlineStr">
         <is>
           <t>0.01</t>
@@ -86179,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>70</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-08-20 14:50 EDT
Score: 62/100
USD/CNY: 6.74
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -82193,10 +82193,10 @@
         <v>0.005300045013427734</v>
       </c>
       <c r="I502" t="n">
-        <v>100.9899978637695</v>
+        <v>101.1800003051758</v>
       </c>
       <c r="J502" t="n">
-        <v>0</v>
+        <v>0.001881398608033935</v>
       </c>
       <c r="K502" t="n">
         <v>2.9911</v>
@@ -82273,10 +82273,10 @@
         <v>-0.3271701475293147</v>
       </c>
       <c r="AI502" t="n">
-        <v>6.748378446675487</v>
+        <v>6.751667781721844</v>
       </c>
       <c r="AJ502" t="n">
-        <v>0.02412159147148518</v>
+        <v>0.02083225642512865</v>
       </c>
       <c r="AK502" t="n">
         <v>6.753855191419989</v>
@@ -82294,40 +82294,40 @@
         <v>0.6129676701055393</v>
       </c>
       <c r="AP502" t="n">
-        <v>1.516238046243956</v>
+        <v>1.481626746283946</v>
       </c>
       <c r="AQ502" t="n">
-        <v>80.36437246963563</v>
+        <v>79.95951417004048</v>
       </c>
       <c r="AR502" t="n">
-        <v>-0.007003369303381745</v>
+        <v>-0.006834851647461734</v>
       </c>
       <c r="AS502" t="n">
-        <v>6.7778000831604</v>
+        <v>6.777712926884361</v>
       </c>
       <c r="AT502" t="n">
-        <v>-0.0228000831604005</v>
+        <v>-0.02271292688436155</v>
       </c>
       <c r="AU502" t="n">
         <v>-0.0228000831604005</v>
       </c>
       <c r="AV502" t="n">
-        <v>-0.003806119313183887</v>
+        <v>-0.003801761499381939</v>
       </c>
       <c r="AW502" t="n">
         <v/>
       </c>
       <c r="AX502" t="n">
-        <v>0.008409599086111854</v>
+        <v>0.008409381195421756</v>
       </c>
       <c r="AY502" t="n">
         <v>43.85964912280701</v>
       </c>
       <c r="AZ502" t="n">
-        <v>74.18018893387314</v>
+        <v>74.05873144399459</v>
       </c>
       <c r="BA502" t="n">
-        <v>73.17838659582718</v>
+        <v>73.15409509785147</v>
       </c>
     </row>
     <row r="503">
@@ -82358,10 +82358,10 @@
         <v>0.01219987869262695</v>
       </c>
       <c r="I503" t="n">
-        <v>100.9899978637695</v>
+        <v>101.1399993896484</v>
       </c>
       <c r="J503" t="n">
-        <v>0</v>
+        <v>-0.000395344093760519</v>
       </c>
       <c r="K503" t="n">
         <v>3.0451</v>
@@ -82438,10 +82438,10 @@
         <v>-0.3380039445079355</v>
       </c>
       <c r="AI503" t="n">
-        <v>6.727199502804298</v>
+        <v>6.729738669869288</v>
       </c>
       <c r="AJ503" t="n">
-        <v>0.03840070166347509</v>
+        <v>0.03586153459848518</v>
       </c>
       <c r="AK503" t="n">
         <v>6.736226026398153</v>
@@ -82450,40 +82450,40 @@
         <v>0.02937417806962017</v>
       </c>
       <c r="AM503" t="n">
-        <v>-0.3963830856482191</v>
+        <v>-0.3964908591695859</v>
       </c>
       <c r="AN503" t="n">
-        <v>0.0173931510924123</v>
+        <v>0.01740130648959376</v>
       </c>
       <c r="AO503" t="n">
-        <v>0.6198612076146387</v>
+        <v>0.6198907013195262</v>
       </c>
       <c r="AP503" t="n">
-        <v>1.655818986435509</v>
+        <v>1.629728716463947</v>
       </c>
       <c r="AQ503" t="n">
         <v>77.82258064516128</v>
       </c>
       <c r="AR503" t="n">
-        <v>-0.007508207188564227</v>
+        <v>-0.007224318615641348</v>
       </c>
       <c r="AS503" t="n">
-        <v>6.7778000831604</v>
+        <v>6.777819441178935</v>
       </c>
       <c r="AT503" t="n">
-        <v>-0.0170000831603998</v>
+        <v>-0.01701944117893461</v>
       </c>
       <c r="AU503" t="n">
         <v>-0.0170000831603998</v>
       </c>
       <c r="AV503" t="n">
-        <v>-0.005721728419019989</v>
+        <v>-0.005718338506144782</v>
       </c>
       <c r="AW503" t="n">
         <v/>
       </c>
       <c r="AX503" t="n">
-        <v>0.007421458294070871</v>
+        <v>0.007421070907737014</v>
       </c>
       <c r="AY503" t="n">
         <v>53.44827586206896</v>
@@ -82492,7 +82492,7 @@
         <v>77.05367074527251</v>
       </c>
       <c r="BA503" t="n">
-        <v>74.68432037218193</v>
+        <v>74.66002887420622</v>
       </c>
     </row>
     <row r="504">
@@ -82526,7 +82526,7 @@
         <v>101.4300003051758</v>
       </c>
       <c r="J504" t="n">
-        <v>0.004356891283429754</v>
+        <v>0.002867321705333437</v>
       </c>
       <c r="K504" t="n">
         <v>3.1009</v>
@@ -82603,10 +82603,10 @@
         <v>-0.2945538086312354</v>
       </c>
       <c r="AI504" t="n">
-        <v>6.713441687447537</v>
+        <v>6.713320364291503</v>
       </c>
       <c r="AJ504" t="n">
-        <v>0.05905835069943599</v>
+        <v>0.05917967385546952</v>
       </c>
       <c r="AK504" t="n">
         <v>6.717723214958548</v>
@@ -82615,40 +82615,40 @@
         <v>0.05477682318842447</v>
       </c>
       <c r="AM504" t="n">
-        <v>-0.3945367333325842</v>
+        <v>-0.394760534481672</v>
       </c>
       <c r="AN504" t="n">
-        <v>0.01740213766857585</v>
+        <v>0.01742962324324016</v>
       </c>
       <c r="AO504" t="n">
-        <v>0.6272161240534573</v>
+        <v>0.6272835381163622</v>
       </c>
       <c r="AP504" t="n">
-        <v>1.858394344516194</v>
+        <v>1.860612816686509</v>
       </c>
       <c r="AQ504" t="n">
         <v>84.13654618473896</v>
       </c>
       <c r="AR504" t="n">
-        <v>-0.005732026124068684</v>
+        <v>-0.006140390830400948</v>
       </c>
       <c r="AS504" t="n">
-        <v>6.777630815637345</v>
+        <v>6.777680749986533</v>
       </c>
       <c r="AT504" t="n">
-        <v>-0.01173081563734524</v>
+        <v>-0.01178074998653234</v>
       </c>
       <c r="AU504" t="n">
         <v>-0.01190008316040014</v>
       </c>
       <c r="AV504" t="n">
-        <v>-0.006738630211570174</v>
+        <v>-0.006737737016154322</v>
       </c>
       <c r="AW504" t="n">
         <v/>
       </c>
       <c r="AX504" t="n">
-        <v>0.00666969425085053</v>
+        <v>0.00666926220474588</v>
       </c>
       <c r="AY504" t="n">
         <v>67.79661016949152</v>
@@ -82657,7 +82657,7 @@
         <v>83.9697774147437</v>
       </c>
       <c r="BA504" t="n">
-        <v>77.05157397292058</v>
+        <v>77.02728247494488</v>
       </c>
     </row>
     <row r="505">
@@ -82768,10 +82768,10 @@
         <v>-0.3026099231499435</v>
       </c>
       <c r="AI505" t="n">
-        <v>6.731291413833156</v>
+        <v>6.731179671396989</v>
       </c>
       <c r="AJ505" t="n">
-        <v>0.04120862431381678</v>
+        <v>0.04132036674998396</v>
       </c>
       <c r="AK505" t="n">
         <v>6.699415101064979</v>
@@ -82780,40 +82780,40 @@
         <v>0.07308493708199393</v>
       </c>
       <c r="AM505" t="n">
-        <v>-0.3928212926594107</v>
+        <v>-0.3930396958464927</v>
       </c>
       <c r="AN505" t="n">
-        <v>0.0176401990086969</v>
+        <v>0.01766596732646103</v>
       </c>
       <c r="AO505" t="n">
-        <v>0.63334722370496</v>
+        <v>0.6334129699358579</v>
       </c>
       <c r="AP505" t="n">
-        <v>1.65713401518142</v>
+        <v>1.659142843632353</v>
       </c>
       <c r="AQ505" t="n">
         <v>83.59999999999999</v>
       </c>
       <c r="AR505" t="n">
-        <v>-0.003614816218188613</v>
+        <v>-0.00402343440628195</v>
       </c>
       <c r="AS505" t="n">
-        <v>6.777790420905697</v>
+        <v>6.777789328686129</v>
       </c>
       <c r="AT505" t="n">
-        <v>-0.01859042090569751</v>
+        <v>-0.01858932868612939</v>
       </c>
       <c r="AU505" t="n">
         <v>-0.01860008316040052</v>
       </c>
       <c r="AV505" t="n">
-        <v>-0.008164386281758151</v>
+        <v>-0.008163438475363893</v>
       </c>
       <c r="AW505" t="n">
-        <v>-0.02279977790053673</v>
+        <v>-0.02279946196507197</v>
       </c>
       <c r="AX505" t="n">
-        <v>0.006200721387929589</v>
+        <v>0.006200241951505226</v>
       </c>
       <c r="AY505" t="n">
         <v>50</v>
@@ -82822,7 +82822,7 @@
         <v>77.44</v>
       </c>
       <c r="BA505" t="n">
-        <v>76.96077619926567</v>
+        <v>76.93648470128997</v>
       </c>
     </row>
     <row r="506">
@@ -82933,10 +82933,10 @@
         <v>-0.3108543589941197</v>
       </c>
       <c r="AI506" t="n">
-        <v>6.741058756412103</v>
+        <v>6.740946959621007</v>
       </c>
       <c r="AJ506" t="n">
-        <v>0.03074128478662708</v>
+        <v>0.03085308157772371</v>
       </c>
       <c r="AK506" t="n">
         <v>6.714685154719483</v>
@@ -82945,40 +82945,40 @@
         <v>0.05711488647924767</v>
       </c>
       <c r="AM506" t="n">
-        <v>-0.3927252921266378</v>
+        <v>-0.3929423394238508</v>
       </c>
       <c r="AN506" t="n">
-        <v>0.01839707693354764</v>
+        <v>0.01842070378092631</v>
       </c>
       <c r="AO506" t="n">
-        <v>0.6403084753775724</v>
+        <v>0.640374511165978</v>
       </c>
       <c r="AP506" t="n">
-        <v>1.544874484275931</v>
+        <v>1.546825022153</v>
       </c>
       <c r="AQ506" t="n">
         <v>81.8</v>
       </c>
       <c r="AR506" t="n">
-        <v>-0.00372044226664241</v>
+        <v>-0.004129968227456095</v>
       </c>
       <c r="AS506" t="n">
-        <v>6.777790142491924</v>
+        <v>6.777789048277441</v>
       </c>
       <c r="AT506" t="n">
-        <v>-0.02539014249192384</v>
+        <v>-0.02538904827744126</v>
       </c>
       <c r="AU506" t="n">
         <v>-0.02540008316040065</v>
       </c>
       <c r="AV506" t="n">
-        <v>-0.009804064379371003</v>
+        <v>-0.009803061862252615</v>
       </c>
       <c r="AW506" t="n">
-        <v>-0.02311310812701238</v>
+        <v>-0.02311277395463958</v>
       </c>
       <c r="AX506" t="n">
-        <v>0.006017450167113423</v>
+        <v>0.00601692060483314</v>
       </c>
       <c r="AY506" t="n">
         <v>40.98360655737705</v>
@@ -82987,7 +82987,7 @@
         <v>73.46426229508197</v>
       </c>
       <c r="BA506" t="n">
-        <v>77.22157987779426</v>
+        <v>77.19728837981856</v>
       </c>
     </row>
     <row r="507">
@@ -83098,10 +83098,10 @@
         <v>-0.3288542807561932</v>
       </c>
       <c r="AI507" t="n">
-        <v>6.759064466295768</v>
+        <v>6.7589577577717</v>
       </c>
       <c r="AJ507" t="n">
-        <v>0.006635397138070154</v>
+        <v>0.006742105662137732</v>
       </c>
       <c r="AK507" t="n">
         <v>6.722064699270507</v>
@@ -83110,40 +83110,40 @@
         <v>0.04363516416333102</v>
       </c>
       <c r="AM507" t="n">
-        <v>-0.3929227883143734</v>
+        <v>-0.3931401656438959</v>
       </c>
       <c r="AN507" t="n">
-        <v>0.01900432654710715</v>
+        <v>0.01902711841846483</v>
       </c>
       <c r="AO507" t="n">
-        <v>0.6484185000485352</v>
+        <v>0.648485714148394</v>
       </c>
       <c r="AP507" t="n">
-        <v>1.291348423746136</v>
+        <v>1.29314447754431</v>
       </c>
       <c r="AQ507" t="n">
         <v>76.40000000000001</v>
       </c>
       <c r="AR507" t="n">
-        <v>-0.003402651081290555</v>
+        <v>-0.00381190517071866</v>
       </c>
       <c r="AS507" t="n">
-        <v>6.77782961952222</v>
+        <v>6.77783317201014</v>
       </c>
       <c r="AT507" t="n">
-        <v>-0.02182961952221962</v>
+        <v>-0.02183317201013946</v>
       </c>
       <c r="AU507" t="n">
         <v>-0.02180008316040016</v>
       </c>
       <c r="AV507" t="n">
-        <v>-0.01075524508840355</v>
+        <v>-0.01075442019568116</v>
       </c>
       <c r="AW507" t="n">
-        <v>-0.02335893228676951</v>
+        <v>-0.02335865732252871</v>
       </c>
       <c r="AX507" t="n">
-        <v>0.006072400260325801</v>
+        <v>0.006071829453409399</v>
       </c>
       <c r="AY507" t="n">
         <v>43.54838709677419</v>
@@ -83263,10 +83263,10 @@
         <v>-0.3275028220247851</v>
       </c>
       <c r="AI508" t="n">
-        <v>6.763325216522089</v>
+        <v>6.763209774497792</v>
       </c>
       <c r="AJ508" t="n">
-        <v>0.007674691925176447</v>
+        <v>0.007790133949473699</v>
       </c>
       <c r="AK508" t="n">
         <v>6.739235851443908</v>
@@ -83275,40 +83275,40 @@
         <v>0.03176405700335749</v>
       </c>
       <c r="AM508" t="n">
-        <v>-0.394950414749964</v>
+        <v>-0.3951733572725242</v>
       </c>
       <c r="AN508" t="n">
-        <v>0.01994113462732905</v>
+        <v>0.019963995720711</v>
       </c>
       <c r="AO508" t="n">
-        <v>0.6590084916407786</v>
+        <v>0.6590798145480943</v>
       </c>
       <c r="AP508" t="n">
-        <v>1.302392211302197</v>
+        <v>1.304270996662537</v>
       </c>
       <c r="AQ508" t="n">
         <v>77.2</v>
       </c>
       <c r="AR508" t="n">
-        <v>-0.005757564598953709</v>
+        <v>-0.006169407306945171</v>
       </c>
       <c r="AS508" t="n">
-        <v>6.778023337007266</v>
+        <v>6.778039306514387</v>
       </c>
       <c r="AT508" t="n">
-        <v>-0.02062333700726526</v>
+        <v>-0.02063930651438639</v>
       </c>
       <c r="AU508" t="n">
         <v>-0.02040008316039987</v>
       </c>
       <c r="AV508" t="n">
-        <v>-0.01182775615682918</v>
+        <v>-0.01182772973946284</v>
       </c>
       <c r="AW508" t="n">
-        <v>-0.02319952570921598</v>
+        <v>-0.0231995169034272</v>
       </c>
       <c r="AX508" t="n">
-        <v>0.006186333780400277</v>
+        <v>0.006185761652615558</v>
       </c>
       <c r="AY508" t="n">
         <v>49.2063492063492</v>
@@ -83317,7 +83317,7 @@
         <v>74.12222222222222</v>
       </c>
       <c r="BA508" t="n">
-        <v>76.23563948318377</v>
+        <v>76.23563948318376</v>
       </c>
     </row>
     <row r="509">
@@ -83428,10 +83428,10 @@
         <v>-0.3308550871256273</v>
       </c>
       <c r="AI509" t="n">
-        <v>6.740382201199143</v>
+        <v>6.740243824085885</v>
       </c>
       <c r="AJ509" t="n">
-        <v>0.02571772861042732</v>
+        <v>0.02585610572368502</v>
       </c>
       <c r="AK509" t="n">
         <v>6.75259493782903</v>
@@ -83440,40 +83440,40 @@
         <v>0.01350499198054056</v>
       </c>
       <c r="AM509" t="n">
-        <v>-0.3957745806072295</v>
+        <v>-0.3960001863323608</v>
       </c>
       <c r="AN509" t="n">
-        <v>0.0204092996144366</v>
+        <v>0.02043272610569408</v>
       </c>
       <c r="AO509" t="n">
-        <v>0.6685102590632164</v>
+        <v>0.6685846444009622</v>
       </c>
       <c r="AP509" t="n">
-        <v>1.491667939420019</v>
+        <v>1.493832689756023</v>
       </c>
       <c r="AQ509" t="n">
         <v>79</v>
       </c>
       <c r="AR509" t="n">
-        <v>-0.002540174468858691</v>
+        <v>-0.002937734575748914</v>
       </c>
       <c r="AS509" t="n">
-        <v>6.777935016525326</v>
+        <v>6.7779561348082</v>
       </c>
       <c r="AT509" t="n">
-        <v>-0.03663501652532641</v>
+        <v>-0.03665613480819996</v>
       </c>
       <c r="AU509" t="n">
         <v>-0.03650008316040054</v>
       </c>
       <c r="AV509" t="n">
-        <v>-0.01341344907844983</v>
+        <v>-0.01341447857522717</v>
       </c>
       <c r="AW509" t="n">
-        <v>-0.0231762992347812</v>
+        <v>-0.02317664240037365</v>
       </c>
       <c r="AX509" t="n">
-        <v>0.006404964405292553</v>
+        <v>0.0064044437523467</v>
       </c>
       <c r="AY509" t="n">
         <v>26.5625</v>
@@ -83513,10 +83513,10 @@
         <v>0.02279996871948242</v>
       </c>
       <c r="I510" t="n">
-        <v>100.0100021362305</v>
+        <v>99.80000305175781</v>
       </c>
       <c r="J510" t="n">
-        <v>0</v>
+        <v>-0.002099780821788189</v>
       </c>
       <c r="K510" t="n">
         <v>3.0194</v>
@@ -83593,10 +83593,10 @@
         <v>-0.3203246073380841</v>
       </c>
       <c r="AI510" t="n">
-        <v>6.719227909990969</v>
+        <v>6.714622134232894</v>
       </c>
       <c r="AJ510" t="n">
-        <v>0.03577220444994911</v>
+        <v>0.04037798020802441</v>
       </c>
       <c r="AK510" t="n">
         <v>6.746779913842831</v>
@@ -83605,49 +83605,49 @@
         <v>0.008220200598087146</v>
       </c>
       <c r="AM510" t="n">
-        <v>-0.3965158172760009</v>
+        <v>-0.396740905361911</v>
       </c>
       <c r="AN510" t="n">
-        <v>0.02118581013855175</v>
+        <v>0.02120763540003751</v>
       </c>
       <c r="AO510" t="n">
-        <v>0.6777101403370329</v>
+        <v>0.6777865296786982</v>
       </c>
       <c r="AP510" t="n">
-        <v>1.594761412423886</v>
+        <v>1.643209728592377</v>
       </c>
       <c r="AQ510" t="n">
-        <v>81.40000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="AR510" t="n">
-        <v>-0.003502047583293226</v>
+        <v>-0.002865452421907262</v>
       </c>
       <c r="AS510" t="n">
-        <v>6.7778000831604</v>
+        <v>6.777840863977332</v>
       </c>
       <c r="AT510" t="n">
-        <v>-0.03560008316039998</v>
+        <v>-0.03564086397733135</v>
       </c>
       <c r="AU510" t="n">
         <v>-0.03560008316039998</v>
       </c>
       <c r="AV510" t="n">
-        <v>-0.0147634490784498</v>
+        <v>-0.0147665176160737</v>
       </c>
       <c r="AW510" t="n">
-        <v>-0.02309247644221311</v>
+        <v>-0.02309349928808775</v>
       </c>
       <c r="AX510" t="n">
-        <v>0.006674982565092018</v>
+        <v>0.006674615339027361</v>
       </c>
       <c r="AY510" t="n">
         <v>29.23076923076923</v>
       </c>
       <c r="AZ510" t="n">
-        <v>69.09076923076923</v>
+        <v>69.15076923076923</v>
       </c>
       <c r="BA510" t="n">
-        <v>71.14721284638888</v>
+        <v>71.15921284638887</v>
       </c>
     </row>
     <row r="511">
@@ -83681,7 +83681,7 @@
         <v>99.95999908447266</v>
       </c>
       <c r="J511" t="n">
-        <v>-0.0004999805088464759</v>
+        <v>0.00160316661144666</v>
       </c>
       <c r="K511" t="n">
         <v>2.9854</v>
@@ -83758,10 +83758,10 @@
         <v>-0.3340959985244947</v>
       </c>
       <c r="AI511" t="n">
-        <v>6.731608564083782</v>
+        <v>6.731570059394423</v>
       </c>
       <c r="AJ511" t="n">
-        <v>0.01929122763374735</v>
+        <v>0.01932973232310609</v>
       </c>
       <c r="AK511" t="n">
         <v>6.728823425344638</v>
@@ -83770,40 +83770,40 @@
         <v>0.02207636637289134</v>
       </c>
       <c r="AM511" t="n">
-        <v>-0.3968707490690719</v>
+        <v>-0.3968575339788111</v>
       </c>
       <c r="AN511" t="n">
-        <v>0.02204310237142126</v>
+        <v>0.0220082962170377</v>
       </c>
       <c r="AO511" t="n">
-        <v>0.6856948527327844</v>
+        <v>0.6856993240123035</v>
       </c>
       <c r="AP511" t="n">
-        <v>1.419585320459278</v>
+        <v>1.420026821077208</v>
       </c>
       <c r="AQ511" t="n">
         <v>77.39999999999999</v>
       </c>
       <c r="AR511" t="n">
-        <v>-0.002947463179424537</v>
+        <v>-0.00257722937529213</v>
       </c>
       <c r="AS511" t="n">
-        <v>6.777810071429111</v>
+        <v>6.777772079133445</v>
       </c>
       <c r="AT511" t="n">
-        <v>-0.03271007142911131</v>
+        <v>-0.03267207913344539</v>
       </c>
       <c r="AU511" t="n">
         <v>-0.03270008316040052</v>
       </c>
       <c r="AV511" t="n">
-        <v>-0.01668834783162216</v>
+        <v>-0.01668951675446277</v>
       </c>
       <c r="AW511" t="n">
-        <v>-0.02286367664309125</v>
+        <v>-0.02286406628403812</v>
       </c>
       <c r="AX511" t="n">
-        <v>0.007072036444398397</v>
+        <v>0.007071727664475771</v>
       </c>
       <c r="AY511" t="n">
         <v>33.33333333333333</v>
@@ -83812,7 +83812,7 @@
         <v>68.62666666666667</v>
       </c>
       <c r="BA511" t="n">
-        <v>70.17969372070581</v>
+        <v>70.1916937207058</v>
       </c>
     </row>
     <row r="512">
@@ -83923,10 +83923,10 @@
         <v>-0.3456268937433125</v>
       </c>
       <c r="AI512" t="n">
-        <v>6.748101272412299</v>
+        <v>6.748064561399866</v>
       </c>
       <c r="AJ512" t="n">
-        <v>0.004198513201714604</v>
+        <v>0.004235224214148126</v>
       </c>
       <c r="AK512" t="n">
         <v>6.740096815166266</v>
@@ -83935,40 +83935,40 @@
         <v>0.01220297044774732</v>
       </c>
       <c r="AM512" t="n">
-        <v>-0.3977059644204096</v>
+        <v>-0.3976889317784199</v>
       </c>
       <c r="AN512" t="n">
-        <v>0.02271888896632723</v>
+        <v>0.02268190844878654</v>
       </c>
       <c r="AO512" t="n">
-        <v>0.6953537478383294</v>
+        <v>0.6953567146475523</v>
       </c>
       <c r="AP512" t="n">
-        <v>1.261451878023444</v>
+        <v>1.261868708113399</v>
       </c>
       <c r="AQ512" t="n">
         <v>72</v>
       </c>
       <c r="AR512" t="n">
-        <v>-0.001667844427570216</v>
+        <v>-0.001295276208961914</v>
       </c>
       <c r="AS512" t="n">
-        <v>6.777807999313707</v>
+        <v>6.777806230979031</v>
       </c>
       <c r="AT512" t="n">
-        <v>-0.04200799931370636</v>
+        <v>-0.04200623097903033</v>
       </c>
       <c r="AU512" t="n">
         <v>-0.04200008316040016</v>
       </c>
       <c r="AV512" t="n">
-        <v>-0.01908940212389187</v>
+        <v>-0.01909048262999868</v>
       </c>
       <c r="AW512" t="n">
-        <v>-0.02282818487393242</v>
+        <v>-0.0228285450426347</v>
       </c>
       <c r="AX512" t="n">
-        <v>0.007648422767917895</v>
+        <v>0.007648168013300609</v>
       </c>
       <c r="AY512" t="n">
         <v>20.8955223880597</v>
@@ -83977,7 +83977,7 @@
         <v>61.39343283582089</v>
       </c>
       <c r="BA512" t="n">
-        <v>68.0219931910958</v>
+        <v>68.0339931910958</v>
       </c>
     </row>
     <row r="513">
@@ -84088,10 +84088,10 @@
         <v>-0.3468885181379404</v>
       </c>
       <c r="AI513" t="n">
-        <v>6.747255722628349</v>
+        <v>6.747226278872152</v>
       </c>
       <c r="AJ513" t="n">
-        <v>0.00594433154035201</v>
+        <v>0.005973775296548745</v>
       </c>
       <c r="AK513" t="n">
         <v>6.755554272205931</v>
@@ -84100,40 +84100,40 @@
         <v>-0.002354218037229572</v>
       </c>
       <c r="AM513" t="n">
-        <v>-0.400375027138847</v>
+        <v>-0.4003515275861345</v>
       </c>
       <c r="AN513" t="n">
-        <v>0.02402774236102168</v>
+        <v>0.02398656672240618</v>
       </c>
       <c r="AO513" t="n">
-        <v>0.7067971474351272</v>
+        <v>0.7067969646460921</v>
       </c>
       <c r="AP513" t="n">
-        <v>1.280261960188511</v>
+        <v>1.280599476642095</v>
       </c>
       <c r="AQ513" t="n">
         <v>72</v>
       </c>
       <c r="AR513" t="n">
-        <v>-0.002571042581132646</v>
+        <v>-0.002197804801327254</v>
       </c>
       <c r="AS513" t="n">
-        <v>6.777834973032914</v>
+        <v>6.777829908076522</v>
       </c>
       <c r="AT513" t="n">
-        <v>-0.04083497303291406</v>
+        <v>-0.04082990807652198</v>
       </c>
       <c r="AU513" t="n">
         <v>-0.04080008316040029</v>
       </c>
       <c r="AV513" t="n">
-        <v>-0.02186591568249581</v>
+        <v>-0.02186674294078301</v>
       </c>
       <c r="AW513" t="n">
-        <v>-0.02266050197588759</v>
+        <v>-0.02266077772864999</v>
       </c>
       <c r="AX513" t="n">
-        <v>0.008435733076265082</v>
+        <v>0.008435519684562156</v>
       </c>
       <c r="AY513" t="n">
         <v>23.52941176470588</v>
@@ -84142,7 +84142,7 @@
         <v>61.89529411764705</v>
       </c>
       <c r="BA513" t="n">
-        <v>65.57660757018076</v>
+        <v>65.58860757018076</v>
       </c>
     </row>
     <row r="514">
@@ -84253,10 +84253,10 @@
         <v>-0.3419644234534092</v>
       </c>
       <c r="AI514" t="n">
-        <v>6.725029661829083</v>
+        <v>6.724989986752571</v>
       </c>
       <c r="AJ514" t="n">
-        <v>0.024670407598407</v>
+        <v>0.02471008267491914</v>
       </c>
       <c r="AK514" t="n">
         <v>6.75925064743029</v>
@@ -84265,40 +84265,40 @@
         <v>-0.009550578002800236</v>
       </c>
       <c r="AM514" t="n">
-        <v>-0.4018162797423327</v>
+        <v>-0.4017887258056133</v>
       </c>
       <c r="AN514" t="n">
-        <v>0.02486590604389916</v>
+        <v>0.02482212216928553</v>
       </c>
       <c r="AO514" t="n">
-        <v>0.7173010872263644</v>
+        <v>0.7172988664983253</v>
       </c>
       <c r="AP514" t="n">
-        <v>1.475588032504229</v>
+        <v>1.476029071691014</v>
       </c>
       <c r="AQ514" t="n">
         <v>76</v>
       </c>
       <c r="AR514" t="n">
-        <v>-0.003048533390401412</v>
+        <v>-0.002676225531211758</v>
       </c>
       <c r="AS514" t="n">
-        <v>6.777742048928296</v>
+        <v>6.777749136467762</v>
       </c>
       <c r="AT514" t="n">
-        <v>-0.03894204892829567</v>
+        <v>-0.03894913646776121</v>
       </c>
       <c r="AU514" t="n">
         <v>-0.03900008316040005</v>
       </c>
       <c r="AV514" t="n">
-        <v>-0.02398129735366554</v>
+        <v>-0.02398247898892603</v>
       </c>
       <c r="AW514" t="n">
-        <v>-0.02242539258919371</v>
+        <v>-0.02242578646761387</v>
       </c>
       <c r="AX514" t="n">
-        <v>0.009369073681460472</v>
+        <v>0.009368919371520569</v>
       </c>
       <c r="AY514" t="n">
         <v>26.08695652173913</v>
@@ -84307,7 +84307,7 @@
         <v>66.23043478260868</v>
       </c>
       <c r="BA514" t="n">
-        <v>65.4473195267025</v>
+        <v>65.4593195267025</v>
       </c>
     </row>
     <row r="515">
@@ -84418,10 +84418,10 @@
         <v>-0.3448997849091837</v>
       </c>
       <c r="AI515" t="n">
-        <v>6.738255595412468</v>
+        <v>6.738231277482312</v>
       </c>
       <c r="AJ515" t="n">
-        <v>0.01054420546033441</v>
+        <v>0.01056852339049108</v>
       </c>
       <c r="AK515" t="n">
         <v>6.734775445902895</v>
@@ -84430,40 +84430,40 @@
         <v>0.01402435496990773</v>
       </c>
       <c r="AM515" t="n">
-        <v>-0.4022609316376698</v>
+        <v>-0.4022294042554291</v>
       </c>
       <c r="AN515" t="n">
-        <v>0.02550387683415684</v>
+        <v>0.02545790195722747</v>
       </c>
       <c r="AO515" t="n">
-        <v>0.7273351886096061</v>
+        <v>0.7273309315128231</v>
       </c>
       <c r="AP515" t="n">
-        <v>1.327674329276297</v>
+        <v>1.327950493923702</v>
       </c>
       <c r="AQ515" t="n">
         <v>73.40000000000001</v>
       </c>
       <c r="AR515" t="n">
-        <v>-0.003209446091365261</v>
+        <v>-0.00283897806389091</v>
       </c>
       <c r="AS515" t="n">
-        <v>6.777880593950862</v>
+        <v>6.777871300548548</v>
       </c>
       <c r="AT515" t="n">
-        <v>-0.04368059395086288</v>
+        <v>-0.04367130054854851</v>
       </c>
       <c r="AU515" t="n">
         <v>-0.04360008316040087</v>
       </c>
       <c r="AV515" t="n">
-        <v>-0.02549716202171321</v>
+        <v>-0.02549787898685798</v>
       </c>
       <c r="AW515" t="n">
-        <v>-0.02268435352002974</v>
+        <v>-0.02268459250841133</v>
       </c>
       <c r="AX515" t="n">
-        <v>0.0104097382888749</v>
+        <v>0.01040961982719224</v>
       </c>
       <c r="AY515" t="n">
         <v>18.57142857142857</v>
@@ -84583,10 +84583,10 @@
         <v>-0.3389992354304407</v>
       </c>
       <c r="AI516" t="n">
-        <v>6.718233131673284</v>
+        <v>6.718201282169581</v>
       </c>
       <c r="AJ516" t="n">
-        <v>0.02916667530303485</v>
+        <v>0.02919852480673768</v>
       </c>
       <c r="AK516" t="n">
         <v>6.753996132599221</v>
@@ -84595,40 +84595,40 @@
         <v>-0.00659632562290291</v>
       </c>
       <c r="AM516" t="n">
-        <v>-0.4028302582145923</v>
+        <v>-0.4027953816469058</v>
       </c>
       <c r="AN516" t="n">
-        <v>0.02613064267520054</v>
+        <v>0.02608258444417638</v>
       </c>
       <c r="AO516" t="n">
-        <v>0.736680621170787</v>
+        <v>0.736674421029931</v>
       </c>
       <c r="AP516" t="n">
-        <v>1.519404100140539</v>
+        <v>1.519755165509982</v>
       </c>
       <c r="AQ516" t="n">
         <v>77.40000000000001</v>
       </c>
       <c r="AR516" t="n">
-        <v>-0.002316067232288264</v>
+        <v>-0.001943929707255048</v>
       </c>
       <c r="AS516" t="n">
-        <v>6.777766985447334</v>
+        <v>6.77777230347129</v>
       </c>
       <c r="AT516" t="n">
-        <v>-0.04466698544733472</v>
+        <v>-0.04467230347129014</v>
       </c>
       <c r="AU516" t="n">
         <v>-0.04470008316040097</v>
       </c>
       <c r="AV516" t="n">
-        <v>-0.02727547540728308</v>
+        <v>-0.02727645827362562</v>
       </c>
       <c r="AW516" t="n">
-        <v>-0.02273936236900309</v>
+        <v>-0.02273968999111727</v>
       </c>
       <c r="AX516" t="n">
-        <v>0.01159900799371883</v>
+        <v>0.01159893867535329</v>
       </c>
       <c r="AY516" t="n">
         <v>16.90140845070422</v>
@@ -84748,10 +84748,10 @@
         <v>-0.3329117502755388</v>
       </c>
       <c r="AI517" t="n">
-        <v>6.730931854936179</v>
+        <v>6.730898772467414</v>
       </c>
       <c r="AJ517" t="n">
-        <v>0.01646795204013962</v>
+        <v>0.01650103450890406</v>
       </c>
       <c r="AK517" t="n">
         <v>6.732394407262716</v>
@@ -84760,40 +84760,40 @@
         <v>0.01500539971360215</v>
       </c>
       <c r="AM517" t="n">
-        <v>-0.4025465822999924</v>
+        <v>-0.4025099007694142</v>
       </c>
       <c r="AN517" t="n">
-        <v>0.02639266239094257</v>
+        <v>0.02634377330607651</v>
       </c>
       <c r="AO517" t="n">
-        <v>0.7465684054287068</v>
+        <v>0.746561519528266</v>
       </c>
       <c r="AP517" t="n">
-        <v>1.38648834307159</v>
+        <v>1.386847953743529</v>
       </c>
       <c r="AQ517" t="n">
         <v>78</v>
       </c>
       <c r="AR517" t="n">
-        <v>0.000398730842820588</v>
+        <v>0.0007826925161683791</v>
       </c>
       <c r="AS517" t="n">
-        <v>6.777800353984499</v>
+        <v>6.77780061477715</v>
       </c>
       <c r="AT517" t="n">
-        <v>-0.04510035398449919</v>
+        <v>-0.04510061477715066</v>
       </c>
       <c r="AU517" t="n">
         <v>-0.04510008316040093</v>
       </c>
       <c r="AV517" t="n">
-        <v>-0.02849847336672493</v>
+        <v>-0.02849946927270004</v>
       </c>
       <c r="AW517" t="n">
-        <v>-0.02305851159320798</v>
+        <v>-0.02305884356186635</v>
       </c>
       <c r="AX517" t="n">
-        <v>0.01288089136988278</v>
+        <v>0.012880871846816</v>
       </c>
       <c r="AY517" t="n">
         <v>16.66666666666666</v>
@@ -84913,10 +84913,10 @@
         <v>-0.3335936335657701</v>
       </c>
       <c r="AI518" t="n">
-        <v>6.740623868728166</v>
+        <v>6.740580458294252</v>
       </c>
       <c r="AJ518" t="n">
-        <v>0.00437601683091593</v>
+        <v>0.004419427264830134</v>
       </c>
       <c r="AK518" t="n">
         <v>6.74318350621926</v>
@@ -84925,40 +84925,40 @@
         <v>0.001816379339821594</v>
       </c>
       <c r="AM518" t="n">
-        <v>-0.4034654226643876</v>
+        <v>-0.4034224290251451</v>
       </c>
       <c r="AN518" t="n">
-        <v>0.02741459853506639</v>
+        <v>0.02736182786837871</v>
       </c>
       <c r="AO518" t="n">
-        <v>0.7552010609216553</v>
+        <v>0.755189863471066</v>
       </c>
       <c r="AP518" t="n">
-        <v>1.258871370070383</v>
+        <v>1.259334239690847</v>
       </c>
       <c r="AQ518" t="n">
         <v>76.2</v>
       </c>
       <c r="AR518" t="n">
-        <v>0.004293437255601791</v>
+        <v>0.004684779010825857</v>
       </c>
       <c r="AS518" t="n">
-        <v>6.777855473686805</v>
+        <v>6.777860522468127</v>
       </c>
       <c r="AT518" t="n">
-        <v>-0.0457554736868051</v>
+        <v>-0.04576052246812701</v>
       </c>
       <c r="AU518" t="n">
         <v>-0.04570008316040042</v>
       </c>
       <c r="AV518" t="n">
-        <v>-0.02970335352472828</v>
+        <v>-0.02970460186976949</v>
       </c>
       <c r="AW518" t="n">
-        <v>-0.02310297375138447</v>
+        <v>-0.02310338986639821</v>
       </c>
       <c r="AX518" t="n">
-        <v>0.01424313050944462</v>
+        <v>0.0142431734036299</v>
       </c>
       <c r="AY518" t="n">
         <v>15.06849315068493</v>
@@ -85078,10 +85078,10 @@
         <v>-0.3086955151355042</v>
       </c>
       <c r="AI519" t="n">
-        <v>6.755750978622371</v>
+        <v>6.755708466794879</v>
       </c>
       <c r="AJ519" t="n">
-        <v>-0.01245101753228273</v>
+        <v>-0.01240850570479068</v>
       </c>
       <c r="AK519" t="n">
         <v>6.746865899087779</v>
@@ -85090,40 +85090,40 @@
         <v>-0.003565937997691115</v>
       </c>
       <c r="AM519" t="n">
-        <v>-0.4037527699419104</v>
+        <v>-0.4037073020769307</v>
       </c>
       <c r="AN519" t="n">
-        <v>0.02783693810207571</v>
+        <v>0.02778289906564352</v>
       </c>
       <c r="AO519" t="n">
-        <v>0.7638345477935677</v>
+        <v>0.7638221248099442</v>
       </c>
       <c r="AP519" t="n">
-        <v>1.083114808402871</v>
+        <v>1.083564796528327</v>
       </c>
       <c r="AQ519" t="n">
         <v>78.40000000000001</v>
       </c>
       <c r="AR519" t="n">
-        <v>0.002685989934888373</v>
+        <v>0.003077728100043848</v>
       </c>
       <c r="AS519" t="n">
-        <v>6.777790980963837</v>
+        <v>6.777789653454104</v>
       </c>
       <c r="AT519" t="n">
-        <v>-0.04589098096383637</v>
+        <v>-0.04588965345410401</v>
       </c>
       <c r="AU519" t="n">
         <v>-0.04590008316039995</v>
       </c>
       <c r="AV519" t="n">
-        <v>-0.03114978747105965</v>
+        <v>-0.03115096944061424</v>
       </c>
       <c r="AW519" t="n">
-        <v>-0.02326898278119868</v>
+        <v>-0.02326937677105021</v>
       </c>
       <c r="AX519" t="n">
-        <v>0.0156832187845257</v>
+        <v>0.01568332077718871</v>
       </c>
       <c r="AY519" t="n">
         <v>14.86486486486486</v>
@@ -85132,7 +85132,7 @@
         <v>59.6627027027027</v>
       </c>
       <c r="BA519" t="n">
-        <v>61.48110031930444</v>
+        <v>61.48110031930445</v>
       </c>
     </row>
     <row r="520">
@@ -85243,10 +85243,10 @@
         <v>-0.3044857117372084</v>
       </c>
       <c r="AI520" t="n">
-        <v>6.736041496771461</v>
+        <v>6.73601646973098</v>
       </c>
       <c r="AJ520" t="n">
-        <v>0.006758738976830436</v>
+        <v>0.006783766017311343</v>
       </c>
       <c r="AK520" t="n">
         <v>6.761018647414997</v>
@@ -85255,40 +85255,40 @@
         <v>-0.01821841166670612</v>
       </c>
       <c r="AM520" t="n">
-        <v>-0.4035582267671979</v>
+        <v>-0.403510818895136</v>
       </c>
       <c r="AN520" t="n">
-        <v>0.02811368720091384</v>
+        <v>0.02805871830419215</v>
       </c>
       <c r="AO520" t="n">
-        <v>0.7684053332209008</v>
+        <v>0.7683919203573231</v>
       </c>
       <c r="AP520" t="n">
-        <v>1.283237597505188</v>
+        <v>1.283500676883961</v>
       </c>
       <c r="AQ520" t="n">
         <v>82.80000000000001</v>
       </c>
       <c r="AR520" t="n">
-        <v>0.002512847725393273</v>
+        <v>0.002903283150327664</v>
       </c>
       <c r="AS520" t="n">
-        <v>6.777750671658804</v>
+        <v>6.777742994313127</v>
       </c>
       <c r="AT520" t="n">
-        <v>-0.04745067165880457</v>
+        <v>-0.04744299431312715</v>
       </c>
       <c r="AU520" t="n">
         <v>-0.04750008316040066</v>
       </c>
       <c r="AV520" t="n">
-        <v>-0.03291383961704222</v>
+        <v>-0.03291463771931293</v>
       </c>
       <c r="AW520" t="n">
-        <v>-0.02330436538000775</v>
+        <v>-0.02330463141409799</v>
       </c>
       <c r="AX520" t="n">
-        <v>0.01721383580295904</v>
+        <v>0.01721397770073558</v>
       </c>
       <c r="AY520" t="n">
         <v>13.33333333333333</v>
@@ -85408,10 +85408,10 @@
         <v>-0.3058180386269767</v>
       </c>
       <c r="AI521" t="n">
-        <v>6.727097306239223</v>
+        <v>6.727075391426066</v>
       </c>
       <c r="AJ521" t="n">
-        <v>0.01570292950906804</v>
+        <v>0.0157248443222251</v>
       </c>
       <c r="AK521" t="n">
         <v>6.751365564447465</v>
@@ -85420,40 +85420,40 @@
         <v>-0.008565328699174479</v>
       </c>
       <c r="AM521" t="n">
-        <v>-0.4028391433898537</v>
+        <v>-0.4027898636641267</v>
       </c>
       <c r="AN521" t="n">
-        <v>0.02832926039605738</v>
+        <v>0.02827333203020888</v>
       </c>
       <c r="AO521" t="n">
-        <v>0.772697704205352</v>
+        <v>0.7726830480787004</v>
       </c>
       <c r="AP521" t="n">
-        <v>1.374437475397088</v>
+        <v>1.374664583418879</v>
       </c>
       <c r="AQ521" t="n">
         <v>83.39999999999999</v>
       </c>
       <c r="AR521" t="n">
-        <v>0.003102787852250152</v>
+        <v>0.003496032653493206</v>
       </c>
       <c r="AS521" t="n">
-        <v>6.777793753506412</v>
+        <v>6.777792951291229</v>
       </c>
       <c r="AT521" t="n">
-        <v>-0.04919375350641175</v>
+        <v>-0.04919295129122858</v>
       </c>
       <c r="AU521" t="n">
         <v>-0.04920008316040025</v>
       </c>
       <c r="AV521" t="n">
-        <v>-0.03432167537367801</v>
+        <v>-0.03432243336518957</v>
       </c>
       <c r="AW521" t="n">
-        <v>-0.02314093031627589</v>
+        <v>-0.02314118298011308</v>
       </c>
       <c r="AX521" t="n">
-        <v>0.01879897788904702</v>
+        <v>0.01879915768639914</v>
       </c>
       <c r="AY521" t="n">
         <v>13.1578947368421</v>
@@ -85573,10 +85573,10 @@
         <v>-0.3061509986743562</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.725827786095255</v>
+        <v>6.725806144687715</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.01407232605684428</v>
+        <v>0.01409396746438496</v>
       </c>
       <c r="AK522" t="n">
         <v>6.744478107428201</v>
@@ -85585,40 +85585,40 @@
         <v>-0.004577995276100921</v>
       </c>
       <c r="AM522" t="n">
-        <v>-0.4028436036871637</v>
+        <v>-0.4027900432658338</v>
       </c>
       <c r="AN522" t="n">
-        <v>0.02897312163273263</v>
+        <v>0.02891453613228628</v>
       </c>
       <c r="AO522" t="n">
-        <v>0.77845375368416</v>
+        <v>0.7784357006627721</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.355267848979187</v>
+        <v>1.355489422378676</v>
       </c>
       <c r="AQ522" t="n">
         <v>83</v>
       </c>
       <c r="AR522" t="n">
-        <v>0.003144246289783567</v>
+        <v>0.00353753124109526</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.777802222424294</v>
+        <v>6.777802490005207</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.04580222242429421</v>
+        <v>-0.0458024900052072</v>
       </c>
       <c r="AU522" t="n">
         <v>-0.04580008316040018</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.03547178233687269</v>
+        <v>-0.03547691152123185</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02297823852258113</v>
+        <v>-0.0229784956461002</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.02038226104023146</v>
+        <v>0.02038291518749163</v>
       </c>
       <c r="AY522" t="n">
         <v>18.18181818181818</v>
@@ -85738,10 +85738,10 @@
         <v>-0.2816739226305129</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.700825207080349</v>
+        <v>6.700854569500288</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.04177475706149636</v>
+        <v>0.04174539464155735</v>
       </c>
       <c r="AK523" t="n">
         <v>6.743301592583855</v>
@@ -85750,40 +85750,40 @@
         <v>-0.0007016284420089391</v>
       </c>
       <c r="AM523" t="n">
-        <v>-0.402800556007337</v>
+        <v>-0.402742697458547</v>
       </c>
       <c r="AN523" t="n">
-        <v>0.02961696780468992</v>
+        <v>0.02955568036482276</v>
       </c>
       <c r="AO523" t="n">
-        <v>0.7839607851241809</v>
+        <v>0.7839391318357882</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.635849330461463</v>
+        <v>1.635541400731503</v>
       </c>
       <c r="AQ523" t="n">
         <v>88</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.001099449811417698</v>
+        <v>0.001482633885639268</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.777738763386478</v>
+        <v>6.777717392005486</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.06033876338647737</v>
+        <v>-0.06031739200548536</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.06040008316039991</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.03763871634817657</v>
+        <v>-0.03764180906255939</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.02294832967567872</v>
+        <v>-0.0229482306095146</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.02197811043668929</v>
+        <v>0.02197908871531237</v>
       </c>
       <c r="AY523" t="n">
         <v>7.692307692307693</v>
@@ -85814,13 +85814,13 @@
         <v>6.742599964141846</v>
       </c>
       <c r="F524" t="n">
-        <v>6.72445011138916</v>
+        <v>6.72599983215332</v>
       </c>
       <c r="G524" t="n">
-        <v>6.7126</v>
+        <v>6.7123</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01814985275268555</v>
+        <v>-0.01660013198852539</v>
       </c>
       <c r="I524" t="n">
         <v>98.83000183105469</v>
@@ -85903,10 +85903,10 @@
         <v>-0.292031968188172</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.700987071445542</v>
+        <v>6.70101752749652</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.04161289269630331</v>
+        <v>0.04158243664532613</v>
       </c>
       <c r="AK524" t="n">
         <v>6.74285285202661</v>
@@ -85915,40 +85915,40 @@
         <v>-0.0002528878847645188</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.4016479100718945</v>
+        <v>-0.401588500320058</v>
       </c>
       <c r="AN524" t="n">
-        <v>0.02991561487494565</v>
+        <v>0.02985284499018426</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.7880527230405053</v>
+        <v>0.7880284607160943</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.624363684557714</v>
+        <v>1.624050314085442</v>
       </c>
       <c r="AQ524" t="n">
         <v>87.40000000000001</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.0005908780548055115</v>
+        <v>0.0009798171680228706</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
       </c>
       <c r="AT524" t="n">
-        <v>-0.06520008316040027</v>
+        <v>-0.06550008316040046</v>
       </c>
       <c r="AU524" t="n">
-        <v>-0.06520008316040027</v>
+        <v>-0.06550008316040046</v>
       </c>
       <c r="AV524" t="n">
-        <v>-0.04031217972432932</v>
+        <v>-0.04032777572125279</v>
       </c>
       <c r="AW524" t="n">
-        <v>-0.02294157367062549</v>
+        <v>-0.02294647460446136</v>
       </c>
       <c r="AX524" t="n">
-        <v>0.02365678791232725</v>
+        <v>0.02365859065056729</v>
       </c>
       <c r="AY524" t="n">
         <v>6.329113924050633</v>
@@ -85957,7 +85957,7 @@
         <v>61.40518987341772</v>
       </c>
       <c r="BA524" t="n">
-        <v>62.35861275078463</v>
+        <v>62.35861275078464</v>
       </c>
     </row>
   </sheetData>
@@ -86174,7 +86174,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.72</t>
+          <t>6.73</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-08-24 11:29 EDT
Score: 62/100
USD/CNY: 6.72
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.722499847412109</v>
       </c>
       <c r="F522" t="n">
-        <v>6.723060131072998</v>
+        <v>6.7217698097229</v>
       </c>
       <c r="G522" t="n">
-        <v>6.710199999999999</v>
+        <v>6.710599999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>0.0005602836608886719</v>
+        <v>-0.0007300376892089844</v>
       </c>
       <c r="I522" t="n">
         <v>98.80000305175781</v>
@@ -85606,19 +85606,19 @@
         <v>6.7778000831604</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.06760008316040089</v>
+        <v>-0.06720008316040094</v>
       </c>
       <c r="AU522" t="n">
-        <v>-0.06760008316040089</v>
+        <v>-0.06720008316040094</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.04489321414777044</v>
+        <v>-0.04487321414777044</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02272192160190579</v>
+        <v>-0.02271525493523912</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.02714406602550303</v>
+        <v>0.02714306602550303</v>
       </c>
       <c r="AY522" t="n">
         <v>6.172839506172839</v>

</xml_diff>

<commit_message>
auto: data update 2026-08-24 14:50 EDT
Score: 62/100
USD/CNY: 6.72
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.722499847412109</v>
       </c>
       <c r="F522" t="n">
-        <v>6.7217698097229</v>
+        <v>6.7223801612854</v>
       </c>
       <c r="G522" t="n">
-        <v>6.710599999999999</v>
+        <v>6.710199999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.0007300376892089844</v>
+        <v>-0.0001196861267089844</v>
       </c>
       <c r="I522" t="n">
         <v>98.80000305175781</v>
@@ -85606,19 +85606,19 @@
         <v>6.7778000831604</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.06720008316040094</v>
+        <v>-0.06760008316040089</v>
       </c>
       <c r="AU522" t="n">
-        <v>-0.06720008316040094</v>
+        <v>-0.06760008316040089</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.04487321414777044</v>
+        <v>-0.04489321414777044</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.02271525493523912</v>
+        <v>-0.02272192160190579</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.02714306602550303</v>
+        <v>0.02714406602550303</v>
       </c>
       <c r="AY522" t="n">
         <v>6.172839506172839</v>

</xml_diff>

<commit_message>
auto: data update 2026-08-27 22:08 EDT
Score: 59/100
USD/CNY: 6.72
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85658,10 +85658,10 @@
         <v>0.05530023574829102</v>
       </c>
       <c r="I523" t="n">
-        <v>99.11100006103516</v>
+        <v>99.1510009765625</v>
       </c>
       <c r="J523" t="n">
-        <v>-0.0005949189170060265</v>
+        <v>-0.000191561891031311</v>
       </c>
       <c r="K523" t="n">
         <v>2.946</v>
@@ -85738,10 +85738,10 @@
         <v>-0.2936792078827581</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.717149638221525</v>
+        <v>6.718389873540735</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.00535020919058482</v>
+        <v>0.004109973871374351</v>
       </c>
       <c r="AK523" t="n">
         <v>6.750203856204787</v>
@@ -85759,40 +85759,40 @@
         <v>0.8091236362457368</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.232941714499793</v>
+        <v>1.22029923996184</v>
       </c>
       <c r="AQ523" t="n">
-        <v>83.40000000000001</v>
+        <v>82.80000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.001163355780539243</v>
+        <v>0.001248696127393385</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.77779539222896</v>
+        <v>6.777798461893056</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.06909539222895944</v>
+        <v>-0.06909846189305568</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.06910008316040006</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.05120807644166923</v>
+        <v>-0.05120822992487404</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.02455446386583358</v>
+        <v>-0.02455451502690185</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.03274761744791971</v>
+        <v>0.03274762512207995</v>
       </c>
       <c r="AY523" t="n">
         <v>5.952380952380952</v>
       </c>
       <c r="AZ523" t="n">
-        <v>58.46333333333333</v>
+        <v>58.28333333333334</v>
       </c>
       <c r="BA523" t="n">
-        <v>59.42659029251604</v>
+        <v>59.39059029251605</v>
       </c>
     </row>
     <row r="524">
@@ -85814,16 +85814,16 @@
         <v>6.722499847412109</v>
       </c>
       <c r="F524" t="n">
-        <v>6.719840049743652</v>
+        <v>6.719880104064941</v>
       </c>
       <c r="G524" t="n">
-        <v>6.710800000000001</v>
+        <v>6.7105</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.002659797668457031</v>
+        <v>-0.002619743347167969</v>
       </c>
       <c r="I524" t="n">
-        <v>99.11100006103516</v>
+        <v>99.1510009765625</v>
       </c>
       <c r="J524" t="n">
         <v>0</v>
@@ -85903,10 +85903,10 @@
         <v>-0.2841274887968197</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.716951256372843</v>
+        <v>6.718184747298512</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.005548591039266526</v>
+        <v>0.004315100113597481</v>
       </c>
       <c r="AK524" t="n">
         <v>6.74780904069481</v>
@@ -85915,49 +85915,49 @@
         <v>-0.02530919328270098</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.3964150137766067</v>
+        <v>-0.3964490104347927</v>
       </c>
       <c r="AN524" t="n">
-        <v>0.03138815023505231</v>
+        <v>0.03139513852215547</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.8123509842810366</v>
+        <v>0.8123536141048051</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.231376023962598</v>
+        <v>1.218950111394028</v>
       </c>
       <c r="AQ524" t="n">
-        <v>83.80000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.001100583460408415</v>
+        <v>0.001185203606268944</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
       </c>
       <c r="AT524" t="n">
-        <v>-0.06700008316039963</v>
+        <v>-0.0673000831604007</v>
       </c>
       <c r="AU524" t="n">
-        <v>-0.06700008316039963</v>
+        <v>-0.0673000831604007</v>
       </c>
       <c r="AV524" t="n">
-        <v>-0.05277603740082264</v>
+        <v>-0.05279119088402751</v>
       </c>
       <c r="AW524" t="n">
-        <v>-0.02563521363311894</v>
+        <v>-0.02564026479418723</v>
       </c>
       <c r="AX524" t="n">
-        <v>0.03464809343715716</v>
+        <v>0.03464885878547765</v>
       </c>
       <c r="AY524" t="n">
         <v>9.411764705882353</v>
       </c>
       <c r="AZ524" t="n">
-        <v>59.72411764705883</v>
+        <v>59.60411764705883</v>
       </c>
       <c r="BA524" t="n">
-        <v>59.10941382192781</v>
+        <v>59.04941382192781</v>
       </c>
     </row>
   </sheetData>
@@ -86194,7 +86194,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.11</t>
+          <t>99.15</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86284,7 +86284,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-08-27 22:27 EDT
Score: 59/100
USD/CNY: 6.72
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85658,10 +85658,10 @@
         <v>0.05530023574829102</v>
       </c>
       <c r="I523" t="n">
-        <v>99.1510009765625</v>
+        <v>99.16899871826172</v>
       </c>
       <c r="J523" t="n">
-        <v>-0.000191561891031311</v>
+        <v>-1.007815571285597e-05</v>
       </c>
       <c r="K523" t="n">
         <v>2.946</v>
@@ -85738,10 +85738,10 @@
         <v>-0.2936792078827581</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.718389873540735</v>
+        <v>6.718947896641635</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.004109973871374351</v>
+        <v>0.003551950770474654</v>
       </c>
       <c r="AK523" t="n">
         <v>6.750203856204787</v>
@@ -85759,31 +85759,31 @@
         <v>0.8091236362457368</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.22029923996184</v>
+        <v>1.214610194557186</v>
       </c>
       <c r="AQ523" t="n">
         <v>82.80000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.001248696127393385</v>
+        <v>0.00128704986279593</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.777798461893056</v>
+        <v>6.777799995244952</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.06909846189305568</v>
+        <v>-0.06909999524495181</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.06910008316040006</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.05120822992487404</v>
+        <v>-0.05120830659246885</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.02455451502690185</v>
+        <v>-0.02455454058276678</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.03274762512207995</v>
+        <v>0.03274762895545969</v>
       </c>
       <c r="AY523" t="n">
         <v>5.952380952380952</v>
@@ -85814,16 +85814,16 @@
         <v>6.722499847412109</v>
       </c>
       <c r="F524" t="n">
-        <v>6.719880104064941</v>
+        <v>6.720749855041504</v>
       </c>
       <c r="G524" t="n">
         <v>6.7105</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.002619743347167969</v>
+        <v>-0.001749992370605469</v>
       </c>
       <c r="I524" t="n">
-        <v>99.1510009765625</v>
+        <v>99.16899871826172</v>
       </c>
       <c r="J524" t="n">
         <v>0</v>
@@ -85903,10 +85903,10 @@
         <v>-0.2841274887968197</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.718184747298512</v>
+        <v>6.718740063284643</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.004315100113597481</v>
+        <v>0.003759784127466581</v>
       </c>
       <c r="AK524" t="n">
         <v>6.74780904069481</v>
@@ -85915,22 +85915,22 @@
         <v>-0.02530919328270098</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.3964490104347927</v>
+        <v>-0.3964639927027396</v>
       </c>
       <c r="AN524" t="n">
-        <v>0.03139513852215547</v>
+        <v>0.03139812368678613</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.8123536141048051</v>
+        <v>0.8123545829088162</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.218950111394028</v>
+        <v>1.213354429867917</v>
       </c>
       <c r="AQ524" t="n">
-        <v>83.40000000000001</v>
+        <v>83.2</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.001185203606268944</v>
+        <v>0.001223235789574726</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85942,22 +85942,22 @@
         <v>-0.0673000831604007</v>
       </c>
       <c r="AV524" t="n">
-        <v>-0.05279119088402751</v>
+        <v>-0.05279126755162231</v>
       </c>
       <c r="AW524" t="n">
-        <v>-0.02564026479418723</v>
+        <v>-0.02564029035005217</v>
       </c>
       <c r="AX524" t="n">
-        <v>0.03464885878547765</v>
+        <v>0.03464886645223712</v>
       </c>
       <c r="AY524" t="n">
         <v>9.411764705882353</v>
       </c>
       <c r="AZ524" t="n">
-        <v>59.60411764705883</v>
+        <v>59.54411764705883</v>
       </c>
       <c r="BA524" t="n">
-        <v>59.04941382192781</v>
+        <v>59.03741382192781</v>
       </c>
     </row>
   </sheetData>
@@ -86194,7 +86194,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.15</t>
+          <t>99.17</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-08-28 19:16 EDT
Score: 61/100
USD/CNY: 6.72
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85658,10 +85658,10 @@
         <v>0.05530023574829102</v>
       </c>
       <c r="I523" t="n">
-        <v>99.16899871826172</v>
+        <v>99.16000366210938</v>
       </c>
       <c r="J523" t="n">
-        <v>-1.007815571285597e-05</v>
+        <v>-0.0001007815571288928</v>
       </c>
       <c r="K523" t="n">
         <v>2.946</v>
@@ -85685,28 +85685,28 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.02</v>
+        <v>4.04</v>
       </c>
       <c r="S523" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
       <c r="T523" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
       <c r="U523" t="n">
         <v>-4.36860118332041</v>
       </c>
       <c r="V523" t="n">
-        <v>6.5428</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.673110472159945</v>
+        <v>-1.843062108209725</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2405695131407759</v>
+        <v>0.6424781826185999</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.032128514056225</v>
+        <v>33.33333333333334</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85717,10 +85717,10 @@
         <v>1.66939</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.61939</v>
+        <v>1.6297</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.39053</v>
+        <v>1.37409</v>
       </c>
       <c r="AD523" t="n">
         <v>0.1893899999999999</v>
@@ -85729,7 +85729,7 @@
         <v>5.357142857142857</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4299595131407763</v>
+        <v>0.4530881826185995</v>
       </c>
       <c r="AG523" t="n">
         <v>7.016179055294868</v>
@@ -85738,10 +85738,10 @@
         <v>-0.2936792078827581</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.718947896641635</v>
+        <v>6.718669003366535</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.003551950770474654</v>
+        <v>0.003830844045574544</v>
       </c>
       <c r="AK523" t="n">
         <v>6.750203856204787</v>
@@ -85759,31 +85759,31 @@
         <v>0.8091236362457368</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.214610194557186</v>
+        <v>1.217453571381047</v>
       </c>
       <c r="AQ523" t="n">
         <v>82.80000000000001</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.00128704986279593</v>
+        <v>0.001267884840392782</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.777799995244952</v>
+        <v>6.777799217097114</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.06909999524495181</v>
+        <v>-0.06909921709711409</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.06910008316040006</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.05120830659246885</v>
+        <v>-0.05120826768507696</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.02455454058276678</v>
+        <v>-0.02455452761363615</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.03274762895545969</v>
+        <v>0.0327476270100901</v>
       </c>
       <c r="AY523" t="n">
         <v>5.952380952380952</v>
@@ -85802,64 +85802,64 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.2</v>
+        <v>4.34</v>
       </c>
       <c r="C524" t="n">
-        <v>1.254</v>
+        <v>1.2547</v>
       </c>
       <c r="D524" t="n">
-        <v>2.946</v>
+        <v>3.0853</v>
       </c>
       <c r="E524" t="n">
         <v>6.722499847412109</v>
       </c>
       <c r="F524" t="n">
-        <v>6.720749855041504</v>
+        <v>6.729420185089111</v>
       </c>
       <c r="G524" t="n">
-        <v>6.7105</v>
+        <v>6.7182</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.001749992370605469</v>
+        <v>0.006920337677001953</v>
       </c>
       <c r="I524" t="n">
-        <v>99.16899871826172</v>
+        <v>99.16000366210938</v>
       </c>
       <c r="J524" t="n">
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>2.946</v>
+        <v>3.0853</v>
       </c>
       <c r="L524" t="n">
-        <v>2.958845</v>
+        <v>2.96581</v>
       </c>
       <c r="M524" t="n">
-        <v>2.931215</v>
+        <v>2.933536666666667</v>
       </c>
       <c r="N524" t="n">
-        <v>2.773515833333333</v>
+        <v>2.774676666666666</v>
       </c>
       <c r="O524" t="n">
-        <v>89.40000000000001</v>
+        <v>99.60000000000001</v>
       </c>
       <c r="P524" t="n">
-        <v>86.72654690618762</v>
+        <v>95.60878243512974</v>
       </c>
       <c r="Q524" t="n">
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>4.02</v>
+        <v>4.04</v>
       </c>
       <c r="S524" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
       <c r="T524" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.22651536252838</v>
+        <v>-3.948444785735005</v>
       </c>
       <c r="V524" t="n">
         <v>6.5428</v>
@@ -85868,10 +85868,10 @@
         <v>-2.673110472159945</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2405695131407759</v>
+        <v>-0.221104135235195</v>
       </c>
       <c r="Y524" t="n">
-        <v>8.23293172690763</v>
+        <v>8.835341365461847</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85882,10 +85882,10 @@
         <v>1.66939</v>
       </c>
       <c r="AB524" t="n">
-        <v>1.61939</v>
+        <v>1.6297</v>
       </c>
       <c r="AC524" t="n">
-        <v>1.39053</v>
+        <v>1.37409</v>
       </c>
       <c r="AD524" t="n">
         <v>0.1893899999999999</v>
@@ -85894,19 +85894,19 @@
         <v>5.555555555555555</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4299595131407763</v>
+        <v>-0.4104941352351954</v>
       </c>
       <c r="AG524" t="n">
-        <v>7.006627336208929</v>
+        <v>6.987934042108296</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.2841274887968197</v>
+        <v>-0.2654341946961871</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.718740063284643</v>
+        <v>6.663236103674507</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.003759784127466581</v>
+        <v>0.05926374373760268</v>
       </c>
       <c r="AK524" t="n">
         <v>6.74780904069481</v>
@@ -85915,49 +85915,49 @@
         <v>-0.02530919328270098</v>
       </c>
       <c r="AM524" t="n">
-        <v>-0.3964639927027396</v>
+        <v>-0.3964565291282772</v>
       </c>
       <c r="AN524" t="n">
-        <v>0.03139812368678613</v>
+        <v>0.03139664408873172</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.8123545829088162</v>
+        <v>0.8123541153569376</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.213354429867917</v>
+        <v>1.775623573144163</v>
       </c>
       <c r="AQ524" t="n">
-        <v>83.2</v>
+        <v>90</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.001223235789574726</v>
+        <v>0.00120423127913602</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
       </c>
       <c r="AT524" t="n">
-        <v>-0.0673000831604007</v>
+        <v>-0.0596000831604</v>
       </c>
       <c r="AU524" t="n">
-        <v>-0.0673000831604007</v>
+        <v>-0.0596000831604</v>
       </c>
       <c r="AV524" t="n">
-        <v>-0.05279126755162231</v>
+        <v>-0.05240622864423039</v>
       </c>
       <c r="AW524" t="n">
-        <v>-0.02564029035005217</v>
+        <v>-0.0255119440475882</v>
       </c>
       <c r="AX524" t="n">
-        <v>0.03464886645223712</v>
+        <v>0.03462961256149793</v>
       </c>
       <c r="AY524" t="n">
-        <v>9.411764705882353</v>
+        <v>15.29411764705882</v>
       </c>
       <c r="AZ524" t="n">
-        <v>59.54411764705883</v>
+        <v>67.21294117647059</v>
       </c>
       <c r="BA524" t="n">
-        <v>59.03741382192781</v>
+        <v>60.57117852781016</v>
       </c>
     </row>
   </sheetData>
@@ -86174,17 +86174,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>6.73</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>6.72</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6.71</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.20</t>
+          <t>4.34</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86194,22 +86194,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.17</t>
+          <t>99.16</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>3.09</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>96</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.02</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.54</t>
+          <t>2.56</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86254,12 +86254,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.37</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86274,17 +86274,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.43</t>
+          <t>-0.41</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86324,12 +86324,12 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.06</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.06</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
@@ -86344,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>61</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-08-29 16:49 EDT
Score: 61/100
USD/CNY: 6.72
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85658,10 +85658,10 @@
         <v>0.05530023574829102</v>
       </c>
       <c r="I523" t="n">
-        <v>99.16000366210938</v>
+        <v>99.69999694824219</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>0.005445676343184269</v>
       </c>
       <c r="K523" t="n">
         <v>3.0853</v>
@@ -85738,10 +85738,10 @@
         <v>-0.2654341946961871</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.663236103674507</v>
+        <v>6.680190080689523</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.05926374373760268</v>
+        <v>0.04230976672258624</v>
       </c>
       <c r="AK523" t="n">
         <v>6.74780904069481</v>
@@ -85759,40 +85759,40 @@
         <v>0.8123541153569376</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.775623573144163</v>
+        <v>1.604493248424094</v>
       </c>
       <c r="AQ523" t="n">
-        <v>90</v>
+        <v>89.8</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.001204231279136019</v>
+        <v>0.001653266510124163</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7778000831604</v>
+        <v>6.777861104740521</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.0596000831604</v>
+        <v>-0.05966110474052044</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.0596000831604</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.05240622864423039</v>
+        <v>-0.05240927972323641</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.0255119440475882</v>
+        <v>-0.02551296107392353</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.03462961256149793</v>
+        <v>0.03462976511544823</v>
       </c>
       <c r="AY523" t="n">
         <v>15.29411764705882</v>
       </c>
       <c r="AZ523" t="n">
-        <v>67.21294117647059</v>
+        <v>67.15294117647059</v>
       </c>
       <c r="BA523" t="n">
-        <v>60.57117852781016</v>
+        <v>60.55917852781016</v>
       </c>
     </row>
   </sheetData>
@@ -86029,7 +86029,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.16</t>
+          <t>99.70</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86119,7 +86119,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86144,17 +86144,17 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.002</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.7778</t>
+          <t>6.7779</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-01 16:55 EDT
Score: 62/100
USD/CNY: 6.73
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85516,13 +85516,13 @@
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>4.15</v>
+        <v>4.16</v>
       </c>
       <c r="S522" t="n">
-        <v>2.67</v>
+        <v>2.68</v>
       </c>
       <c r="T522" t="n">
-        <v>2.67</v>
+        <v>2.68</v>
       </c>
       <c r="U522" t="n">
         <v>-3.87136277760201</v>
@@ -85534,7 +85534,7 @@
         <v>-1.894139686776253</v>
       </c>
       <c r="X522" t="n">
-        <v>0.6972535162225402</v>
+        <v>0.7070641022538737</v>
       </c>
       <c r="Y522" t="n">
         <v>34.93975903614458</v>
@@ -85560,7 +85560,7 @@
         <v>5.555555555555555</v>
       </c>
       <c r="AF522" t="n">
-        <v>0.5078635162225398</v>
+        <v>0.5176741022538733</v>
       </c>
       <c r="AG522" t="n">
         <v>6.986387686076878</v>
@@ -85645,13 +85645,13 @@
         <v>6.72599983215332</v>
       </c>
       <c r="F523" t="n">
-        <v>6.722179889678955</v>
+        <v>6.721399784088135</v>
       </c>
       <c r="G523" t="n">
         <v>6.7088</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.003819942474365234</v>
+        <v>-0.004600048065185547</v>
       </c>
       <c r="I523" t="n">
         <v>99.43000030517578</v>
@@ -85681,13 +85681,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.15</v>
+        <v>4.16</v>
       </c>
       <c r="S523" t="n">
-        <v>2.67</v>
+        <v>2.68</v>
       </c>
       <c r="T523" t="n">
-        <v>2.67</v>
+        <v>2.68</v>
       </c>
       <c r="U523" t="n">
         <v>-3.871326025807375</v>
@@ -85699,10 +85699,10 @@
         <v>-2.792147440378345</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2380215591540225</v>
+        <v>-0.2283007738980602</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.032128514056225</v>
+        <v>8.433734939759036</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85725,7 +85725,7 @@
         <v>5.753968253968254</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4274115591540228</v>
+        <v>-0.4176907738980606</v>
       </c>
       <c r="AG523" t="n">
         <v>6.986385214151232</v>
@@ -86050,12 +86050,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.16</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>2.68</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86065,7 +86065,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86105,7 +86105,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.43</t>
+          <t>-0.42</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-04 16:39 EDT
Score: 64/100
USD/CNY: 6.72
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.16</v>
+        <v>4.11</v>
       </c>
       <c r="S523" t="n">
-        <v>2.68</v>
+        <v>2.63</v>
       </c>
       <c r="T523" t="n">
-        <v>2.68</v>
+        <v>2.63</v>
       </c>
       <c r="U523" t="n">
         <v>-3.910309214249079</v>
@@ -85703,10 +85703,10 @@
         <v>-1.791931316144391</v>
       </c>
       <c r="X523" t="n">
-        <v>0.8135243411040216</v>
+        <v>0.7644203067620703</v>
       </c>
       <c r="Y523" t="n">
-        <v>36.14457831325301</v>
+        <v>35.7429718875502</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>0.7936507936507936</v>
       </c>
       <c r="AF523" t="n">
-        <v>0.6268543411040106</v>
+        <v>0.5777503067620593</v>
       </c>
       <c r="AG523" t="n">
         <v>6.981733533406302</v>
@@ -85814,13 +85814,13 @@
         <v>6.718999862670898</v>
       </c>
       <c r="F524" t="n">
-        <v>6.708199977874756</v>
+        <v>6.707399845123291</v>
       </c>
       <c r="G524" t="n">
         <v>6.7001</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01079988479614258</v>
+        <v>-0.01160001754760742</v>
       </c>
       <c r="I524" t="n">
         <v>99</v>
@@ -85850,13 +85850,13 @@
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>4.16</v>
+        <v>4.11</v>
       </c>
       <c r="S524" t="n">
-        <v>2.68</v>
+        <v>2.63</v>
       </c>
       <c r="T524" t="n">
-        <v>2.68</v>
+        <v>2.63</v>
       </c>
       <c r="U524" t="n">
         <v>-3.830975075219038</v>
@@ -85868,10 +85868,10 @@
         <v>-2.835241353840001</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2731873941597351</v>
+        <v>-0.3217697734828162</v>
       </c>
       <c r="Y524" t="n">
-        <v>7.228915662650603</v>
+        <v>5.622489959839357</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,7 +85894,7 @@
         <v>0.992063492063492</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4598573941597461</v>
+        <v>-0.5084397734828272</v>
       </c>
       <c r="AG524" t="n">
         <v>6.976403072713822</v>
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>4.11</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.68</t>
+          <t>2.63</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.27</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.46</t>
+          <t>-0.51</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-08 17:01 EDT
Score: 63/100
USD/CNY: 6.71
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85355,13 +85355,13 @@
         <v>1.48</v>
       </c>
       <c r="R521" t="n">
-        <v>4.11</v>
+        <v>4.13</v>
       </c>
       <c r="S521" t="n">
-        <v>2.63</v>
+        <v>2.65</v>
       </c>
       <c r="T521" t="n">
-        <v>2.63</v>
+        <v>2.65</v>
       </c>
       <c r="U521" t="n">
         <v>-3.771293527335415</v>
@@ -85373,10 +85373,10 @@
         <v>-1.791931316144391</v>
       </c>
       <c r="X521" t="n">
-        <v>0.7644203067620703</v>
+        <v>0.7840619204988464</v>
       </c>
       <c r="Y521" t="n">
-        <v>35.94377510040161</v>
+        <v>36.14457831325301</v>
       </c>
       <c r="Z521" t="inlineStr">
         <is>
@@ -85399,7 +85399,7 @@
         <v>6.349206349206349</v>
       </c>
       <c r="AF521" t="n">
-        <v>0.5750303067620699</v>
+        <v>0.594671920498846</v>
       </c>
       <c r="AG521" t="n">
         <v>6.972393069593481</v>
@@ -85520,13 +85520,13 @@
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>4.11</v>
+        <v>4.13</v>
       </c>
       <c r="S522" t="n">
-        <v>2.63</v>
+        <v>2.65</v>
       </c>
       <c r="T522" t="n">
-        <v>2.63</v>
+        <v>2.65</v>
       </c>
       <c r="U522" t="n">
         <v>-3.734772917128601</v>
@@ -85538,7 +85538,7 @@
         <v>-1.671934315448642</v>
       </c>
       <c r="X522" t="n">
-        <v>0.8893491841864165</v>
+        <v>0.9090147973233265</v>
       </c>
       <c r="Y522" t="n">
         <v>37.34939759036145</v>
@@ -85564,7 +85564,7 @@
         <v>0.7936507936507936</v>
       </c>
       <c r="AF522" t="n">
-        <v>0.7072291841864198</v>
+        <v>0.7268947973233297</v>
       </c>
       <c r="AG522" t="n">
         <v>6.961433318203772</v>
@@ -85649,13 +85649,13 @@
         <v>6.710800170898438</v>
       </c>
       <c r="F523" t="n">
-        <v>6.706540107727051</v>
+        <v>6.705299854278564</v>
       </c>
       <c r="G523" t="n">
         <v>6.698200000000001</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.004260063171386719</v>
+        <v>-0.005500316619873047</v>
       </c>
       <c r="I523" t="n">
         <v>99.16000366210938</v>
@@ -85685,13 +85685,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.11</v>
+        <v>4.13</v>
       </c>
       <c r="S523" t="n">
-        <v>2.63</v>
+        <v>2.65</v>
       </c>
       <c r="T523" t="n">
-        <v>2.63</v>
+        <v>2.65</v>
       </c>
       <c r="U523" t="n">
         <v>-3.864115015069022</v>
@@ -85703,10 +85703,10 @@
         <v>-2.729930354548338</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2121304921202771</v>
+        <v>-0.1926764781911894</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.835341365461847</v>
+        <v>9.236947791164658</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>0.992063492063492</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.3942504921202739</v>
+        <v>-0.3747964781911861</v>
       </c>
       <c r="AG523" t="n">
         <v>6.970113207933402</v>
@@ -86054,12 +86054,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.11</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86069,7 +86069,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.21</t>
+          <t>-0.19</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86109,7 +86109,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.39</t>
+          <t>-0.37</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-09 13:25 EDT
Score: 63/100
USD/CNY: 6.71
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85649,19 +85649,19 @@
         <v>6.710800170898438</v>
       </c>
       <c r="F523" t="n">
-        <v>6.705949783325195</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="G523" t="n">
         <v>6.698200000000001</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.004850387573242188</v>
+        <v>0.06699991226196289</v>
       </c>
       <c r="I523" t="n">
-        <v>99.16000366210938</v>
+        <v>98.83999633789062</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>-0.003227181448169247</v>
       </c>
       <c r="K523" t="n">
         <v>3.151899999999999</v>
@@ -85697,16 +85697,16 @@
         <v>-3.824320335351802</v>
       </c>
       <c r="V523" t="n">
-        <v>6.5276</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-2.729930354548338</v>
+        <v>-1.671934315448642</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.1926764781911894</v>
+        <v>0.9090147973233265</v>
       </c>
       <c r="Y523" t="n">
-        <v>9.236947791164658</v>
+        <v>37.55020080321285</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85714,22 +85714,22 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.66212</v>
+        <v>1.6603</v>
       </c>
       <c r="AB523" t="n">
         <v>1.63242</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.41591</v>
+        <v>1.39189</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.1821200000000001</v>
+        <v>0.1803000000000001</v>
       </c>
       <c r="AE523" t="n">
-        <v>0.992063492063492</v>
+        <v>0.7936507936507936</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.3747964781911861</v>
+        <v>0.7287147973233266</v>
       </c>
       <c r="AG523" t="n">
         <v>6.96744266649893</v>
@@ -85738,10 +85738,10 @@
         <v>-0.2566424956004925</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.64314492599518</v>
+        <v>6.632036771677475</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.06765524490325703</v>
+        <v>0.07876339922096243</v>
       </c>
       <c r="AK523" t="n">
         <v>6.692627206904497</v>
@@ -85759,40 +85759,205 @@
         <v>0.8315239871298428</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.767586764552923</v>
+        <v>1.875440190456845</v>
       </c>
       <c r="AQ523" t="n">
-        <v>90.59999999999999</v>
+        <v>91</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.002173799094896913</v>
+        <v>0.001883967383495537</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7778000831604</v>
+        <v>6.777758874782571</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.07960008316039957</v>
+        <v>-0.0795588747825704</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.07960008316039957</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.06379223999647854</v>
+        <v>-0.06379017957758708</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.03171750503754148</v>
+        <v>-0.03171681823124433</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.0470797200754637</v>
+        <v>0.04707961705451913</v>
       </c>
       <c r="AY523" t="n">
         <v>1.08695652173913</v>
       </c>
       <c r="AZ523" t="n">
-        <v>62.56043478260869</v>
+        <v>62.68043478260869</v>
       </c>
       <c r="BA523" t="n">
-        <v>63.13758059646482</v>
+        <v>63.16158059646482</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2407</v>
+      </c>
+      <c r="D524" t="n">
+        <v>3.151899999999999</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.710800170898438</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.706369876861572</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.6963</v>
+      </c>
+      <c r="H524" t="n">
+        <v>-0.004430294036865234</v>
+      </c>
+      <c r="I524" t="n">
+        <v>98.83999633789062</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>3.151899999999999</v>
+      </c>
+      <c r="L524" t="n">
+        <v>3.033115</v>
+      </c>
+      <c r="M524" t="n">
+        <v>2.973885</v>
+      </c>
+      <c r="N524" t="n">
+        <v>2.818571666666666</v>
+      </c>
+      <c r="O524" t="n">
+        <v>99.80000000000001</v>
+      </c>
+      <c r="P524" t="n">
+        <v>97.30538922155688</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="R524" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-3.89983594807119</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.5224</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-2.807417388397881</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.2733637265387223</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>7.228915662650603</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.6603</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.63242</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.39189</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.1803000000000001</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>0.992063492063492</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.4536637265387222</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>6.972510368366358</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.2617101974679201</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.633976838378616</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>0.07682333251982154</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.685306332307247</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>0.02549383859119025</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.3822510793158705</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>0.03459091746240425</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.8328314813119078</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>1.839976984807577</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>0.002168947374356498</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.7778000831604</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>-0.08150008316040047</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>-0.08150008316040047</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.06557715761220076</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.03258011007182059</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.0488732448416407</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>1.075268817204301</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>62.4863440860215</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>62.9286675954873</v>
       </c>
     </row>
   </sheetData>
@@ -85999,7 +86164,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86029,7 +86194,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.16</t>
+          <t>98.84</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86064,17 +86229,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.53</t>
+          <t>6.52</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.19</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86094,7 +86259,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86109,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.37</t>
+          <t>-0.45</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86119,32 +86284,32 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.385</t>
+          <t>-0.382</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0347</t>
+          <t>0.0346</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.832</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1.84</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86169,7 +86334,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>-0.06</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-11 14:00 EDT
Score: 63/100
USD/CNY: 6.71
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.71049976348877</v>
       </c>
       <c r="F524" t="n">
-        <v>6.708020210266113</v>
+        <v>6.707119941711426</v>
       </c>
       <c r="G524" t="n">
         <v>6.6964</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.00247955322265625</v>
+        <v>-0.00337982177734375</v>
       </c>
       <c r="I524" t="n">
         <v>99.08999633789062</v>

</xml_diff>